<commit_message>
Support multiple contacts per company (contact + additional[])
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z165"/>
+  <dimension ref="A1:AA165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -527,15 +527,16 @@
     <col width="26" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
     <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
-    <col width="20" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="26" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="52" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -665,6 +666,11 @@
         </is>
       </c>
       <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Additional Contacts</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -738,6 +744,7 @@
       <c r="X2" s="4" t="n"/>
       <c r="Y2" s="4" t="n"/>
       <c r="Z2" s="4" t="n"/>
+      <c r="AA2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -822,6 +829,7 @@
       <c r="X3" s="4" t="n"/>
       <c r="Y3" s="4" t="n"/>
       <c r="Z3" s="4" t="n"/>
+      <c r="AA3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -896,6 +904,7 @@
       <c r="X4" s="4" t="n"/>
       <c r="Y4" s="4" t="n"/>
       <c r="Z4" s="4" t="n"/>
+      <c r="AA4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -985,6 +994,7 @@
       <c r="X5" s="4" t="n"/>
       <c r="Y5" s="4" t="n"/>
       <c r="Z5" s="4" t="n"/>
+      <c r="AA5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1054,6 +1064,7 @@
       <c r="X6" s="4" t="n"/>
       <c r="Y6" s="4" t="n"/>
       <c r="Z6" s="4" t="n"/>
+      <c r="AA6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1143,6 +1154,7 @@
       <c r="X7" s="4" t="n"/>
       <c r="Y7" s="4" t="n"/>
       <c r="Z7" s="4" t="n"/>
+      <c r="AA7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1212,6 +1224,7 @@
       <c r="X8" s="4" t="n"/>
       <c r="Y8" s="4" t="n"/>
       <c r="Z8" s="4" t="n"/>
+      <c r="AA8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1296,6 +1309,7 @@
       <c r="X9" s="4" t="n"/>
       <c r="Y9" s="4" t="n"/>
       <c r="Z9" s="4" t="n"/>
+      <c r="AA9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1385,6 +1399,7 @@
       <c r="X10" s="4" t="n"/>
       <c r="Y10" s="4" t="n"/>
       <c r="Z10" s="4" t="n"/>
+      <c r="AA10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1464,6 +1479,7 @@
       <c r="X11" s="4" t="n"/>
       <c r="Y11" s="4" t="n"/>
       <c r="Z11" s="4" t="n"/>
+      <c r="AA11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1533,6 +1549,7 @@
       <c r="X12" s="4" t="n"/>
       <c r="Y12" s="4" t="n"/>
       <c r="Z12" s="4" t="n"/>
+      <c r="AA12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1627,6 +1644,7 @@
       <c r="X13" s="4" t="n"/>
       <c r="Y13" s="4" t="n"/>
       <c r="Z13" s="4" t="n"/>
+      <c r="AA13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1696,6 +1714,7 @@
       <c r="X14" s="4" t="n"/>
       <c r="Y14" s="4" t="n"/>
       <c r="Z14" s="4" t="n"/>
+      <c r="AA14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1775,6 +1794,7 @@
       <c r="X15" s="4" t="n"/>
       <c r="Y15" s="4" t="n"/>
       <c r="Z15" s="4" t="n"/>
+      <c r="AA15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1844,6 +1864,7 @@
       <c r="X16" s="4" t="n"/>
       <c r="Y16" s="4" t="n"/>
       <c r="Z16" s="4" t="n"/>
+      <c r="AA16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1903,6 +1924,7 @@
       <c r="X17" s="4" t="n"/>
       <c r="Y17" s="4" t="n"/>
       <c r="Z17" s="4" t="n"/>
+      <c r="AA17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1972,6 +1994,7 @@
       <c r="X18" s="4" t="n"/>
       <c r="Y18" s="4" t="n"/>
       <c r="Z18" s="4" t="n"/>
+      <c r="AA18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2041,6 +2064,7 @@
       <c r="X19" s="4" t="n"/>
       <c r="Y19" s="4" t="n"/>
       <c r="Z19" s="4" t="n"/>
+      <c r="AA19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2130,6 +2154,7 @@
       <c r="X20" s="4" t="n"/>
       <c r="Y20" s="4" t="n"/>
       <c r="Z20" s="4" t="n"/>
+      <c r="AA20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2219,6 +2244,7 @@
       <c r="X21" s="4" t="n"/>
       <c r="Y21" s="4" t="n"/>
       <c r="Z21" s="4" t="n"/>
+      <c r="AA21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2288,6 +2314,7 @@
       <c r="X22" s="4" t="n"/>
       <c r="Y22" s="4" t="n"/>
       <c r="Z22" s="4" t="n"/>
+      <c r="AA22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2382,6 +2409,7 @@
       <c r="X23" s="4" t="n"/>
       <c r="Y23" s="4" t="n"/>
       <c r="Z23" s="4" t="n"/>
+      <c r="AA23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2466,6 +2494,7 @@
       <c r="X24" s="4" t="n"/>
       <c r="Y24" s="4" t="n"/>
       <c r="Z24" s="4" t="n"/>
+      <c r="AA24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2525,6 +2554,7 @@
       <c r="X25" s="4" t="n"/>
       <c r="Y25" s="4" t="n"/>
       <c r="Z25" s="4" t="n"/>
+      <c r="AA25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2614,6 +2644,7 @@
       <c r="X26" s="4" t="n"/>
       <c r="Y26" s="4" t="n"/>
       <c r="Z26" s="4" t="n"/>
+      <c r="AA26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2683,6 +2714,7 @@
       <c r="X27" s="4" t="n"/>
       <c r="Y27" s="4" t="n"/>
       <c r="Z27" s="4" t="n"/>
+      <c r="AA27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2767,6 +2799,7 @@
       <c r="X28" s="4" t="n"/>
       <c r="Y28" s="4" t="n"/>
       <c r="Z28" s="4" t="n"/>
+      <c r="AA28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2836,6 +2869,7 @@
       <c r="X29" s="4" t="n"/>
       <c r="Y29" s="4" t="n"/>
       <c r="Z29" s="4" t="n"/>
+      <c r="AA29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2905,6 +2939,7 @@
       <c r="X30" s="4" t="n"/>
       <c r="Y30" s="4" t="n"/>
       <c r="Z30" s="4" t="n"/>
+      <c r="AA30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2964,6 +2999,7 @@
       <c r="X31" s="4" t="n"/>
       <c r="Y31" s="4" t="n"/>
       <c r="Z31" s="4" t="n"/>
+      <c r="AA31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3053,6 +3089,7 @@
       <c r="X32" s="4" t="n"/>
       <c r="Y32" s="4" t="n"/>
       <c r="Z32" s="4" t="n"/>
+      <c r="AA32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3122,6 +3159,7 @@
       <c r="X33" s="4" t="n"/>
       <c r="Y33" s="4" t="n"/>
       <c r="Z33" s="4" t="n"/>
+      <c r="AA33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3191,6 +3229,7 @@
       <c r="X34" s="4" t="n"/>
       <c r="Y34" s="4" t="n"/>
       <c r="Z34" s="4" t="n"/>
+      <c r="AA34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3265,6 +3304,7 @@
       <c r="X35" s="4" t="n"/>
       <c r="Y35" s="4" t="n"/>
       <c r="Z35" s="4" t="n"/>
+      <c r="AA35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3354,6 +3394,7 @@
       <c r="X36" s="4" t="n"/>
       <c r="Y36" s="4" t="n"/>
       <c r="Z36" s="4" t="n"/>
+      <c r="AA36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3433,6 +3474,7 @@
       <c r="X37" s="4" t="n"/>
       <c r="Y37" s="4" t="n"/>
       <c r="Z37" s="4" t="n"/>
+      <c r="AA37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3502,6 +3544,7 @@
       <c r="X38" s="4" t="n"/>
       <c r="Y38" s="4" t="n"/>
       <c r="Z38" s="4" t="n"/>
+      <c r="AA38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3571,6 +3614,7 @@
       <c r="X39" s="4" t="n"/>
       <c r="Y39" s="4" t="n"/>
       <c r="Z39" s="4" t="n"/>
+      <c r="AA39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3640,6 +3684,7 @@
       <c r="X40" s="4" t="n"/>
       <c r="Y40" s="4" t="n"/>
       <c r="Z40" s="4" t="n"/>
+      <c r="AA40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3709,6 +3754,7 @@
       <c r="X41" s="4" t="n"/>
       <c r="Y41" s="4" t="n"/>
       <c r="Z41" s="4" t="n"/>
+      <c r="AA41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3798,6 +3844,7 @@
       <c r="X42" s="4" t="n"/>
       <c r="Y42" s="4" t="n"/>
       <c r="Z42" s="4" t="n"/>
+      <c r="AA42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3887,6 +3934,7 @@
       <c r="X43" s="4" t="n"/>
       <c r="Y43" s="4" t="n"/>
       <c r="Z43" s="4" t="n"/>
+      <c r="AA43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3971,6 +4019,7 @@
       <c r="X44" s="4" t="n"/>
       <c r="Y44" s="4" t="n"/>
       <c r="Z44" s="4" t="n"/>
+      <c r="AA44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4040,6 +4089,7 @@
       <c r="X45" s="4" t="n"/>
       <c r="Y45" s="4" t="n"/>
       <c r="Z45" s="4" t="n"/>
+      <c r="AA45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4109,6 +4159,7 @@
       <c r="X46" s="4" t="n"/>
       <c r="Y46" s="4" t="n"/>
       <c r="Z46" s="4" t="n"/>
+      <c r="AA46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4178,6 +4229,7 @@
       <c r="X47" s="4" t="n"/>
       <c r="Y47" s="4" t="n"/>
       <c r="Z47" s="4" t="n"/>
+      <c r="AA47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4267,6 +4319,7 @@
       <c r="X48" s="4" t="n"/>
       <c r="Y48" s="4" t="n"/>
       <c r="Z48" s="4" t="n"/>
+      <c r="AA48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4361,6 +4414,7 @@
       <c r="X49" s="4" t="n"/>
       <c r="Y49" s="4" t="n"/>
       <c r="Z49" s="4" t="n"/>
+      <c r="AA49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4450,6 +4504,7 @@
       <c r="X50" s="4" t="n"/>
       <c r="Y50" s="4" t="n"/>
       <c r="Z50" s="4" t="n"/>
+      <c r="AA50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4529,6 +4584,7 @@
       <c r="X51" s="4" t="n"/>
       <c r="Y51" s="4" t="n"/>
       <c r="Z51" s="4" t="n"/>
+      <c r="AA51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4618,6 +4674,7 @@
       <c r="X52" s="4" t="n"/>
       <c r="Y52" s="4" t="n"/>
       <c r="Z52" s="4" t="n"/>
+      <c r="AA52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4687,6 +4744,7 @@
       <c r="X53" s="4" t="n"/>
       <c r="Y53" s="4" t="n"/>
       <c r="Z53" s="4" t="n"/>
+      <c r="AA53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4746,6 +4804,7 @@
       <c r="X54" s="4" t="n"/>
       <c r="Y54" s="4" t="n"/>
       <c r="Z54" s="4" t="n"/>
+      <c r="AA54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4835,6 +4894,7 @@
       <c r="X55" s="4" t="n"/>
       <c r="Y55" s="4" t="n"/>
       <c r="Z55" s="4" t="n"/>
+      <c r="AA55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4904,6 +4964,7 @@
       <c r="X56" s="4" t="n"/>
       <c r="Y56" s="4" t="n"/>
       <c r="Z56" s="4" t="n"/>
+      <c r="AA56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4993,6 +5054,7 @@
       <c r="X57" s="4" t="n"/>
       <c r="Y57" s="4" t="n"/>
       <c r="Z57" s="4" t="n"/>
+      <c r="AA57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5082,6 +5144,7 @@
       <c r="X58" s="4" t="n"/>
       <c r="Y58" s="4" t="n"/>
       <c r="Z58" s="4" t="n"/>
+      <c r="AA58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5141,6 +5204,7 @@
       <c r="X59" s="4" t="n"/>
       <c r="Y59" s="4" t="n"/>
       <c r="Z59" s="4" t="n"/>
+      <c r="AA59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5230,6 +5294,7 @@
       <c r="X60" s="4" t="n"/>
       <c r="Y60" s="4" t="n"/>
       <c r="Z60" s="4" t="n"/>
+      <c r="AA60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5299,6 +5364,7 @@
       <c r="X61" s="4" t="n"/>
       <c r="Y61" s="4" t="n"/>
       <c r="Z61" s="4" t="n"/>
+      <c r="AA61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5358,6 +5424,7 @@
       <c r="X62" s="4" t="n"/>
       <c r="Y62" s="4" t="n"/>
       <c r="Z62" s="4" t="n"/>
+      <c r="AA62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5417,6 +5484,7 @@
       <c r="X63" s="4" t="n"/>
       <c r="Y63" s="4" t="n"/>
       <c r="Z63" s="4" t="n"/>
+      <c r="AA63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5501,6 +5569,7 @@
       <c r="X64" s="4" t="n"/>
       <c r="Y64" s="4" t="n"/>
       <c r="Z64" s="4" t="n"/>
+      <c r="AA64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5590,6 +5659,7 @@
       <c r="X65" s="4" t="n"/>
       <c r="Y65" s="4" t="n"/>
       <c r="Z65" s="4" t="n"/>
+      <c r="AA65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5659,6 +5729,7 @@
       <c r="X66" s="4" t="n"/>
       <c r="Y66" s="4" t="n"/>
       <c r="Z66" s="4" t="n"/>
+      <c r="AA66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5748,6 +5819,7 @@
       <c r="X67" s="4" t="n"/>
       <c r="Y67" s="4" t="n"/>
       <c r="Z67" s="4" t="n"/>
+      <c r="AA67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5837,6 +5909,7 @@
       <c r="X68" s="4" t="n"/>
       <c r="Y68" s="4" t="n"/>
       <c r="Z68" s="4" t="n"/>
+      <c r="AA68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5921,6 +5994,7 @@
       <c r="X69" s="4" t="n"/>
       <c r="Y69" s="4" t="n"/>
       <c r="Z69" s="4" t="n"/>
+      <c r="AA69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6010,6 +6084,7 @@
       <c r="X70" s="4" t="n"/>
       <c r="Y70" s="4" t="n"/>
       <c r="Z70" s="4" t="n"/>
+      <c r="AA70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6099,6 +6174,7 @@
       <c r="X71" s="4" t="n"/>
       <c r="Y71" s="4" t="n"/>
       <c r="Z71" s="4" t="n"/>
+      <c r="AA71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6188,6 +6264,7 @@
       <c r="X72" s="4" t="n"/>
       <c r="Y72" s="4" t="n"/>
       <c r="Z72" s="4" t="n"/>
+      <c r="AA72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6257,6 +6334,7 @@
       <c r="X73" s="4" t="n"/>
       <c r="Y73" s="4" t="n"/>
       <c r="Z73" s="4" t="n"/>
+      <c r="AA73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6346,6 +6424,7 @@
       <c r="X74" s="4" t="n"/>
       <c r="Y74" s="4" t="n"/>
       <c r="Z74" s="4" t="n"/>
+      <c r="AA74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6415,6 +6494,7 @@
       <c r="X75" s="4" t="n"/>
       <c r="Y75" s="4" t="n"/>
       <c r="Z75" s="4" t="n"/>
+      <c r="AA75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6474,6 +6554,7 @@
       <c r="X76" s="4" t="n"/>
       <c r="Y76" s="4" t="n"/>
       <c r="Z76" s="4" t="n"/>
+      <c r="AA76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6543,6 +6624,7 @@
       <c r="X77" s="4" t="n"/>
       <c r="Y77" s="4" t="n"/>
       <c r="Z77" s="4" t="n"/>
+      <c r="AA77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6627,6 +6709,7 @@
       <c r="X78" s="4" t="n"/>
       <c r="Y78" s="4" t="n"/>
       <c r="Z78" s="4" t="n"/>
+      <c r="AA78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6716,6 +6799,7 @@
       <c r="X79" s="4" t="n"/>
       <c r="Y79" s="4" t="n"/>
       <c r="Z79" s="4" t="n"/>
+      <c r="AA79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6795,6 +6879,7 @@
       <c r="X80" s="4" t="n"/>
       <c r="Y80" s="4" t="n"/>
       <c r="Z80" s="4" t="n"/>
+      <c r="AA80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6884,6 +6969,7 @@
       <c r="X81" s="4" t="n"/>
       <c r="Y81" s="4" t="n"/>
       <c r="Z81" s="4" t="n"/>
+      <c r="AA81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6963,6 +7049,7 @@
       <c r="X82" s="4" t="n"/>
       <c r="Y82" s="4" t="n"/>
       <c r="Z82" s="4" t="n"/>
+      <c r="AA82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7032,6 +7119,7 @@
       <c r="X83" s="4" t="n"/>
       <c r="Y83" s="4" t="n"/>
       <c r="Z83" s="4" t="n"/>
+      <c r="AA83" s="4" t="n"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7091,6 +7179,7 @@
       <c r="X84" s="4" t="n"/>
       <c r="Y84" s="4" t="n"/>
       <c r="Z84" s="4" t="n"/>
+      <c r="AA84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7175,6 +7264,7 @@
       <c r="X85" s="4" t="n"/>
       <c r="Y85" s="4" t="n"/>
       <c r="Z85" s="4" t="n"/>
+      <c r="AA85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7254,6 +7344,7 @@
       <c r="X86" s="4" t="n"/>
       <c r="Y86" s="4" t="n"/>
       <c r="Z86" s="4" t="n"/>
+      <c r="AA86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7318,6 +7409,7 @@
       <c r="X87" s="4" t="n"/>
       <c r="Y87" s="4" t="n"/>
       <c r="Z87" s="4" t="n"/>
+      <c r="AA87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7377,6 +7469,7 @@
       <c r="X88" s="4" t="n"/>
       <c r="Y88" s="4" t="n"/>
       <c r="Z88" s="4" t="n"/>
+      <c r="AA88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7456,6 +7549,7 @@
       <c r="X89" s="4" t="n"/>
       <c r="Y89" s="4" t="n"/>
       <c r="Z89" s="4" t="n"/>
+      <c r="AA89" s="4" t="n"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7530,6 +7624,7 @@
       <c r="X90" s="4" t="n"/>
       <c r="Y90" s="4" t="n"/>
       <c r="Z90" s="4" t="n"/>
+      <c r="AA90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7599,6 +7694,7 @@
       <c r="X91" s="4" t="n"/>
       <c r="Y91" s="4" t="n"/>
       <c r="Z91" s="4" t="n"/>
+      <c r="AA91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7658,6 +7754,7 @@
       <c r="X92" s="4" t="n"/>
       <c r="Y92" s="4" t="n"/>
       <c r="Z92" s="4" t="n"/>
+      <c r="AA92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7717,6 +7814,7 @@
       <c r="X93" s="4" t="n"/>
       <c r="Y93" s="4" t="n"/>
       <c r="Z93" s="4" t="n"/>
+      <c r="AA93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7806,6 +7904,7 @@
       <c r="X94" s="4" t="n"/>
       <c r="Y94" s="4" t="n"/>
       <c r="Z94" s="4" t="n"/>
+      <c r="AA94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7875,6 +7974,7 @@
       <c r="X95" s="4" t="n"/>
       <c r="Y95" s="4" t="n"/>
       <c r="Z95" s="4" t="n"/>
+      <c r="AA95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7944,6 +8044,7 @@
       <c r="X96" s="4" t="n"/>
       <c r="Y96" s="4" t="n"/>
       <c r="Z96" s="4" t="n"/>
+      <c r="AA96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -8023,6 +8124,7 @@
       <c r="X97" s="4" t="n"/>
       <c r="Y97" s="4" t="n"/>
       <c r="Z97" s="4" t="n"/>
+      <c r="AA97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8082,6 +8184,7 @@
       <c r="X98" s="4" t="n"/>
       <c r="Y98" s="4" t="n"/>
       <c r="Z98" s="4" t="n"/>
+      <c r="AA98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8151,6 +8254,7 @@
       <c r="X99" s="4" t="n"/>
       <c r="Y99" s="4" t="n"/>
       <c r="Z99" s="4" t="n"/>
+      <c r="AA99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -8220,6 +8324,7 @@
       <c r="X100" s="4" t="n"/>
       <c r="Y100" s="4" t="n"/>
       <c r="Z100" s="4" t="n"/>
+      <c r="AA100" s="4" t="n"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8289,6 +8394,7 @@
       <c r="X101" s="4" t="n"/>
       <c r="Y101" s="4" t="n"/>
       <c r="Z101" s="4" t="n"/>
+      <c r="AA101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8378,6 +8484,7 @@
       <c r="X102" s="4" t="n"/>
       <c r="Y102" s="4" t="n"/>
       <c r="Z102" s="4" t="n"/>
+      <c r="AA102" s="4" t="n"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8447,6 +8554,7 @@
       <c r="X103" s="4" t="n"/>
       <c r="Y103" s="4" t="n"/>
       <c r="Z103" s="4" t="n"/>
+      <c r="AA103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8536,6 +8644,7 @@
       <c r="X104" s="4" t="n"/>
       <c r="Y104" s="4" t="n"/>
       <c r="Z104" s="4" t="n"/>
+      <c r="AA104" s="4" t="n"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -8625,6 +8734,7 @@
       <c r="X105" s="4" t="n"/>
       <c r="Y105" s="4" t="n"/>
       <c r="Z105" s="4" t="n"/>
+      <c r="AA105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -8714,6 +8824,7 @@
       <c r="X106" s="4" t="n"/>
       <c r="Y106" s="4" t="n"/>
       <c r="Z106" s="4" t="n"/>
+      <c r="AA106" s="4" t="n"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -8783,6 +8894,7 @@
       <c r="X107" s="4" t="n"/>
       <c r="Y107" s="4" t="n"/>
       <c r="Z107" s="4" t="n"/>
+      <c r="AA107" s="4" t="n"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8852,6 +8964,7 @@
       <c r="X108" s="4" t="n"/>
       <c r="Y108" s="4" t="n"/>
       <c r="Z108" s="4" t="n"/>
+      <c r="AA108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -8941,6 +9054,7 @@
       <c r="X109" s="4" t="n"/>
       <c r="Y109" s="4" t="n"/>
       <c r="Z109" s="4" t="n"/>
+      <c r="AA109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -9000,6 +9114,7 @@
       <c r="X110" s="4" t="n"/>
       <c r="Y110" s="4" t="n"/>
       <c r="Z110" s="4" t="n"/>
+      <c r="AA110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9059,6 +9174,7 @@
       <c r="X111" s="4" t="n"/>
       <c r="Y111" s="4" t="n"/>
       <c r="Z111" s="4" t="n"/>
+      <c r="AA111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9128,6 +9244,7 @@
       <c r="X112" s="4" t="n"/>
       <c r="Y112" s="4" t="n"/>
       <c r="Z112" s="4" t="n"/>
+      <c r="AA112" s="4" t="n"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9207,6 +9324,7 @@
       <c r="X113" s="4" t="n"/>
       <c r="Y113" s="4" t="n"/>
       <c r="Z113" s="4" t="n"/>
+      <c r="AA113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -9276,6 +9394,7 @@
       <c r="X114" s="4" t="n"/>
       <c r="Y114" s="4" t="n"/>
       <c r="Z114" s="4" t="n"/>
+      <c r="AA114" s="4" t="n"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -9345,6 +9464,7 @@
       <c r="X115" s="4" t="n"/>
       <c r="Y115" s="4" t="n"/>
       <c r="Z115" s="4" t="n"/>
+      <c r="AA115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -9404,6 +9524,7 @@
       <c r="X116" s="4" t="n"/>
       <c r="Y116" s="4" t="n"/>
       <c r="Z116" s="4" t="n"/>
+      <c r="AA116" s="4" t="n"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -9483,6 +9604,7 @@
       <c r="X117" s="4" t="n"/>
       <c r="Y117" s="4" t="n"/>
       <c r="Z117" s="4" t="n"/>
+      <c r="AA117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -9557,6 +9679,7 @@
       <c r="X118" s="4" t="n"/>
       <c r="Y118" s="4" t="n"/>
       <c r="Z118" s="4" t="n"/>
+      <c r="AA118" s="4" t="n"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -9626,6 +9749,7 @@
       <c r="X119" s="4" t="n"/>
       <c r="Y119" s="4" t="n"/>
       <c r="Z119" s="4" t="n"/>
+      <c r="AA119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -9695,6 +9819,7 @@
       <c r="X120" s="4" t="n"/>
       <c r="Y120" s="4" t="n"/>
       <c r="Z120" s="4" t="n"/>
+      <c r="AA120" s="4" t="n"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -9769,6 +9894,7 @@
       <c r="X121" s="4" t="n"/>
       <c r="Y121" s="4" t="n"/>
       <c r="Z121" s="4" t="n"/>
+      <c r="AA121" s="4" t="n"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -9828,6 +9954,7 @@
       <c r="X122" s="4" t="n"/>
       <c r="Y122" s="4" t="n"/>
       <c r="Z122" s="4" t="n"/>
+      <c r="AA122" s="4" t="n"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -9902,6 +10029,7 @@
       <c r="X123" s="4" t="n"/>
       <c r="Y123" s="4" t="n"/>
       <c r="Z123" s="4" t="n"/>
+      <c r="AA123" s="4" t="n"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -9961,6 +10089,7 @@
       <c r="X124" s="4" t="n"/>
       <c r="Y124" s="4" t="n"/>
       <c r="Z124" s="4" t="n"/>
+      <c r="AA124" s="4" t="n"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -10050,6 +10179,7 @@
       <c r="X125" s="4" t="n"/>
       <c r="Y125" s="4" t="n"/>
       <c r="Z125" s="4" t="n"/>
+      <c r="AA125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -10119,6 +10249,7 @@
       <c r="X126" s="4" t="n"/>
       <c r="Y126" s="4" t="n"/>
       <c r="Z126" s="4" t="n"/>
+      <c r="AA126" s="4" t="n"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -10178,6 +10309,7 @@
       <c r="X127" s="4" t="n"/>
       <c r="Y127" s="4" t="n"/>
       <c r="Z127" s="4" t="n"/>
+      <c r="AA127" s="4" t="n"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -10237,6 +10369,7 @@
       <c r="X128" s="4" t="n"/>
       <c r="Y128" s="4" t="n"/>
       <c r="Z128" s="4" t="n"/>
+      <c r="AA128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -10306,6 +10439,7 @@
       <c r="X129" s="4" t="n"/>
       <c r="Y129" s="4" t="n"/>
       <c r="Z129" s="4" t="n"/>
+      <c r="AA129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -10375,6 +10509,7 @@
       <c r="X130" s="4" t="n"/>
       <c r="Y130" s="4" t="n"/>
       <c r="Z130" s="4" t="n"/>
+      <c r="AA130" s="4" t="n"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -10434,6 +10569,7 @@
       <c r="X131" s="4" t="n"/>
       <c r="Y131" s="4" t="n"/>
       <c r="Z131" s="4" t="n"/>
+      <c r="AA131" s="4" t="n"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -10523,6 +10659,7 @@
       <c r="X132" s="4" t="n"/>
       <c r="Y132" s="4" t="n"/>
       <c r="Z132" s="4" t="n"/>
+      <c r="AA132" s="4" t="n"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -10597,6 +10734,7 @@
       <c r="X133" s="4" t="n"/>
       <c r="Y133" s="4" t="n"/>
       <c r="Z133" s="4" t="n"/>
+      <c r="AA133" s="4" t="n"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -10666,6 +10804,7 @@
       <c r="X134" s="4" t="n"/>
       <c r="Y134" s="4" t="n"/>
       <c r="Z134" s="4" t="n"/>
+      <c r="AA134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -10725,6 +10864,7 @@
       <c r="X135" s="4" t="n"/>
       <c r="Y135" s="4" t="n"/>
       <c r="Z135" s="4" t="n"/>
+      <c r="AA135" s="4" t="n"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -10804,6 +10944,7 @@
       <c r="X136" s="4" t="n"/>
       <c r="Y136" s="4" t="n"/>
       <c r="Z136" s="4" t="n"/>
+      <c r="AA136" s="4" t="n"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -10873,6 +11014,7 @@
       <c r="X137" s="4" t="n"/>
       <c r="Y137" s="4" t="n"/>
       <c r="Z137" s="4" t="n"/>
+      <c r="AA137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -10942,6 +11084,7 @@
       <c r="X138" s="4" t="n"/>
       <c r="Y138" s="4" t="n"/>
       <c r="Z138" s="4" t="n"/>
+      <c r="AA138" s="4" t="n"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -11021,6 +11164,7 @@
       <c r="X139" s="4" t="n"/>
       <c r="Y139" s="4" t="n"/>
       <c r="Z139" s="4" t="n"/>
+      <c r="AA139" s="4" t="n"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -11095,6 +11239,7 @@
       <c r="X140" s="4" t="n"/>
       <c r="Y140" s="4" t="n"/>
       <c r="Z140" s="4" t="n"/>
+      <c r="AA140" s="4" t="n"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -11164,6 +11309,7 @@
       <c r="X141" s="4" t="n"/>
       <c r="Y141" s="4" t="n"/>
       <c r="Z141" s="4" t="n"/>
+      <c r="AA141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -11253,6 +11399,7 @@
       <c r="X142" s="4" t="n"/>
       <c r="Y142" s="4" t="n"/>
       <c r="Z142" s="4" t="n"/>
+      <c r="AA142" s="4" t="n"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -11312,6 +11459,7 @@
       <c r="X143" s="4" t="n"/>
       <c r="Y143" s="4" t="n"/>
       <c r="Z143" s="4" t="n"/>
+      <c r="AA143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -11391,6 +11539,7 @@
       <c r="X144" s="4" t="n"/>
       <c r="Y144" s="4" t="n"/>
       <c r="Z144" s="4" t="n"/>
+      <c r="AA144" s="4" t="n"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -11465,6 +11614,7 @@
       <c r="X145" s="4" t="n"/>
       <c r="Y145" s="4" t="n"/>
       <c r="Z145" s="4" t="n"/>
+      <c r="AA145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -11539,6 +11689,7 @@
       <c r="X146" s="4" t="n"/>
       <c r="Y146" s="4" t="n"/>
       <c r="Z146" s="4" t="n"/>
+      <c r="AA146" s="4" t="n"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -11613,6 +11764,7 @@
       <c r="X147" s="4" t="n"/>
       <c r="Y147" s="4" t="n"/>
       <c r="Z147" s="4" t="n"/>
+      <c r="AA147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -11692,6 +11844,7 @@
       <c r="X148" s="4" t="n"/>
       <c r="Y148" s="4" t="n"/>
       <c r="Z148" s="4" t="n"/>
+      <c r="AA148" s="4" t="n"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -11776,6 +11929,7 @@
       <c r="X149" s="4" t="n"/>
       <c r="Y149" s="4" t="n"/>
       <c r="Z149" s="4" t="n"/>
+      <c r="AA149" s="4" t="n"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -11865,6 +12019,7 @@
       <c r="X150" s="4" t="n"/>
       <c r="Y150" s="4" t="n"/>
       <c r="Z150" s="4" t="n"/>
+      <c r="AA150" s="4" t="n"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -11924,6 +12079,7 @@
       <c r="X151" s="4" t="n"/>
       <c r="Y151" s="4" t="n"/>
       <c r="Z151" s="4" t="n"/>
+      <c r="AA151" s="4" t="n"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -12003,6 +12159,7 @@
       <c r="X152" s="4" t="n"/>
       <c r="Y152" s="4" t="n"/>
       <c r="Z152" s="4" t="n"/>
+      <c r="AA152" s="4" t="n"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -12062,6 +12219,7 @@
       <c r="X153" s="4" t="n"/>
       <c r="Y153" s="4" t="n"/>
       <c r="Z153" s="4" t="n"/>
+      <c r="AA153" s="4" t="n"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -12121,6 +12279,7 @@
       <c r="X154" s="4" t="n"/>
       <c r="Y154" s="4" t="n"/>
       <c r="Z154" s="4" t="n"/>
+      <c r="AA154" s="4" t="n"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -12190,6 +12349,7 @@
       <c r="X155" s="4" t="n"/>
       <c r="Y155" s="4" t="n"/>
       <c r="Z155" s="4" t="n"/>
+      <c r="AA155" s="4" t="n"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -12279,6 +12439,7 @@
       <c r="X156" s="4" t="n"/>
       <c r="Y156" s="4" t="n"/>
       <c r="Z156" s="4" t="n"/>
+      <c r="AA156" s="4" t="n"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -12358,6 +12519,7 @@
       <c r="X157" s="4" t="n"/>
       <c r="Y157" s="4" t="n"/>
       <c r="Z157" s="4" t="n"/>
+      <c r="AA157" s="4" t="n"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -12442,6 +12604,7 @@
       <c r="X158" s="4" t="n"/>
       <c r="Y158" s="4" t="n"/>
       <c r="Z158" s="4" t="n"/>
+      <c r="AA158" s="4" t="n"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -12521,6 +12684,7 @@
       <c r="X159" s="4" t="n"/>
       <c r="Y159" s="4" t="n"/>
       <c r="Z159" s="4" t="n"/>
+      <c r="AA159" s="4" t="n"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -12590,6 +12754,7 @@
       <c r="X160" s="4" t="n"/>
       <c r="Y160" s="4" t="n"/>
       <c r="Z160" s="4" t="n"/>
+      <c r="AA160" s="4" t="n"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -12649,6 +12814,7 @@
       <c r="X161" s="4" t="n"/>
       <c r="Y161" s="4" t="n"/>
       <c r="Z161" s="4" t="n"/>
+      <c r="AA161" s="4" t="n"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -12713,6 +12879,7 @@
       <c r="X162" s="4" t="n"/>
       <c r="Y162" s="4" t="n"/>
       <c r="Z162" s="4" t="n"/>
+      <c r="AA162" s="4" t="n"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -12797,6 +12964,7 @@
       <c r="X163" s="4" t="n"/>
       <c r="Y163" s="4" t="n"/>
       <c r="Z163" s="4" t="n"/>
+      <c r="AA163" s="4" t="n"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -12886,6 +13054,7 @@
       <c r="X164" s="4" t="n"/>
       <c r="Y164" s="4" t="n"/>
       <c r="Z164" s="4" t="n"/>
+      <c r="AA164" s="4" t="n"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -12945,6 +13114,7 @@
       <c r="X165" s="4" t="n"/>
       <c r="Y165" s="4" t="n"/>
       <c r="Z165" s="4" t="n"/>
+      <c r="AA165" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
enrich batch (9PM pass): rows 0-14
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,18 +18,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -81,27 +74,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -122,29 +100,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -540,137 +524,137 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>In-Range Ratings (A to BB)</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>In-Range Rating Count</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Instruments</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>CRAs</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Sub-Sector</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>CIN</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Registered City</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Registered Office Address</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Corporate Office City</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Corporate Office Address</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Corporate Email</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Registered Email</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>HO Email</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>Contact Name</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>Designation</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>Direct Mobile</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>Direct Email</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>Fallback (Landline/IR)</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="X1" s="3" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="Y1" s="3" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="Z1" s="3" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>Additional Contacts</t>
         </is>
       </c>
-      <c r="AA1" s="3" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -735,16 +719,50 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-      <c r="Z2" s="4" t="n"/>
-      <c r="AA2" s="4" t="n"/>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>Ramandeep Singh Gill</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="n"/>
+      <c r="U2" s="3" t="n"/>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>secretarial@muthootcap.com / +91-484-6619600 (company secretarial &amp; investor desk)</t>
+        </is>
+      </c>
+      <c r="W2" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X2" s="3" t="inlineStr">
+        <is>
+          <t>MarketScreener - 'Muthoot Capital Services Names New CFO'; Bloomberg Markets profile - Ramandeep Singh Gill; Simply Wall St management page</t>
+        </is>
+      </c>
+      <c r="Y2" s="3" t="inlineStr">
+        <is>
+          <t>Appointed CFO effective Dec 6, 2022, succeeding Vinodkumar Madhavan Panicker; confirmed via 3 independent sources. Direct personal email/phone could not be independently verified; NOT used per no-fabrication rule. Fallback is the company's investor/secretarial contact.</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>Deepa Gopalakrishnan (Deepa G) | Company Secretary &amp; Compliance Officer | +91-484-6619672 | secretarial@muthootcap.com  (LOW)
+Srikanth G Menon | Company Secretary &amp; Compliance Officer (per Mar 2024 appointment) | +91-484-6619672 | srikanth.m@muthootcap.com  (LOW)
+Tina Suzanne George | Whole-time/Executive Director (Chartered Accountant; ex-Deloitte, EY)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -820,16 +838,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R3" s="4" t="n"/>
-      <c r="S3" s="4" t="n"/>
-      <c r="T3" s="4" t="n"/>
-      <c r="U3" s="4" t="n"/>
-      <c r="V3" s="4" t="n"/>
-      <c r="W3" s="4" t="n"/>
-      <c r="X3" s="4" t="n"/>
-      <c r="Y3" s="4" t="n"/>
-      <c r="Z3" s="4" t="n"/>
-      <c r="AA3" s="4" t="n"/>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>Gagan Aggarwal</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="n"/>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>gagan.aggarwal@clix.capital</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="n"/>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>PeopleMatters - 'Fintech solutions Clix Capital hires Gagan Aggarwal as its CFO'; LinkedIn; TheOrg org chart</t>
+        </is>
+      </c>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>Name/designation high-confidence (news + LinkedIn + org chart). Email is INFERRED from the firstname.lastname@clix.capital pattern (confirmed real via CS contact Vinu.Kalra@clix.capital) - not independently confirmed for this individual, so downgraded to medium.</t>
+        </is>
+      </c>
+      <c r="Z3" s="4" t="inlineStr">
+        <is>
+          <t>Dhairya Parikh | Head, Treasury  (MEDIUM)
+Vinu Rajat Kalra | AVP &amp; Company Secretary / Compliance Officer | 0120-6465400 | Vinu.Kalra@clix.capital  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -895,16 +946,56 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R4" s="4" t="n"/>
-      <c r="S4" s="4" t="n"/>
-      <c r="T4" s="4" t="n"/>
-      <c r="U4" s="4" t="n"/>
-      <c r="V4" s="4" t="n"/>
-      <c r="W4" s="4" t="n"/>
-      <c r="X4" s="4" t="n"/>
-      <c r="Y4" s="4" t="n"/>
-      <c r="Z4" s="4" t="n"/>
-      <c r="AA4" s="4" t="n"/>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>Tarun Khurana</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>Company Secretary &amp; Compliance Officer, Edelweiss Financial Services Ltd (group-level; handles investor/debt grievance across group entities)</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>+91 22 4079 5199</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>investors@edelweissfin.com</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
+          <t>+91 22 2286 4400 / Fax +91 22 4079 5099</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X4" s="5" t="inlineStr">
+        <is>
+          <t>Edelweiss Financial Services Investor Services page; Trendlyne CS profile; BSE corporate filing</t>
+        </is>
+      </c>
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>Edelweiss Retail Finance Ltd (ERFL) is a wholly-owned subsidiary sharing group finance/secretarial functions; no standalone CFO/CS identified as ERFL's own KMP. Domain matches ERFL's on-file registered email but 1:1 match not confirmed - verify before outreach.</t>
+        </is>
+      </c>
+      <c r="Z4" s="4" t="inlineStr">
+        <is>
+          <t>Ananya Suneja | President &amp; Chief Financial Officer, Edelweiss Financial Services Ltd (Group CFO)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -985,16 +1076,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R5" s="4" t="n"/>
-      <c r="S5" s="4" t="n"/>
-      <c r="T5" s="4" t="n"/>
-      <c r="U5" s="4" t="n"/>
-      <c r="V5" s="4" t="n"/>
-      <c r="W5" s="4" t="n"/>
-      <c r="X5" s="4" t="n"/>
-      <c r="Y5" s="4" t="n"/>
-      <c r="Z5" s="4" t="n"/>
-      <c r="AA5" s="4" t="n"/>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>Thanish Dalee</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="n"/>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>cfo@klmaxiva.com</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>+91-484-281125 (finance desk landline)</t>
+        </is>
+      </c>
+      <c r="W5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X5" s="3" t="inlineStr">
+        <is>
+          <t>ZoomInfo and RocketReach independently list Thanish Dalee as CFO of KLM Axiva Finvest with this email/phone; company site/SEBI prospectus could not be directly fetched (network egress blocked) for primary-source cross-check</t>
+        </is>
+      </c>
+      <c r="Y5" s="3" t="inlineStr">
+        <is>
+          <t>Two independent data-aggregator sources agree on name/title/email/phone, but not primary-source confirmed - recommend a verification call before outreach.</t>
+        </is>
+      </c>
+      <c r="Z5" s="4" t="inlineStr">
+        <is>
+          <t>Srikanth G. Menon | Company Secretary &amp; Compliance Officer | cs@klmaxiva.com | +91-484-4281118  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1055,16 +1182,36 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R6" s="4" t="n"/>
-      <c r="S6" s="4" t="n"/>
-      <c r="T6" s="4" t="n"/>
-      <c r="U6" s="4" t="n"/>
-      <c r="V6" s="4" t="n"/>
-      <c r="W6" s="4" t="n"/>
-      <c r="X6" s="4" t="n"/>
-      <c r="Y6" s="4" t="n"/>
+      <c r="R6" s="6" t="n"/>
+      <c r="S6" s="6" t="n"/>
+      <c r="T6" s="6" t="n"/>
+      <c r="U6" s="6" t="n"/>
+      <c r="V6" s="6" t="inlineStr">
+        <is>
+          <t>Registered office: Shakti Bhawan, 14 Ashok Marg, Lucknow (UPPTCL headquarters)</t>
+        </is>
+      </c>
+      <c r="W6" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X6" s="6" t="inlineStr">
+        <is>
+          <t>upptcl.org Corporate Directory page, via search snippet - direct WebFetch to upptcl.org was blocked by network egress so could not be independently confirmed</t>
+        </is>
+      </c>
+      <c r="Y6" s="6" t="inlineStr">
+        <is>
+          <t>UPPTCL is a UP state-government transmission utility. Extensive search did not turn up a distinctly named CFO/Director(Finance)/Finance Controller for UPPTCL specifically - most 'Director (Finance)' hits found (e.g. Nidhi Narang, Sanjay Mehrotra) belong to the separate sister entity UPPCL and must NOT be used for this row. MD Mayur Maheshwari, IAS is the best-verified named senior contact but is not a finance-specific role, so omitted from contact and left as fallback-only. Existing on-file contact (hem.kumar.agrawar@gmail.com) was not re-verified.</t>
+        </is>
+      </c>
       <c r="Z6" s="4" t="n"/>
-      <c r="AA6" s="4" t="n"/>
+      <c r="AA6" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1145,16 +1292,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R7" s="4" t="n"/>
-      <c r="S7" s="4" t="n"/>
-      <c r="T7" s="4" t="n"/>
-      <c r="U7" s="4" t="n"/>
-      <c r="V7" s="4" t="n"/>
-      <c r="W7" s="4" t="n"/>
-      <c r="X7" s="4" t="n"/>
-      <c r="Y7" s="4" t="n"/>
-      <c r="Z7" s="4" t="n"/>
-      <c r="AA7" s="4" t="n"/>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>Gunjan Jain (CA)</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="n"/>
+      <c r="U7" s="3" t="n"/>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>ir@mufinfinance.com / vishwas.kumar@mufinfinance.com (Investor Relations)</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>BSE corporate filing (Oct 2025); Bloomberg Markets profile; MarketScreener insider profile; Energetica India interview (May 2026)</t>
+        </is>
+      </c>
+      <c r="Y7" s="3" t="inlineStr">
+        <is>
+          <t>One search pass surfaced an unverified claim of her departure (Mar 2026) but this was not corroborated by later 2026 sources (interview / earnings-call reference) - recommend confirming she is still in-role before outreach. No direct personal email/mobile found; used verified IR contacts as fallback.</t>
+        </is>
+      </c>
+      <c r="Z7" s="4" t="inlineStr">
+        <is>
+          <t>Vishwas Kumar | Investor Relations Manager | vishwas.kumar@mufinfinance.com | 011-43094300 (general company line, on file) / info@mufinfinance.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1215,16 +1394,54 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R8" s="4" t="n"/>
-      <c r="S8" s="4" t="n"/>
-      <c r="T8" s="4" t="n"/>
-      <c r="U8" s="4" t="n"/>
-      <c r="V8" s="4" t="n"/>
-      <c r="W8" s="4" t="n"/>
-      <c r="X8" s="4" t="n"/>
-      <c r="Y8" s="4" t="n"/>
-      <c r="Z8" s="4" t="n"/>
-      <c r="AA8" s="4" t="n"/>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>Atul Tibrewal</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="n"/>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>atul.tibrewal@northernarc.com</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>ir.investments@northernarc.com / +91-44-6668 7000 (registered office)</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X8" s="5" t="inlineStr">
+        <is>
+          <t>Bloomberg Markets profile and Northern Arc management-team page confirm Atul Tibrewal as CFO since May 2021; email is INFERRED from the confirmed firstname.lastname@northernarc.com pattern (verified via Chetan Parmar's official press-release address, see additional[0])</t>
+        </is>
+      </c>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>Identity/designation well-corroborated (Bloomberg + company site + ZoomInfo/RocketReach agree), but no personal email/mobile for Tibrewal independently found - email listed is a pattern-based inference, treat as medium only. Use IR desk fallback for reliable outreach.</t>
+        </is>
+      </c>
+      <c r="Z8" s="4" t="inlineStr">
+        <is>
+          <t>Chetan Parmar | Head - Investor Relations | chetan.parmar@northernarc.com  (HIGH)
+Prakash Chandra Panda | Company Secretary &amp; Compliance Officer / Investor Grievance Nodal Officer | cs@northernarc.com | +91-44-6668 7000  (HIGH)
+Investor Relations desk (general) | ir.investments@northernarc.com  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA8" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1300,16 +1517,53 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R9" s="4" t="n"/>
-      <c r="S9" s="4" t="n"/>
-      <c r="T9" s="4" t="n"/>
-      <c r="U9" s="4" t="n"/>
-      <c r="V9" s="4" t="n"/>
-      <c r="W9" s="4" t="n"/>
-      <c r="X9" s="4" t="n"/>
-      <c r="Y9" s="4" t="n"/>
-      <c r="Z9" s="4" t="n"/>
-      <c r="AA9" s="4" t="n"/>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>Jasmine M.P</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="n"/>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>cfo@chemmanurcredits.com</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="inlineStr">
+        <is>
+          <t>+91-487-7121200 / 2424010, Extn. 213</t>
+        </is>
+      </c>
+      <c r="W9" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X9" s="3" t="inlineStr">
+        <is>
+          <t>Chemmanur Credits and Investments Ltd. Draft Prospectus - NCD Public Issue VI, dated 09-May-2025, hosted on BSE</t>
+        </is>
+      </c>
+      <c r="Y9" s="3" t="inlineStr">
+        <is>
+          <t>Company's own most recent (2025) NCD offer document naming the CFO with direct email and extension - strongest available source. Older annual reports named a different CFO (Pramod M) - superseded, see additional entry.</t>
+        </is>
+      </c>
+      <c r="Z9" s="4" t="inlineStr">
+        <is>
+          <t>Anju Thomas | Company Secretary &amp; Compliance Officer | cs@chemmanurcredits.com | +91-487-7121200 / 2424010, Extn. 204  (HIGH)
+Pramod M (Muthu Pramod) | Former Chief Financial Officer (historical, per 2021/2023-24 annual reports) | pramod@chemmanurcredits.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1390,16 +1644,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R10" s="4" t="n"/>
-      <c r="S10" s="4" t="n"/>
-      <c r="T10" s="4" t="n"/>
-      <c r="U10" s="4" t="n"/>
-      <c r="V10" s="4" t="n"/>
-      <c r="W10" s="4" t="n"/>
-      <c r="X10" s="4" t="n"/>
-      <c r="Y10" s="4" t="n"/>
-      <c r="Z10" s="4" t="n"/>
-      <c r="AA10" s="4" t="n"/>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>Ashok Kumar Modi</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="n"/>
+      <c r="U10" s="5" t="n"/>
+      <c r="V10" s="5" t="inlineStr">
+        <is>
+          <t>srghousing@gmail.com / +91-294-2412609, +91-294-2561882 (registered office)</t>
+        </is>
+      </c>
+      <c r="W10" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X10" s="5" t="inlineStr">
+        <is>
+          <t>Bloomberg Markets profile; LinkedIn; Trendlyne CFO salary page; company website management bio (srghousing.com)</t>
+        </is>
+      </c>
+      <c r="Y10" s="5" t="inlineStr">
+        <is>
+          <t>Identity/designation (CFO since 21-Oct-2014) corroborated by 4 independent sources - high confidence on person, but no personal email/mobile verified so left null per hard rules. NHB nodal-officer PDF associates a grievance mailbox (cgrcell@srghousing.com) with the company but not confirmed as his personal address.</t>
+        </is>
+      </c>
+      <c r="Z10" s="4" t="inlineStr">
+        <is>
+          <t>Tanushree Trivedi | Company Secretary &amp; Compliance Officer | srghousing@gmail.com | +91-294-2412609 / +91-294-2561882  (HIGH)
+Investor/Grievance mailbox (NHB nodal officer contact) | cgrcell@srghousing.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA10" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1470,16 +1757,50 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R11" s="4" t="n"/>
-      <c r="S11" s="4" t="n"/>
-      <c r="T11" s="4" t="n"/>
-      <c r="U11" s="4" t="n"/>
-      <c r="V11" s="4" t="n"/>
-      <c r="W11" s="4" t="n"/>
-      <c r="X11" s="4" t="n"/>
-      <c r="Y11" s="4" t="n"/>
-      <c r="Z11" s="4" t="n"/>
-      <c r="AA11" s="4" t="n"/>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>Jhummi Mantri</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (appointed w.e.f. 27-Jun-2024)</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="n"/>
+      <c r="U11" s="5" t="n"/>
+      <c r="V11" s="5" t="inlineStr">
+        <is>
+          <t>connect@aviom.in (on file); toll-free 1800 120 3466 (10AM-5PM Mon-Sat)</t>
+        </is>
+      </c>
+      <c r="W11" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X11" s="5" t="inlineStr">
+        <is>
+          <t>Aviom price-sensitive disclosure PDF re: CFO appointment, corroborated by RocketReach/ZoomInfo profile listings</t>
+        </is>
+      </c>
+      <c r="Y11" s="5" t="inlineStr">
+        <is>
+          <t>IMPORTANT: RBI superseded Aviom's board on 27-Jan-2025 over governance/fraud concerns; NCLT admitted CIRP on 20-Feb-2025 with an Administrator appointed. Unverified whether Jhummi Mantri remains CFO post-supersession - normal CFO-level outreach may not be operative; the Administrator/Resolution Professional is now the practical decision-making authority. No direct email/mobile found.</t>
+        </is>
+      </c>
+      <c r="Z11" s="4" t="inlineStr">
+        <is>
+          <t>Ram Kumar | RBI/NCLT-appointed Administrator (company under CIRP since Feb-2025)  (HIGH)
+Divyani Chand | Chief Compliance Officer &amp; Company Secretary  (LOW)
+Grievance Redressal / Nodal Officer desk (named individual conflicts across sources) | 8076298526 (general); toll-free 1800 120 3466 | Gro@aviom.in | 8076298526  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA11" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1540,16 +1861,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R12" s="4" t="n"/>
-      <c r="S12" s="4" t="n"/>
-      <c r="T12" s="4" t="n"/>
-      <c r="U12" s="4" t="n"/>
-      <c r="V12" s="4" t="n"/>
-      <c r="W12" s="4" t="n"/>
-      <c r="X12" s="4" t="n"/>
-      <c r="Y12" s="4" t="n"/>
-      <c r="Z12" s="4" t="n"/>
-      <c r="AA12" s="4" t="n"/>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>Amit Mor</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Prestige Group (Prestige Estates Projects Ltd - the listed parent)</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="n"/>
+      <c r="U12" s="5" t="n"/>
+      <c r="V12" s="5" t="inlineStr">
+        <is>
+          <t>investors@prestigeconstructions.com; +91 80 2599 1080 (Prestige Group HQ, Bengaluru)</t>
+        </is>
+      </c>
+      <c r="W12" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X12" s="5" t="inlineStr">
+        <is>
+          <t>prestigeconstructions.com/about-us/cfo/amit-mor, corroborated by Crunchbase and LinkedIn profiles</t>
+        </is>
+      </c>
+      <c r="Y12" s="5" t="inlineStr">
+        <is>
+          <t>Prestige Projects Pvt. Ltd. is a wholly-owned, debt-listed subsidiary used to issue NCDs/OCDs; does not appear to have its own dedicated CFO. Directors on record look like nominee/legal directors. Amit Mor as Group CFO oversees Treasury/Fund Raising group-wide but this is an inference, not a subsidiary-specific appointment. Personal email found only masked on RocketReach - not verifiable, left null.</t>
+        </is>
+      </c>
+      <c r="Z12" s="4" t="inlineStr">
+        <is>
+          <t>Registered/Secretarial email of Prestige Projects Pvt. Ltd. specifically | secretarial@prestigeconstructions.com | secretarial@prestigeconstructions.com  (MEDIUM)
+Manoj Krishna J V | Company Secretary &amp; Compliance Officer, Prestige Estates Projects Limited (parent)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA12" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1635,16 +1989,50 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R13" s="4" t="n"/>
-      <c r="S13" s="4" t="n"/>
-      <c r="T13" s="4" t="n"/>
-      <c r="U13" s="4" t="n"/>
-      <c r="V13" s="4" t="n"/>
-      <c r="W13" s="4" t="n"/>
-      <c r="X13" s="4" t="n"/>
-      <c r="Y13" s="4" t="n"/>
-      <c r="Z13" s="4" t="n"/>
-      <c r="AA13" s="4" t="n"/>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>Krishan Gopal</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer &amp; Key Managerial Personnel (effective 17-Jan-2026)</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="n"/>
+      <c r="U13" s="3" t="n"/>
+      <c r="V13" s="3" t="inlineStr">
+        <is>
+          <t>91-124-6910500 (corporate office, on file); customercare@fusionfin.com</t>
+        </is>
+      </c>
+      <c r="W13" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X13" s="3" t="inlineStr">
+        <is>
+          <t>MarketScreener/BSE-filing summary, corroborated independently by LinkedIn posts (CXO Lanes, Uni Network Group) and Prysm.fi news</t>
+        </is>
+      </c>
+      <c r="Y13" s="3" t="inlineStr">
+        <is>
+          <t>Prior CFO Gaurav Maheshwari (existing on-file email) resigned ~25-Jun-2025; Amandeep Singh served as Interim CFO until Krishan Gopal's appointment 17-Jan-2026. No personal email/mobile found - the existing gourav@fusionmicrofinance.com on file is now stale (predecessor).</t>
+        </is>
+      </c>
+      <c r="Z13" s="4" t="inlineStr">
+        <is>
+          <t>Amandeep Singh (CA) | Head of Finance &amp; Accounts (formerly Interim CFO, 26-Jun-2025 to 17-Jan-2026)  (HIGH)
+Vikrant Sadana | Company Secretary &amp; Compliance Officer (appointed w.e.f. 18-Aug-2025)  (HIGH)
+Deepak Madaan | Former Company Secretary &amp; Chief Compliance Officer (2013-circa 2025, superseded by Vikrant Sadana) | +91-124-6910600 | companysecretary@fusionmicrofinance.com | companysecretary@fusionmicrofinance.com / +91-124-6910600  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA13" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1705,16 +2093,49 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R14" s="4" t="n"/>
-      <c r="S14" s="4" t="n"/>
-      <c r="T14" s="4" t="n"/>
-      <c r="U14" s="4" t="n"/>
-      <c r="V14" s="4" t="n"/>
-      <c r="W14" s="4" t="n"/>
-      <c r="X14" s="4" t="n"/>
-      <c r="Y14" s="4" t="n"/>
-      <c r="Z14" s="4" t="n"/>
-      <c r="AA14" s="4" t="n"/>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>Vijendra Singh Shekhawat</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>CEO &amp; Director, Choice Finserv Pvt. Ltd. (CA; previously VP-Finance &amp; Accounts, Religare Enterprises Ltd.)</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="n"/>
+      <c r="U14" s="3" t="n"/>
+      <c r="V14" s="3" t="inlineStr">
+        <is>
+          <t>cfpl@choiceindia.com</t>
+        </is>
+      </c>
+      <c r="W14" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X14" s="3" t="inlineStr">
+        <is>
+          <t>MarketScreener India bio; whispersinthecorridors.com news item (Mar 2026); corroborated by LinkedIn profile and social posts</t>
+        </is>
+      </c>
+      <c r="Y14" s="3" t="inlineStr">
+        <is>
+          <t>Appointed CEO &amp; Director ~March 2026; strong finance background (ex VP-Finance &amp; Accounts, Religare) though current title is CEO not CFO - captured as best-available named finance-adjacent leader since no dedicated CFO verified for this subsidiary. A RocketReach-aggregated mobile surfaced but unconfirmed, deliberately omitted per no-fabrication policy.</t>
+        </is>
+      </c>
+      <c r="Z14" s="4" t="inlineStr">
+        <is>
+          <t>Ayush Sharma | CFO, Choice International Ltd. (listed parent / group CFO) | cfpl@choiceindia.com  (MEDIUM)
+Manoj Singhania | Former CFO, Choice International Ltd.; historically listed as a Director of Choice Finserv Pvt Ltd  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA14" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1785,16 +2206,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R15" s="4" t="n"/>
-      <c r="S15" s="4" t="n"/>
-      <c r="T15" s="4" t="n"/>
-      <c r="U15" s="4" t="n"/>
-      <c r="V15" s="4" t="n"/>
-      <c r="W15" s="4" t="n"/>
-      <c r="X15" s="4" t="n"/>
-      <c r="Y15" s="4" t="n"/>
-      <c r="Z15" s="4" t="n"/>
-      <c r="AA15" s="4" t="n"/>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Madhura Devidas Kale</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>Company Secretary, Hazaribagh Ranchi Expressway Ltd.</t>
+        </is>
+      </c>
+      <c r="T15" s="5" t="n"/>
+      <c r="U15" s="5" t="n"/>
+      <c r="V15" s="5" t="inlineStr">
+        <is>
+          <t>secretarial@roadstarinfra.com (Tel: 022-26533333, Fax: 022-26523979)</t>
+        </is>
+      </c>
+      <c r="W15" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X15" s="5" t="inlineStr">
+        <is>
+          <t>thecompanycheck.com company profile (MCA-derived KMP data) - appointed CS 17 July 2023</t>
+        </is>
+      </c>
+      <c r="Y15" s="5" t="inlineStr">
+        <is>
+          <t>No CFO or Treasury head identified for this SPV. Ownership transferred from IL&amp;FS Transportation Networks Ltd to Roadstar Infra Investment Trust on 16 Dec 2022, so on-file itnl.secretarial@ilfsindia.com is very likely stale. Current registered contact confirmed via two independent recent NSE filings, so treated as high confidence even though named-person link is single-source/medium.</t>
+        </is>
+      </c>
+      <c r="Z15" s="4" t="inlineStr">
+        <is>
+          <t>Roadstar Infra secretarial/compliance desk (handles HREL's NCD and debt-related filings) | secretarial@roadstarinfra.com | 022-26533333 / fax 022-26523979  (HIGH)
+Sunil Hemchand Patel | Director, Hazaribagh Ranchi Expressway Ltd.  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA15" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1855,16 +2309,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R16" s="4" t="n"/>
-      <c r="S16" s="4" t="n"/>
-      <c r="T16" s="4" t="n"/>
-      <c r="U16" s="4" t="n"/>
-      <c r="V16" s="4" t="n"/>
-      <c r="W16" s="4" t="n"/>
-      <c r="X16" s="4" t="n"/>
-      <c r="Y16" s="4" t="n"/>
-      <c r="Z16" s="4" t="n"/>
-      <c r="AA16" s="4" t="n"/>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>Saket Saraf</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Dar Credit &amp; Capital Ltd.</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="n"/>
+      <c r="U16" s="5" t="n"/>
+      <c r="V16" s="5" t="inlineStr">
+        <is>
+          <t>kolkata@darcredit.com (Tel: +91-33-40646495 / 22873355)</t>
+        </is>
+      </c>
+      <c r="W16" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn (title: CFO - Dar Credit &amp; Capital Ltd.); corroborated by ZoomInfo/thecompanycheck.com listing the same KMP set (Jayanta Banik-CEO, Saket Saraf-CFO, Priya Kumari-CS)</t>
+        </is>
+      </c>
+      <c r="Y16" s="5" t="inlineStr">
+        <is>
+          <t>Company site darcredit.com was inaccessible (egress-blocked) so KMP page not directly verified. One search summary asserted a 'Megha Saraf' as CFO but no corroborating link found - likely a summarization artifact; flag for manual double-check against live site before outreach. No personal email/mobile independently verified.</t>
+        </is>
+      </c>
+      <c r="Z16" s="4" t="inlineStr">
+        <is>
+          <t>Priya Kumari | Company Secretary &amp; Compliance Officer, Dar Credit &amp; Capital Ltd. | Co.secretary@darcredit.com | kolkata@darcredit.com  (HIGH)
+Jayanta Banik | CEO, Dar Credit &amp; Capital Ltd. | kolkata@darcredit.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA16" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13117,7 +13604,7 @@
       <c r="AA165" s="4" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -13135,88 +13622,88 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>NCD Mobile - Enrichment legend</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr"/>
+      <c r="B1" s="8" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr"/>
-      <c r="B2" s="6" t="inlineStr"/>
+      <c r="A2" s="9" t="inlineStr"/>
+      <c r="B2" s="8" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Meaning (surety of the added contact)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>High - verified: official site / annual report / MCA / NCD offer doc, or 2+ sources agree</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>YELLOW</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Medium - plausible: single source, LinkedIn, or inferred email pattern</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>RED</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Low - weak / fallback: generic landline used instead of a person, or unverified</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr"/>
-      <c r="B7" s="6" t="inlineStr"/>
+      <c r="A7" s="9" t="inlineStr"/>
+      <c r="B7" s="8" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Priority order</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>CFO -&gt; Treasury head -&gt; Finance team -&gt; Fallback (landline / IR desk)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Rule</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Never fabricate a number. If nothing found, leave blank and mark status not_found.</t>
         </is>

</xml_diff>

<commit_message>
enrich batch (9PM pass): rows 15-29
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -2402,16 +2402,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R17" s="4" t="n"/>
-      <c r="S17" s="4" t="n"/>
-      <c r="T17" s="4" t="n"/>
-      <c r="U17" s="4" t="n"/>
-      <c r="V17" s="4" t="n"/>
-      <c r="W17" s="4" t="n"/>
-      <c r="X17" s="4" t="n"/>
-      <c r="Y17" s="4" t="n"/>
-      <c r="Z17" s="4" t="n"/>
-      <c r="AA17" s="4" t="n"/>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>Neeraj Gautam (Niraj Kumar Gautam)</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer, Puravankara Limited (parent group)</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="n"/>
+      <c r="U17" s="3" t="inlineStr">
+        <is>
+          <t>neeraj.gautam@puravankara.com</t>
+        </is>
+      </c>
+      <c r="V17" s="3" t="inlineStr">
+        <is>
+          <t>+91-80-4343 9794 (direct line, per Puravankara investor disclosure); investors@puravankara.com (Group IR desk); +91 80 2559 9000 (registered office)</t>
+        </is>
+      </c>
+      <c r="W17" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X17" s="3" t="inlineStr">
+        <is>
+          <t>Puravankara Ltd. investor-relations/regulatory contact disclosure (Nodal Officer-CFO listing); CFO-appointment announcements (MarketScreener, boardstewardship.com)</t>
+        </is>
+      </c>
+      <c r="Y17" s="3" t="inlineStr">
+        <is>
+          <t>Provident Cedar Pvt Ltd is a wholly-owned SPV under Provident Housing Ltd within the Puravankara Group; no dedicated CFO for this SPV was found (only non-finance directors listed). Finance is handled at Puravankara Group level. Neeraj Gautam elevated from Deputy-CFO to Group CFO effective 24-Sep-2025.</t>
+        </is>
+      </c>
+      <c r="Z17" s="4" t="inlineStr">
+        <is>
+          <t>Group Investor Relations desk | investors@puravankara.com | +91 80 2559 9000 / 4343 9999  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA17" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2472,16 +2508,48 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R18" s="4" t="n"/>
-      <c r="S18" s="4" t="n"/>
-      <c r="T18" s="4" t="n"/>
-      <c r="U18" s="4" t="n"/>
-      <c r="V18" s="4" t="n"/>
-      <c r="W18" s="4" t="n"/>
-      <c r="X18" s="4" t="n"/>
-      <c r="Y18" s="4" t="n"/>
-      <c r="Z18" s="4" t="n"/>
-      <c r="AA18" s="4" t="n"/>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>Rajesh Poddar (Rajesh Kumar Poddar)</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Adani Airport Holdings Ltd. (appointed effective 29-Apr-2025)</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="n"/>
+      <c r="U18" s="3" t="n"/>
+      <c r="V18" s="3" t="inlineStr">
+        <is>
+          <t>aahl.feedback@adani.com; Tel +91 79 2656 5555 (AAHL registered office, Ahmedabad)</t>
+        </is>
+      </c>
+      <c r="W18" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X18" s="3" t="inlineStr">
+        <is>
+          <t>Equilar ExecAtlas, LinkedIn, corroborated by RocketReach and ZoomInfo profiles all naming him CFO of AAHL since Apr-2025</t>
+        </is>
+      </c>
+      <c r="Y18" s="3" t="inlineStr">
+        <is>
+          <t>Name/title/appointment date corroborated across 3+ independent sources, but direct email/mobile only found masked in paid people-databases - not independently verified so left null. Predecessor Rakesh Kumar Tiwary resigned ~Mar-2025, moved to CFO of Ambuja Cements Ltd.</t>
+        </is>
+      </c>
+      <c r="Z18" s="4" t="inlineStr">
+        <is>
+          <t>Corporate/Investor feedback desk, Adani Airport Holdings Ltd. | aahl.feedback@adani.com | +91 79 2656 5555  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA18" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2542,16 +2610,45 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R19" s="4" t="n"/>
-      <c r="S19" s="4" t="n"/>
-      <c r="T19" s="4" t="n"/>
-      <c r="U19" s="4" t="n"/>
-      <c r="V19" s="4" t="n"/>
-      <c r="W19" s="4" t="n"/>
-      <c r="X19" s="4" t="n"/>
-      <c r="Y19" s="4" t="n"/>
-      <c r="Z19" s="4" t="n"/>
-      <c r="AA19" s="4" t="n"/>
+      <c r="R19" s="3" t="inlineStr">
+        <is>
+          <t>Amit Mor</t>
+        </is>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer, Prestige Group / Prestige Estates Projects Ltd.</t>
+        </is>
+      </c>
+      <c r="T19" s="3" t="n"/>
+      <c r="U19" s="3" t="n"/>
+      <c r="V19" s="3" t="n"/>
+      <c r="W19" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X19" s="3" t="inlineStr">
+        <is>
+          <t>Prestige Group's own leadership bio page corroborated by LinkedIn; ICRA rating rationale confirms Prestige Group holds 51% of Bamboo Hotel &amp; Global Centre (Delhi) Pvt Ltd and PEPL guarantees its NCDs</t>
+        </is>
+      </c>
+      <c r="Y19" s="3" t="inlineStr">
+        <is>
+          <t>Bamboo Hotel is an SPV/JV - Prestige Group 51%, Valor Estate Group (ex-DB Realty) 49% - with no standalone CFO for the SPV itself. Prestige's Group CFO Amit Mor is the most relevant single contact as majority partner and NCD guarantor.</t>
+        </is>
+      </c>
+      <c r="Z19" s="4" t="inlineStr">
+        <is>
+          <t>Atul Bhatnagar | Chief Financial Officer (also 'Joint CFO'), Valor Estate Ltd. (formerly DB Realty Ltd.; 49% JV partner)  (HIGH)
+Deepak Ghangurde | Chief Financial Officer / VP-Legal &amp; Finance, Balwa Group (promoter family group behind Valor Estate/DB Realty)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA19" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2632,16 +2729,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R20" s="4" t="n"/>
-      <c r="S20" s="4" t="n"/>
-      <c r="T20" s="4" t="n"/>
-      <c r="U20" s="4" t="n"/>
-      <c r="V20" s="4" t="n"/>
-      <c r="W20" s="4" t="n"/>
-      <c r="X20" s="4" t="n"/>
-      <c r="Y20" s="4" t="n"/>
-      <c r="Z20" s="4" t="n"/>
-      <c r="AA20" s="4" t="n"/>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>Sonal Sharma</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>Company Secretary &amp; Compliance Officer, TruCap Finance Ltd.</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="n"/>
+      <c r="U20" s="3" t="inlineStr">
+        <is>
+          <t>corpsec@trucapfinance.com</t>
+        </is>
+      </c>
+      <c r="V20" s="3" t="inlineStr">
+        <is>
+          <t>022-6845 7200 (company landline)</t>
+        </is>
+      </c>
+      <c r="W20" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X20" s="3" t="inlineStr">
+        <is>
+          <t>TruCap Finance Ltd. official Investor Relations / Board &amp; Management pages and multiple corroborating BSE/NSE compliance filing references</t>
+        </is>
+      </c>
+      <c r="Y20" s="3" t="inlineStr">
+        <is>
+          <t>TruCap Finance has NO confirmed permanent CFO as of Aug 2026: former CFO Sanjay Kukreja departed; interim CFO Vishal Miglani (appointed 14-Nov-2025) resigned effective 24-May-2026; an earlier Finance Head appointee (Saurabh Sethi) also exited. Captured the Company Secretary handling compliance/debt correspondence as the best verified contact.</t>
+        </is>
+      </c>
+      <c r="Z20" s="4" t="inlineStr">
+        <is>
+          <t>Amruta Kamat | Manager - Corporate Secretarial and Compliance, TruCap Finance Ltd. | corpsec@trucapfinance.com | 022-6845 7200  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA20" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2722,16 +2855,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R21" s="4" t="n"/>
-      <c r="S21" s="4" t="n"/>
-      <c r="T21" s="4" t="n"/>
-      <c r="U21" s="4" t="n"/>
-      <c r="V21" s="4" t="n"/>
-      <c r="W21" s="4" t="n"/>
-      <c r="X21" s="4" t="n"/>
-      <c r="Y21" s="4" t="n"/>
-      <c r="Z21" s="4" t="n"/>
-      <c r="AA21" s="4" t="n"/>
+      <c r="R21" s="3" t="inlineStr">
+        <is>
+          <t>Anurag Kapil</t>
+        </is>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>Director (Finance) &amp; Chief Financial Officer, NMDC Steel Ltd. (DIN 06640383)</t>
+        </is>
+      </c>
+      <c r="T21" s="3" t="n"/>
+      <c r="U21" s="3" t="n"/>
+      <c r="V21" s="3" t="inlineStr">
+        <is>
+          <t>cs_nisp@nmdc.co.in / 040-23538713, 040-23538723, 040-23538767 (NMDC Steel corporate office, Hyderabad)</t>
+        </is>
+      </c>
+      <c r="W21" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X21" s="3" t="inlineStr">
+        <is>
+          <t>Ministry of Steel order/exchange filing dated 31-Mar-2026, corroborated by TipRanks, InvestyWise, ScanX, PSU Connect, IndianMasterminds</t>
+        </is>
+      </c>
+      <c r="Y21" s="3" t="inlineStr">
+        <is>
+          <t>Appointed by the Ministry of Steel for a 5-year term effective 31-Mar-2026, replacing K Raj Shekhar. No direct personal email/mobile found publicly; corporate-office contact used as fallback (distinct from parent NMDC Ltd.'s cs@nmdc.co.in on file).</t>
+        </is>
+      </c>
+      <c r="Z21" s="4" t="inlineStr">
+        <is>
+          <t>Paraj Kanti Saha | Company Secretary &amp; Compliance Officer, NMDC Steel Ltd. | cs_nisp@nmdc.co.in | 040-23538713 / 23538723 / 23538767  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA21" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2792,16 +2957,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R22" s="4" t="n"/>
-      <c r="S22" s="4" t="n"/>
-      <c r="T22" s="4" t="n"/>
-      <c r="U22" s="4" t="n"/>
-      <c r="V22" s="4" t="n"/>
-      <c r="W22" s="4" t="n"/>
-      <c r="X22" s="4" t="n"/>
-      <c r="Y22" s="4" t="n"/>
-      <c r="Z22" s="4" t="n"/>
-      <c r="AA22" s="4" t="n"/>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>Mayank Jiniwal</t>
+        </is>
+      </c>
+      <c r="S22" s="5" t="inlineStr">
+        <is>
+          <t>CFO, DBL Infra Assets Pvt. Ltd. (also General Manager - Finance, Dilip Buildcon Ltd., the group/parent company)</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="n"/>
+      <c r="U22" s="5" t="n"/>
+      <c r="V22" s="5" t="inlineStr">
+        <is>
+          <t>dblinfraassets@gmail.com (existing registered email on file)</t>
+        </is>
+      </c>
+      <c r="W22" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X22" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn profile identifying him as CFO, DBL Infra Assets Pvt Ltd; corroborated by ZaubaCorp director listing for the company</t>
+        </is>
+      </c>
+      <c r="Y22" s="5" t="inlineStr">
+        <is>
+          <t>Designation confirmed via LinkedIn only, capped at medium confidence. A masked RocketReach email (Dilip Buildcon domain) is unverified and not usable. No public direct phone number found.</t>
+        </is>
+      </c>
+      <c r="Z22" s="4" t="inlineStr">
+        <is>
+          <t>Sanjay Kumar Bansal | CFO, Dilip Buildcon Ltd. (parent/group company of DBL Infra Assets) | +91-755-4029999 (Dilip Buildcon Ltd. general company line, Bhopal)  (LOW)
+Gautam Jain | Head - Investor Relations, Dilip Buildcon Ltd. (parent group company)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA22" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2887,16 +3085,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R23" s="4" t="n"/>
-      <c r="S23" s="4" t="n"/>
-      <c r="T23" s="4" t="n"/>
-      <c r="U23" s="4" t="n"/>
-      <c r="V23" s="4" t="n"/>
-      <c r="W23" s="4" t="n"/>
-      <c r="X23" s="4" t="n"/>
-      <c r="Y23" s="4" t="n"/>
-      <c r="Z23" s="4" t="n"/>
-      <c r="AA23" s="4" t="n"/>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Bipeen (Bipin) Yashwant Valame</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>Group CFO &amp; Executive Director</t>
+        </is>
+      </c>
+      <c r="T23" s="5" t="n"/>
+      <c r="U23" s="5" t="inlineStr">
+        <is>
+          <t>bipeen.valame@jains.com</t>
+        </is>
+      </c>
+      <c r="V23" s="5" t="inlineStr">
+        <is>
+          <t>jisl@jains.com / investor.corr@jains.com, +91-257-2258011</t>
+        </is>
+      </c>
+      <c r="W23" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X23" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn, TheOrg, MarketScreener bio, and Q4FY26/Q1FY27 earnings-call coverage all confirm Bipeen Valame as CFO since March 2023</t>
+        </is>
+      </c>
+      <c r="Y23" s="5" t="inlineStr">
+        <is>
+          <t>Name/designation high confidence (3+ sources). Personal email NOT independently verified - inferred from the confirmed firstname.lastname@jains.com domain pattern (verified via CS Avdhut Ghodgaonkar's real address). Treat email as medium-confidence inference.</t>
+        </is>
+      </c>
+      <c r="Z23" s="4" t="inlineStr">
+        <is>
+          <t>Avdhut V. Ghodgaonkar | Company Secretary &amp; Chief Compliance Officer (handles SEBI/stock-exchange &amp; debt compliance matters) | avdhut.ghodgaonkar@jains.com | Tel +91-257-2258011, Fax +91-257-2258111  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA23" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2972,16 +3206,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R24" s="4" t="n"/>
-      <c r="S24" s="4" t="n"/>
-      <c r="T24" s="4" t="n"/>
-      <c r="U24" s="4" t="n"/>
-      <c r="V24" s="4" t="n"/>
-      <c r="W24" s="4" t="n"/>
-      <c r="X24" s="4" t="n"/>
-      <c r="Y24" s="4" t="n"/>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
+          <t>Manish Girish Modani</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T24" s="3" t="n"/>
+      <c r="U24" s="3" t="inlineStr">
+        <is>
+          <t>manish.modani@rdcconcreteindia.com</t>
+        </is>
+      </c>
+      <c r="V24" s="3" t="inlineStr">
+        <is>
+          <t>91-11-6854550 (existing on file; note current registered office is Thane, Maharashtra, so this Delhi landline may be outdated)</t>
+        </is>
+      </c>
+      <c r="W24" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X24" s="3" t="inlineStr">
+        <is>
+          <t>TheOrg, LinkedIn, ZoomInfo and RocketReach all independently confirm Manish Modani as CFO with this exact email address</t>
+        </is>
+      </c>
+      <c r="Y24" s="3" t="inlineStr">
+        <is>
+          <t>Confirms the existing_reg_email on file already belongs to the CFO. Modani joined RDC Concrete in 2016 as Head of Finance &amp; Accounts, promoted to CFO in 2019.</t>
+        </is>
+      </c>
       <c r="Z24" s="4" t="n"/>
-      <c r="AA24" s="4" t="n"/>
+      <c r="AA24" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3032,16 +3298,56 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R25" s="4" t="n"/>
-      <c r="S25" s="4" t="n"/>
-      <c r="T25" s="4" t="n"/>
-      <c r="U25" s="4" t="n"/>
-      <c r="V25" s="4" t="n"/>
-      <c r="W25" s="4" t="n"/>
-      <c r="X25" s="4" t="n"/>
-      <c r="Y25" s="4" t="n"/>
-      <c r="Z25" s="4" t="n"/>
-      <c r="AA25" s="4" t="n"/>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>Niraj Kumar Gautam (also seen as "Neeraj Gautam")</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer, Puravankara Limited (parent group; Provident Meryta Pvt Ltd is a Puravankara/Provident Housing project SPV with no separate finance team)</t>
+        </is>
+      </c>
+      <c r="T25" s="5" t="inlineStr">
+        <is>
+          <t>+91-80-4343 9794</t>
+        </is>
+      </c>
+      <c r="U25" s="5" t="inlineStr">
+        <is>
+          <t>neeraj.gautam@puravankara.com</t>
+        </is>
+      </c>
+      <c r="V25" s="5" t="inlineStr">
+        <is>
+          <t>investors@puravankara.com, +91 80 2559 9000 / 4343 9999</t>
+        </is>
+      </c>
+      <c r="W25" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X25" s="5" t="inlineStr">
+        <is>
+          <t>MarketScreener/HR news coverage of his Sept 24, 2025 CFO appointment; email/phone per ZoomInfo and RocketReach aggregator listings</t>
+        </is>
+      </c>
+      <c r="Y25" s="5" t="inlineStr">
+        <is>
+          <t>Provident Meryta itself has no dedicated CFO. Name/appointment corroborated (boardstewardship.com, Business Standard), but personal email/mobile only from data-aggregator sites, capped at medium. The existing_reg_email on file (bindu.d@puravankara.com) appears STALE - current Group Head-CS is Sudip Chatterjee.</t>
+        </is>
+      </c>
+      <c r="Z25" s="4" t="inlineStr">
+        <is>
+          <t>Sudip Chatterjee | Group Head - Company Secretary &amp; Compliance Officer, Puravankara Limited | investors@puravankara.com, +91 80 2559 9000  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA25" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3122,16 +3428,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R26" s="4" t="n"/>
-      <c r="S26" s="4" t="n"/>
-      <c r="T26" s="4" t="n"/>
-      <c r="U26" s="4" t="n"/>
-      <c r="V26" s="4" t="n"/>
-      <c r="W26" s="4" t="n"/>
-      <c r="X26" s="4" t="n"/>
-      <c r="Y26" s="4" t="n"/>
-      <c r="Z26" s="4" t="n"/>
-      <c r="AA26" s="4" t="n"/>
+      <c r="R26" s="3" t="inlineStr">
+        <is>
+          <t>Lalbert Cherian</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="n"/>
+      <c r="U26" s="3" t="n"/>
+      <c r="V26" s="3" t="inlineStr">
+        <is>
+          <t>kings.infra@gmail.com / 91-80-28462200 (registered office)</t>
+        </is>
+      </c>
+      <c r="W26" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X26" s="3" t="inlineStr">
+        <is>
+          <t>Kings Infra Ventures 37th AGM Summary of Proceedings (kingsinfra.com, Sept 2025) naming Lalbert Cheriyan as CFO; corroborated by MarketScreener/Reuters brief and FY2025-26 results press release (June 2026, aninews.in)</t>
+        </is>
+      </c>
+      <c r="Y26" s="3" t="inlineStr">
+        <is>
+          <t>No verified direct email or mobile found; a ZoomInfo masked email could not be confirmed, so excluded rather than guessed.</t>
+        </is>
+      </c>
+      <c r="Z26" s="4" t="inlineStr">
+        <is>
+          <t>Nanditha T | Company Secretary &amp; Compliance Officer | cs@kingsinfra.com (company CS-line email, not individually confirmed as hers)  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA26" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3192,16 +3530,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R27" s="4" t="n"/>
-      <c r="S27" s="4" t="n"/>
-      <c r="T27" s="4" t="n"/>
-      <c r="U27" s="4" t="n"/>
-      <c r="V27" s="4" t="n"/>
-      <c r="W27" s="4" t="n"/>
-      <c r="X27" s="4" t="n"/>
-      <c r="Y27" s="4" t="n"/>
-      <c r="Z27" s="4" t="n"/>
-      <c r="AA27" s="4" t="n"/>
+      <c r="R27" s="5" t="inlineStr">
+        <is>
+          <t>Rajeev Nair (also referenced as M.R. Rajeev / Rajeev Madhavan Nair)</t>
+        </is>
+      </c>
+      <c r="S27" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T27" s="5" t="n"/>
+      <c r="U27" s="5" t="n"/>
+      <c r="V27" s="5" t="inlineStr">
+        <is>
+          <t>muthoot.enterprises@gmail.com (existing registered email)</t>
+        </is>
+      </c>
+      <c r="W27" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X27" s="5" t="inlineStr">
+        <is>
+          <t>RocketReach profile 'Muthoot Mercantile Ltd Chief Financial Officer' (Rajeev Nair); corroborated by a company event reference and director-list name match on ZaubaCorp</t>
+        </is>
+      </c>
+      <c r="Y27" s="5" t="inlineStr">
+        <is>
+          <t>Single confirmed CFO name via 2 low-authority sources plus a director-list match; could not verify via annual report or a personal email/mobile, left null rather than inferred. Confirmed distinct from Muthoot Finance/Muthoot Capital executives.</t>
+        </is>
+      </c>
+      <c r="Z27" s="4" t="inlineStr">
+        <is>
+          <t>Neethu C Biju | Company Secretary &amp; Compliance Officer  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA27" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3277,16 +3647,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R28" s="4" t="n"/>
-      <c r="S28" s="4" t="n"/>
-      <c r="T28" s="4" t="n"/>
-      <c r="U28" s="4" t="n"/>
-      <c r="V28" s="4" t="n"/>
-      <c r="W28" s="4" t="n"/>
-      <c r="X28" s="4" t="n"/>
-      <c r="Y28" s="4" t="n"/>
-      <c r="Z28" s="4" t="n"/>
-      <c r="AA28" s="4" t="n"/>
+      <c r="R28" s="3" t="inlineStr">
+        <is>
+          <t>Saurabh Chawla</t>
+        </is>
+      </c>
+      <c r="S28" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (KMP), GMR Airports Ltd (seconded from GMR Group, where he is Group CFO &amp; Executive Director - Finance &amp; Strategy)</t>
+        </is>
+      </c>
+      <c r="T28" s="3" t="n"/>
+      <c r="U28" s="3" t="n"/>
+      <c r="V28" s="3" t="inlineStr">
+        <is>
+          <t>gil.cosecy@gmrgroup.in / 91-80-49216751 (existing registered CS email/phone)</t>
+        </is>
+      </c>
+      <c r="W28" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X28" s="3" t="inlineStr">
+        <is>
+          <t>Bloomberg Markets executive profile; MarketScreener insider profile; TheOrg GMR Group org chart</t>
+        </is>
+      </c>
+      <c r="Y28" s="3" t="inlineStr">
+        <is>
+          <t>No individually verified direct email/mobile found; not guessed. Entity-level KMP CFO, distinct from GMR Hyderabad Airport (GHIAL) subsidiary's separately reported CFO-designate.</t>
+        </is>
+      </c>
+      <c r="Z28" s="4" t="inlineStr">
+        <is>
+          <t>Ankit Nandu | Associate General Manager - Investor Relations, GMR Group  (MEDIUM)
+Amit Jain | Head - Investor Relations (title per LinkedIn, at 'GMR Ltd')  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA28" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3347,16 +3750,53 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R29" s="4" t="n"/>
-      <c r="S29" s="4" t="n"/>
-      <c r="T29" s="4" t="n"/>
-      <c r="U29" s="4" t="n"/>
-      <c r="V29" s="4" t="n"/>
-      <c r="W29" s="4" t="n"/>
-      <c r="X29" s="4" t="n"/>
-      <c r="Y29" s="4" t="n"/>
-      <c r="Z29" s="4" t="n"/>
-      <c r="AA29" s="4" t="n"/>
+      <c r="R29" s="5" t="inlineStr">
+        <is>
+          <t>Niraj Kumar Gautam</t>
+        </is>
+      </c>
+      <c r="S29" s="5" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer, Puravankara Limited (parent); also listed as a Director of Purva Oak Pvt. Ltd. itself</t>
+        </is>
+      </c>
+      <c r="T29" s="5" t="n"/>
+      <c r="U29" s="5" t="inlineStr">
+        <is>
+          <t>niraj.g@puravankara.com</t>
+        </is>
+      </c>
+      <c r="V29" s="5" t="inlineStr">
+        <is>
+          <t>investors@puravankara.com</t>
+        </is>
+      </c>
+      <c r="W29" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X29" s="5" t="inlineStr">
+        <is>
+          <t>Puravankara Limited official corporate announcement 'Appoints Niraj Kumar Gautam as CFO' effective 24-Sep-2025; ZaubaCorp company record for Purva Oak Pvt. Ltd. lists him among current directors</t>
+        </is>
+      </c>
+      <c r="Y29" s="5" t="inlineStr">
+        <is>
+          <t>Name/designation high-confidence (official appointment + confirmed director on Purva Oak itself). Email is NOT verified for Gautam personally - an INFERRED guess from the on-file address pattern; treat as unconfirmed and verify before use. Downgraded to medium because of the unverified email.</t>
+        </is>
+      </c>
+      <c r="Z29" s="4" t="inlineStr">
+        <is>
+          <t>Jyoti Sahu | Company Secretary &amp; Compliance Officer, Puravankara Limited (handles investor/debenture-holder grievances for the group, including SPVs like Purva Oak) | investors@puravankara.com  (MEDIUM)
+Debenture Trustee (institutional, not a company employee) | Catalyst Trusteeship Limited, 901, 9th Floor, Tower-B, Peninsula Business Park, Lower Parel (W), Mumbai  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA29" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3417,16 +3857,44 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R30" s="4" t="n"/>
-      <c r="S30" s="4" t="n"/>
-      <c r="T30" s="4" t="n"/>
-      <c r="U30" s="4" t="n"/>
-      <c r="V30" s="4" t="n"/>
-      <c r="W30" s="4" t="n"/>
-      <c r="X30" s="4" t="n"/>
-      <c r="Y30" s="4" t="n"/>
+      <c r="R30" s="5" t="inlineStr">
+        <is>
+          <t>Chandramouli Akkiraju (also seen as Akkiraju Chandramouli / Chandra Mouli Akkiraju)</t>
+        </is>
+      </c>
+      <c r="S30" s="5" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer &amp; Director, Heritage Finlease Ltd. (no separately titled CFO/Head-Finance found; at this company size the CEO appears to also oversee finance)</t>
+        </is>
+      </c>
+      <c r="T30" s="5" t="n"/>
+      <c r="U30" s="5" t="n"/>
+      <c r="V30" s="5" t="inlineStr">
+        <is>
+          <t>hfinlease@gmail.com</t>
+        </is>
+      </c>
+      <c r="W30" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X30" s="5" t="inlineStr">
+        <is>
+          <t>Heritage Finlease Ltd. official site (board-of-directors/management-team pages); LinkedIn profile; ZoomInfo company/employee profile</t>
+        </is>
+      </c>
+      <c r="Y30" s="5" t="inlineStr">
+        <is>
+          <t>Consistently named across company site, LinkedIn, ZoomInfo/RocketReach as CEO and board director. No named CFO/VP-Finance/Treasury head found for this small NBFC. Personal email only partially shown by an aggregator, left null.</t>
+        </is>
+      </c>
       <c r="Z30" s="4" t="n"/>
-      <c r="AA30" s="4" t="n"/>
+      <c r="AA30" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3477,16 +3945,52 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R31" s="4" t="n"/>
-      <c r="S31" s="4" t="n"/>
-      <c r="T31" s="4" t="n"/>
-      <c r="U31" s="4" t="n"/>
-      <c r="V31" s="4" t="n"/>
-      <c r="W31" s="4" t="n"/>
-      <c r="X31" s="4" t="n"/>
-      <c r="Y31" s="4" t="n"/>
-      <c r="Z31" s="4" t="n"/>
-      <c r="AA31" s="4" t="n"/>
+      <c r="R31" s="5" t="inlineStr">
+        <is>
+          <t>Rambhupal Reddy</t>
+        </is>
+      </c>
+      <c r="S31" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Virtuous Retail (VR Bharat / VR group - the operating group that runs V R Dakshin Pvt. Ltd.'s malls)</t>
+        </is>
+      </c>
+      <c r="T31" s="5" t="n"/>
+      <c r="U31" s="5" t="inlineStr">
+        <is>
+          <t>r_reddy@virtuousretail.com</t>
+        </is>
+      </c>
+      <c r="V31" s="5" t="inlineStr">
+        <is>
+          <t>cs_vrb@vrbharat.com</t>
+        </is>
+      </c>
+      <c r="W31" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X31" s="5" t="inlineStr">
+        <is>
+          <t>ZoomInfo profile 'Chief Financial Officer at Virtuous Retail - Rambhupal Reddy'; RocketReach Virtuous Retail management/finance-department org chart</t>
+        </is>
+      </c>
+      <c r="Y31" s="5" t="inlineStr">
+        <is>
+          <t>Identified via two independent data-aggregator sources agreeing on name/title, but not confirmed via company site/LinkedIn, kept at medium. Email is an INFERRED guess based on the on-file address pattern; treat as unconfirmed. Could not verify who the existing on-file contact 'R K Malpani' is or whether that person still holds a finance role.</t>
+        </is>
+      </c>
+      <c r="Z31" s="4" t="inlineStr">
+        <is>
+          <t>Company Secretary / Compliance desk, VR Bharat group | cs_vrb@vrbharat.com | cs_vrb@vrbharat.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA31" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">

</xml_diff>

<commit_message>
enrich batch (9PM pass): rows 30-44
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -4071,16 +4071,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R32" s="4" t="n"/>
-      <c r="S32" s="4" t="n"/>
-      <c r="T32" s="4" t="n"/>
-      <c r="U32" s="4" t="n"/>
-      <c r="V32" s="4" t="n"/>
-      <c r="W32" s="4" t="n"/>
-      <c r="X32" s="4" t="n"/>
-      <c r="Y32" s="4" t="n"/>
-      <c r="Z32" s="4" t="n"/>
-      <c r="AA32" s="4" t="n"/>
+      <c r="R32" s="3" t="inlineStr">
+        <is>
+          <t>Nitin Goel</t>
+        </is>
+      </c>
+      <c r="S32" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO) &amp; KMP</t>
+        </is>
+      </c>
+      <c r="T32" s="3" t="n"/>
+      <c r="U32" s="3" t="n"/>
+      <c r="V32" s="3" t="inlineStr">
+        <is>
+          <t>investors@tarc.in</t>
+        </is>
+      </c>
+      <c r="W32" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X32" s="3" t="inlineStr">
+        <is>
+          <t>BSE exchange filing / Trendlyne 'Appointment Of Mr. Nitin Goel As Chief Financial Officer'; IndiaInfoline news; LinkedIn confirms current role 'CFO at TARC Ltd.'</t>
+        </is>
+      </c>
+      <c r="Y32" s="3" t="inlineStr">
+        <is>
+          <t>Appointed CFO &amp; KMP effective 11-Aug-2022; confirmed by 3 independent sources. Direct personal email/mobile could not be verified from an official source - data aggregators show masked/unverified details, deliberately excluded per no-fabrication policy.</t>
+        </is>
+      </c>
+      <c r="Z32" s="4" t="inlineStr">
+        <is>
+          <t>Amit Narayan | Company Secretary (handles investor/debt-related secretarial matters) | cs@tarc.in  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA32" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4141,16 +4173,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R33" s="4" t="n"/>
-      <c r="S33" s="4" t="n"/>
-      <c r="T33" s="4" t="n"/>
-      <c r="U33" s="4" t="n"/>
-      <c r="V33" s="4" t="n"/>
-      <c r="W33" s="4" t="n"/>
-      <c r="X33" s="4" t="n"/>
-      <c r="Y33" s="4" t="n"/>
-      <c r="Z33" s="4" t="n"/>
-      <c r="AA33" s="4" t="n"/>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>Dilip Agarwal</t>
+        </is>
+      </c>
+      <c r="S33" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Tata Realty and Infrastructure Ltd (parent/group finance head; Infopark Properties Ltd is a Tata Realty SPV with no separately reported CFO)</t>
+        </is>
+      </c>
+      <c r="T33" s="3" t="n"/>
+      <c r="U33" s="3" t="n"/>
+      <c r="V33" s="3" t="inlineStr">
+        <is>
+          <t>trilsec@tatarealty.in</t>
+        </is>
+      </c>
+      <c r="W33" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X33" s="3" t="inlineStr">
+        <is>
+          <t>Tata Realty and Infrastructure Ltd 18th Annual Report FY2024-25 lists him as CFO; LinkedIn confirms 'CFO - Tata Realty'</t>
+        </is>
+      </c>
+      <c r="Y33" s="3" t="inlineStr">
+        <is>
+          <t>Older sources list him as 'Deputy CFO' - most recent annual report and LinkedIn treated as authoritative. Infopark Properties itself does not disclose a separate CFO. Direct personal email not verified (masked on ZoomInfo); used confirmed group secretarial mailbox as fallback.</t>
+        </is>
+      </c>
+      <c r="Z33" s="4" t="inlineStr">
+        <is>
+          <t>Arushi Singhal | Company Secretary, Infopark Properties Ltd / TRIL Infopark Ltd | trilsec@tatarealty.in  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA33" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4211,16 +4275,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R34" s="4" t="n"/>
-      <c r="S34" s="4" t="n"/>
-      <c r="T34" s="4" t="n"/>
-      <c r="U34" s="4" t="n"/>
-      <c r="V34" s="4" t="n"/>
-      <c r="W34" s="4" t="n"/>
-      <c r="X34" s="4" t="n"/>
-      <c r="Y34" s="4" t="n"/>
-      <c r="Z34" s="4" t="n"/>
-      <c r="AA34" s="4" t="n"/>
+      <c r="R34" s="3" t="inlineStr">
+        <is>
+          <t>Lalit Kasliwal</t>
+        </is>
+      </c>
+      <c r="S34" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer &amp; Company Secretary (heads Finance &amp; Administration, Legal &amp; Secretarial, and IT), Tata International Ltd</t>
+        </is>
+      </c>
+      <c r="T34" s="3" t="n"/>
+      <c r="U34" s="3" t="n"/>
+      <c r="V34" s="3" t="inlineStr">
+        <is>
+          <t>cslegal.til@tatainternational.com / +91-22-6665-2200 (fax +91-22-6665-2390), VIOS Tower, Wadala, Mumbai</t>
+        </is>
+      </c>
+      <c r="W34" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X34" s="3" t="inlineStr">
+        <is>
+          <t>Official company newsroom (CFO100 2024 Roll of Honour; CFO book feature); official appointment notice PDF; LinkedIn - 4 corroborating sources</t>
+        </is>
+      </c>
+      <c r="Y34" s="3" t="inlineStr">
+        <is>
+          <t>Direct personal email not verified from an official source (masked on aggregators), left null. Used verified Company Secretarial/Legal functional mailbox as fallback.</t>
+        </is>
+      </c>
+      <c r="Z34" s="4" t="inlineStr">
+        <is>
+          <t>Md. Jamshed Alam | Company Secretary / Senior Manager - Group Secretarial Operations, Tata International Ltd | cslegal.til@tatainternational.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA34" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4286,16 +4382,53 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R35" s="4" t="n"/>
-      <c r="S35" s="4" t="n"/>
-      <c r="T35" s="4" t="n"/>
-      <c r="U35" s="4" t="n"/>
-      <c r="V35" s="4" t="n"/>
-      <c r="W35" s="4" t="n"/>
-      <c r="X35" s="4" t="n"/>
-      <c r="Y35" s="4" t="n"/>
-      <c r="Z35" s="4" t="n"/>
-      <c r="AA35" s="4" t="n"/>
+      <c r="R35" s="3" t="inlineStr">
+        <is>
+          <t>Ashok Kumar Gurnani</t>
+        </is>
+      </c>
+      <c r="S35" s="3" t="inlineStr">
+        <is>
+          <t>Company Secretary, Polyplex Corporation Limited (parent/promoter group of Kanchanjunga Power, a Polyplex Hydro SPE)</t>
+        </is>
+      </c>
+      <c r="T35" s="3" t="n"/>
+      <c r="U35" s="3" t="inlineStr">
+        <is>
+          <t>akgurnani@polyplex.com</t>
+        </is>
+      </c>
+      <c r="V35" s="3" t="inlineStr">
+        <is>
+          <t>91-120-4621300 (Polyplex Corp Noida landline, existing on file)</t>
+        </is>
+      </c>
+      <c r="W35" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X35" s="3" t="inlineStr">
+        <is>
+          <t>Existing file record cross-verified via web search (RocketReach/company filings identifying A.K. Gurnani as Polyplex Corporation Company Secretary at this same email)</t>
+        </is>
+      </c>
+      <c r="Y35" s="3" t="inlineStr">
+        <is>
+          <t>Kanchanjunga Power is a wholly-owned Polyplex hydro-power SPE with no independent finance department; run out of Polyplex Corporation's group finance/CS office. Existing on-file contact confirmed still valid.</t>
+        </is>
+      </c>
+      <c r="Z35" s="4" t="inlineStr">
+        <is>
+          <t>Manish Gupta | Group CFO, Polyplex Corporation Limited | mgupta@polyplex.com  (HIGH)
+Amit Kr. Agarwal | CFO, Polyplex Hydro Group (and Head - Family Office)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA35" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4376,16 +4509,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R36" s="4" t="n"/>
-      <c r="S36" s="4" t="n"/>
-      <c r="T36" s="4" t="n"/>
-      <c r="U36" s="4" t="n"/>
-      <c r="V36" s="4" t="n"/>
-      <c r="W36" s="4" t="n"/>
-      <c r="X36" s="4" t="n"/>
-      <c r="Y36" s="4" t="n"/>
-      <c r="Z36" s="4" t="n"/>
-      <c r="AA36" s="4" t="n"/>
+      <c r="R36" s="3" t="inlineStr">
+        <is>
+          <t>Hemant K. Jain</t>
+        </is>
+      </c>
+      <c r="S36" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, IndusInd General Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="T36" s="3" t="n"/>
+      <c r="U36" s="3" t="n"/>
+      <c r="V36" s="3" t="inlineStr">
+        <is>
+          <t>compsec@indusindinsurance.com / +91 22 4173 2000</t>
+        </is>
+      </c>
+      <c r="W36" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X36" s="3" t="inlineStr">
+        <is>
+          <t>Bloomberg Markets profile, GlobalData/Tracxn executive listing, and company management-team page - confirmed still in role after March 2025 IIHL/Hinduja acquisition and Nov 2025 rebrand from Reliance General Insurance</t>
+        </is>
+      </c>
+      <c r="Y36" s="3" t="inlineStr">
+        <is>
+          <t>IMPORTANT: existing on-file record (rgicl.compsec@relianceada.com) is STALE - company renamed from Reliance General Insurance to IndusInd General Insurance after IIHL/Hinduja acquisition via Reliance Capital insolvency (same CIN). No personal email for Hemant Jain verified, left null.</t>
+        </is>
+      </c>
+      <c r="Z36" s="4" t="inlineStr">
+        <is>
+          <t>Sushil Sojitra | Company Secretary &amp; Compliance Officer, IndusInd General Insurance Company Limited | compsec@indusindinsurance.com | +91 22 4173 2000 (Tel), +91 22 4173 2158 (Fax)  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA36" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4456,16 +4621,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R37" s="4" t="n"/>
-      <c r="S37" s="4" t="n"/>
-      <c r="T37" s="4" t="n"/>
-      <c r="U37" s="4" t="n"/>
-      <c r="V37" s="4" t="n"/>
-      <c r="W37" s="4" t="n"/>
-      <c r="X37" s="4" t="n"/>
-      <c r="Y37" s="4" t="n"/>
-      <c r="Z37" s="4" t="n"/>
-      <c r="AA37" s="4" t="n"/>
+      <c r="R37" s="3" t="inlineStr">
+        <is>
+          <t>Rohit Nayyar</t>
+        </is>
+      </c>
+      <c r="S37" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (KMP &amp; Senior Management Personnel), SMC Global Securities Ltd. - effective 1 July 2026</t>
+        </is>
+      </c>
+      <c r="T37" s="3" t="n"/>
+      <c r="U37" s="3" t="inlineStr">
+        <is>
+          <t>rohit.n@smcindiaonline.com</t>
+        </is>
+      </c>
+      <c r="V37" s="3" t="inlineStr">
+        <is>
+          <t>011-30111000 (SMC registered office landline)</t>
+        </is>
+      </c>
+      <c r="W37" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X37" s="3" t="inlineStr">
+        <is>
+          <t>SEBI Reg. 30 board disclosure summarized by TipRanks; ScanX stock-market-news; LinkedIn profile</t>
+        </is>
+      </c>
+      <c r="Y37" s="3" t="inlineStr">
+        <is>
+          <t>Prior CFO Vinod Kumar Jamar retired 30 June 2026 after ~4 decades; Rohit Nayyar took over 1 July 2026 - current CFO as of today (13 Aug 2026). Existing on-file email is a generic company inbox, not person-level.</t>
+        </is>
+      </c>
+      <c r="Z37" s="4" t="inlineStr">
+        <is>
+          <t>Suman Kumar | Company Secretary &amp; Compliance Officer, SMC Global Securities Ltd. | smcncd@smcindiaonline.com | +91-11-3011 1000, +91-11-4075 3333  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA37" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4526,16 +4727,44 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R38" s="4" t="n"/>
-      <c r="S38" s="4" t="n"/>
-      <c r="T38" s="4" t="n"/>
-      <c r="U38" s="4" t="n"/>
-      <c r="V38" s="4" t="n"/>
-      <c r="W38" s="4" t="n"/>
-      <c r="X38" s="4" t="n"/>
-      <c r="Y38" s="4" t="n"/>
-      <c r="Z38" s="4" t="n"/>
-      <c r="AA38" s="4" t="n"/>
+      <c r="R38" s="5" t="inlineStr">
+        <is>
+          <t>Bibhuti Chandan Pradhan</t>
+        </is>
+      </c>
+      <c r="S38" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Rajapushpa Properties Pvt. Ltd. (parent/group entity of Watermarke Estates, same registered office)</t>
+        </is>
+      </c>
+      <c r="T38" s="5" t="n"/>
+      <c r="U38" s="5" t="n"/>
+      <c r="V38" s="5" t="n"/>
+      <c r="W38" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X38" s="5" t="inlineStr">
+        <is>
+          <t>ZoomInfo, RocketReach org-chart/management-team listing, and LinkedIn profile</t>
+        </is>
+      </c>
+      <c r="Y38" s="5" t="inlineStr">
+        <is>
+          <t>Watermarke Estates itself has no independent finance leadership on record (MCA directors are all Parupati family promoters). Group CFO is best available finance contact as an SPV of Raja Pushpa Group. Not confirmed via official annual report/MCA KMP filing for this specific entity, hence medium.</t>
+        </is>
+      </c>
+      <c r="Z38" s="4" t="inlineStr">
+        <is>
+          <t>Alisetti Paramesh | Former CFO, Rajapushpa Properties Pvt. Ltd. - now Chief Financial Officer at Honer Homes | paramesh.a@rajapushpa.in  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA38" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4596,16 +4825,45 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R39" s="4" t="n"/>
-      <c r="S39" s="4" t="n"/>
-      <c r="T39" s="4" t="n"/>
-      <c r="U39" s="4" t="n"/>
-      <c r="V39" s="4" t="n"/>
-      <c r="W39" s="4" t="n"/>
-      <c r="X39" s="4" t="n"/>
-      <c r="Y39" s="4" t="n"/>
-      <c r="Z39" s="4" t="n"/>
-      <c r="AA39" s="4" t="n"/>
+      <c r="R39" s="3" t="inlineStr">
+        <is>
+          <t>Hari Nagrani</t>
+        </is>
+      </c>
+      <c r="S39" s="3" t="inlineStr">
+        <is>
+          <t>Executive Vice President &amp; Chief Financial Officer, Delhi International Airport Ltd.</t>
+        </is>
+      </c>
+      <c r="T39" s="3" t="n"/>
+      <c r="U39" s="3" t="n"/>
+      <c r="V39" s="3" t="n"/>
+      <c r="W39" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X39" s="3" t="inlineStr">
+        <is>
+          <t>Independently corroborated across RocketReach, ZoomInfo, EasyLeadz and Wuzzuf professional profiles</t>
+        </is>
+      </c>
+      <c r="Y39" s="3" t="inlineStr">
+        <is>
+          <t>Name/title verified via 2+ independent sources, but no email or phone could be verified - aggregator sites show only masked addresses, not reconstructed/guessed.</t>
+        </is>
+      </c>
+      <c r="Z39" s="4" t="inlineStr">
+        <is>
+          <t>Amit Jain | Group Head - Investor Relations, GMR Group (covers GMR Airports/DIAL investor communications) | jain.amit@gmrgroup.in  (MEDIUM)
+Abhishek Chawla | Unverified - existing on-file contact | Abhishek.chawla@gmrgroup.in  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA39" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4666,16 +4924,45 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R40" s="4" t="n"/>
-      <c r="S40" s="4" t="n"/>
-      <c r="T40" s="4" t="n"/>
-      <c r="U40" s="4" t="n"/>
-      <c r="V40" s="4" t="n"/>
-      <c r="W40" s="4" t="n"/>
-      <c r="X40" s="4" t="n"/>
-      <c r="Y40" s="4" t="n"/>
-      <c r="Z40" s="4" t="n"/>
-      <c r="AA40" s="4" t="n"/>
+      <c r="R40" s="3" t="inlineStr">
+        <is>
+          <t>Pankaj Rathi</t>
+        </is>
+      </c>
+      <c r="S40" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer / Head of Finance - Hyderabad operations (CapitaLand group; oversees finance for 7 entities including VITP Pvt Ltd)</t>
+        </is>
+      </c>
+      <c r="T40" s="3" t="n"/>
+      <c r="U40" s="3" t="n"/>
+      <c r="V40" s="3" t="n"/>
+      <c r="W40" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X40" s="3" t="inlineStr">
+        <is>
+          <t>MCA/ROC appointment filing (appointed CFO of VITP Private Limited 16-Apr-2025) per Zaubacorp/Tofler, corroborated by TheOrg professional org-chart profile</t>
+        </is>
+      </c>
+      <c r="Y40" s="3" t="inlineStr">
+        <is>
+          <t>Two independent, differently-sourced confirmations of the same name and finance role at the entity that owns VITP. No email/phone verified, left null.</t>
+        </is>
+      </c>
+      <c r="Z40" s="4" t="inlineStr">
+        <is>
+          <t>VVMS Rao | Unverified - existing on-file contact | vvms.rao@ascendas.com  (LOW)
+Clarisse Ong Qiu Ying | Senior Manager, Investor Relations, CapitaLand India Trust Management Pte. Ltd. (Singapore trustee-manager of VITP's parent trust) | +65 6713 3671 | enquiries@clint.com.sg | enquiries@clint.com.sg / +65 6713 3671; office main line +65 6713 2888  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA40" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4736,16 +5023,44 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R41" s="4" t="n"/>
-      <c r="S41" s="4" t="n"/>
-      <c r="T41" s="4" t="n"/>
-      <c r="U41" s="4" t="n"/>
-      <c r="V41" s="4" t="n"/>
-      <c r="W41" s="4" t="n"/>
-      <c r="X41" s="4" t="n"/>
-      <c r="Y41" s="4" t="n"/>
+      <c r="R41" s="3" t="inlineStr">
+        <is>
+          <t>Lalita Rajesh</t>
+        </is>
+      </c>
+      <c r="S41" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T41" s="3" t="n"/>
+      <c r="U41" s="3" t="n"/>
+      <c r="V41" s="3" t="inlineStr">
+        <is>
+          <t>writetous@bbtcl.com / +91-22-22197101 (also IR line +91-22-22079351-54)</t>
+        </is>
+      </c>
+      <c r="W41" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X41" s="3" t="inlineStr">
+        <is>
+          <t>BSE stock-exchange disclosure of CFO change reported via boardstewardship.com, scanx.trade and marketscreener.com (Aug 8-9, 2024 board resolution: retirement of N.H. Datanwala, appointment of Lalita Rajesh w.e.f. Aug 9, 2024)</t>
+        </is>
+      </c>
+      <c r="Y41" s="3" t="inlineStr">
+        <is>
+          <t>CA with 17+ yrs experience, with BBTC since 2019. No personal email/mobile verified from any public source. Existing on-file email bbtcl@bom2.vsnl.net.in appears stale - bbtcl.com/writetous@bbtcl.com is current per company's own contact page and recent BSE filings.</t>
+        </is>
+      </c>
       <c r="Z41" s="4" t="n"/>
-      <c r="AA41" s="4" t="n"/>
+      <c r="AA41" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4826,16 +5141,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R42" s="4" t="n"/>
-      <c r="S42" s="4" t="n"/>
-      <c r="T42" s="4" t="n"/>
-      <c r="U42" s="4" t="n"/>
-      <c r="V42" s="4" t="n"/>
-      <c r="W42" s="4" t="n"/>
-      <c r="X42" s="4" t="n"/>
-      <c r="Y42" s="4" t="n"/>
-      <c r="Z42" s="4" t="n"/>
-      <c r="AA42" s="4" t="n"/>
+      <c r="R42" s="3" t="inlineStr">
+        <is>
+          <t>Yogesh Udhoji</t>
+        </is>
+      </c>
+      <c r="S42" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T42" s="3" t="n"/>
+      <c r="U42" s="3" t="n"/>
+      <c r="V42" s="3" t="inlineStr">
+        <is>
+          <t>91-22-30941400 (registered corporate-office line, on file) / toll-free 1800 267 8811</t>
+        </is>
+      </c>
+      <c r="W42" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X42" s="3" t="inlineStr">
+        <is>
+          <t>theorg.com org chart, muthoothousing.com CFO team page, RocketReach and LinkedIn - all independently identify him as CFO since April 2023</t>
+        </is>
+      </c>
+      <c r="Y42" s="3" t="inlineStr">
+        <is>
+          <t>CA with 30+ yrs experience; ex-Asirvad Micro Finance, Aadhar Housing Finance, Tata Capital. No personal email could be verified for him specifically - did not fabricate a firstname.lastname@muthoot.com guess since the pattern itself is only single-sourced.</t>
+        </is>
+      </c>
+      <c r="Z42" s="4" t="inlineStr">
+        <is>
+          <t>S. Sumesh | Company Secretary &amp; Compliance Officer | sumesh.s@muthoot.com  (MEDIUM)
+Liza Mohanty | Grievance Redressal Officer (not finance leadership, but a real named contact channel) | 022-62728500 ext. 506 | liza.mohanty@muthoot.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA42" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4916,16 +5264,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R43" s="4" t="n"/>
-      <c r="S43" s="4" t="n"/>
-      <c r="T43" s="4" t="n"/>
-      <c r="U43" s="4" t="n"/>
-      <c r="V43" s="4" t="n"/>
-      <c r="W43" s="4" t="n"/>
-      <c r="X43" s="4" t="n"/>
-      <c r="Y43" s="4" t="n"/>
-      <c r="Z43" s="4" t="n"/>
-      <c r="AA43" s="4" t="n"/>
+      <c r="R43" s="5" t="inlineStr">
+        <is>
+          <t>Mehul Jatania</t>
+        </is>
+      </c>
+      <c r="S43" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T43" s="5" t="n"/>
+      <c r="U43" s="5" t="inlineStr">
+        <is>
+          <t>mehul.jatania@centrum.co.in</t>
+        </is>
+      </c>
+      <c r="V43" s="5" t="inlineStr">
+        <is>
+          <t>query.chfl@centrum.co.in / 91-22-42159000 (on file)</t>
+        </is>
+      </c>
+      <c r="W43" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X43" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn, ZoomInfo, RocketReach, and Equilar ExecAtlas independently identify him as CFO of Centrum Housing Finance</t>
+        </is>
+      </c>
+      <c r="Y43" s="5" t="inlineStr">
+        <is>
+          <t>Name/designation high confidence (4 sources agree). Email is an INFERRED firstname.lastname@centrum.co.in pattern based on a confirmed real address at the same company (mayank.jain@centrum.co.in) - his own email only shown masked, so exact address not independently verified; prefer on-file query.chfl@centrum.co.in for first outreach.</t>
+        </is>
+      </c>
+      <c r="Z43" s="4" t="inlineStr">
+        <is>
+          <t>Mayank Jain | AVP - Legal, Company Secretary &amp; Compliance Officer | mayank.jain@centrum.co.in  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA43" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5001,16 +5385,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R44" s="4" t="n"/>
-      <c r="S44" s="4" t="n"/>
-      <c r="T44" s="4" t="n"/>
-      <c r="U44" s="4" t="n"/>
-      <c r="V44" s="4" t="n"/>
-      <c r="W44" s="4" t="n"/>
-      <c r="X44" s="4" t="n"/>
-      <c r="Y44" s="4" t="n"/>
-      <c r="Z44" s="4" t="n"/>
-      <c r="AA44" s="4" t="n"/>
+      <c r="R44" s="3" t="inlineStr">
+        <is>
+          <t>Anshul Khemka</t>
+        </is>
+      </c>
+      <c r="S44" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO), GNRC Group</t>
+        </is>
+      </c>
+      <c r="T44" s="3" t="n"/>
+      <c r="U44" s="3" t="inlineStr">
+        <is>
+          <t>anshul.khemka@gnrchospitals.com</t>
+        </is>
+      </c>
+      <c r="V44" s="3" t="inlineStr">
+        <is>
+          <t>91-361-2227700 (company landline, on file)</t>
+        </is>
+      </c>
+      <c r="W44" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X44" s="3" t="inlineStr">
+        <is>
+          <t>Official BWR credit rating letter dated 12 Apr 2022 addressed 'To, Mr. Anshul Khemka, CFO' (hosted on GNRC Ltd's own site); email corroborated on GNRC Telehealth affiliate privacy policy</t>
+        </is>
+      </c>
+      <c r="Y44" s="3" t="inlineStr">
+        <is>
+          <t>Two independent GNRC-affiliated sources confirm name+role. Email appears under a 'Grievance Officer' listing on the affiliate site but is the same person/domain - treated as verified, not inferred.</t>
+        </is>
+      </c>
+      <c r="Z44" s="4" t="inlineStr">
+        <is>
+          <t>Biswajit Das | Company Secretary &amp; Compliance Officer (ACS 26429) | biswajitdascs@gnrchospitals.com | 91-361-2227700  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA44" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5071,16 +5491,49 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R45" s="4" t="n"/>
-      <c r="S45" s="4" t="n"/>
-      <c r="T45" s="4" t="n"/>
-      <c r="U45" s="4" t="n"/>
-      <c r="V45" s="4" t="n"/>
-      <c r="W45" s="4" t="n"/>
-      <c r="X45" s="4" t="n"/>
-      <c r="Y45" s="4" t="n"/>
-      <c r="Z45" s="4" t="n"/>
-      <c r="AA45" s="4" t="n"/>
+      <c r="R45" s="5" t="inlineStr">
+        <is>
+          <t>Akshay Kumar Chamarasa Kalyanshetti</t>
+        </is>
+      </c>
+      <c r="S45" s="5" t="inlineStr">
+        <is>
+          <t>Director &amp; Company Secretary, Shreshta Infra Projects Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="T45" s="5" t="n"/>
+      <c r="U45" s="5" t="n"/>
+      <c r="V45" s="5" t="inlineStr">
+        <is>
+          <t>control@adarshdevelopers.com (existing on-file reg email); Adarsh Developers group line +91 80 4134 3400</t>
+        </is>
+      </c>
+      <c r="W45" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X45" s="5" t="inlineStr">
+        <is>
+          <t>MCA/Zauba company records for this CIN list him as Director and Company Secretary; group contact number sourced from Adarsh Developers public listings</t>
+        </is>
+      </c>
+      <c r="Y45" s="5" t="inlineStr">
+        <is>
+          <t>Shreshta Infra Projects is an Adarsh Developers group SPV with no independent finance/IR desk found. No verified personal email/phone - no confirmed domain pattern to infer one.</t>
+        </is>
+      </c>
+      <c r="Z45" s="4" t="inlineStr">
+        <is>
+          <t>Nischay Jayeshankar | Director, Shreshta Infra Projects Pvt Ltd / Deputy Managing Director, Adarsh Group | control@adarshdevelopers.com  (MEDIUM)
+Rajashekara S | Manager - Accounts &amp; Finance, Adarsh Developers (group level) | control@adarshdevelopers.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA45" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5141,16 +5594,48 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R46" s="4" t="n"/>
-      <c r="S46" s="4" t="n"/>
-      <c r="T46" s="4" t="n"/>
-      <c r="U46" s="4" t="n"/>
-      <c r="V46" s="4" t="n"/>
-      <c r="W46" s="4" t="n"/>
-      <c r="X46" s="4" t="n"/>
-      <c r="Y46" s="4" t="n"/>
-      <c r="Z46" s="4" t="n"/>
-      <c r="AA46" s="4" t="n"/>
+      <c r="R46" s="3" t="inlineStr">
+        <is>
+          <t>Rajkumar Bansal</t>
+        </is>
+      </c>
+      <c r="S46" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO), Shivalaya Construction Ltd</t>
+        </is>
+      </c>
+      <c r="T46" s="3" t="n"/>
+      <c r="U46" s="3" t="n"/>
+      <c r="V46" s="3" t="inlineStr">
+        <is>
+          <t>compliance@sccgroup.co.in / +91 011 4508 8679 (verified Company Secretary &amp; Compliance Officer line)</t>
+        </is>
+      </c>
+      <c r="W46" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X46" s="3" t="inlineStr">
+        <is>
+          <t>Shivalaya Construction Limited's Draft Red Herring Prospectus (DRHP) filed with SEBI names Rajkumar Bansal as CFO; corroborated by LinkedIn</t>
+        </is>
+      </c>
+      <c r="Y46" s="3" t="inlineStr">
+        <is>
+          <t>CFO name/role verified via an official SEBI regulatory filing plus LinkedIn. Personal email only visible masked, left null; used verified compliance-desk contact from the same DRHP as fallback.</t>
+        </is>
+      </c>
+      <c r="Z46" s="4" t="inlineStr">
+        <is>
+          <t>Vijay Gupta | Company Secretary &amp; Compliance Officer, Shivalaya Construction Ltd | compliance@sccgroup.co.in | +91 011 4508 8679  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA46" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">

</xml_diff>

<commit_message>
enrich batch (9PM pass): rows 45-59
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -5696,16 +5696,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R47" s="4" t="n"/>
-      <c r="S47" s="4" t="n"/>
-      <c r="T47" s="4" t="n"/>
-      <c r="U47" s="4" t="n"/>
-      <c r="V47" s="4" t="n"/>
-      <c r="W47" s="4" t="n"/>
-      <c r="X47" s="4" t="n"/>
-      <c r="Y47" s="4" t="n"/>
-      <c r="Z47" s="4" t="n"/>
-      <c r="AA47" s="4" t="n"/>
+      <c r="R47" s="5" t="inlineStr">
+        <is>
+          <t>Anil Kumar Upadhaya</t>
+        </is>
+      </c>
+      <c r="S47" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T47" s="5" t="n"/>
+      <c r="U47" s="5" t="n"/>
+      <c r="V47" s="5" t="inlineStr">
+        <is>
+          <t>info@frankrosspharmacy.com / +91-33-2248-2248 (Investor Relations office, 23 R.N. Mukherjee Road, Kolkata)</t>
+        </is>
+      </c>
+      <c r="W47" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X47" s="5" t="inlineStr">
+        <is>
+          <t>ZoomInfo profile 'Anil Upadhaya - Chief Financial Officer at Frank Ross Pharmacy'; frankrosspharmacy.com/investor-relations page (via search index); 2021 annual report showed a different, earlier CFO confirming turnover since</t>
+        </is>
+      </c>
+      <c r="Y47" s="5" t="inlineStr">
+        <is>
+          <t>Single-source name (ZoomInfo only), could not corroborate via 2024 annual report. Email shown masked, real domain confirmed but exact address unverified, left null. Existing on-file email (frmspl@cal2.vsnl.net.in) is a defunct VSNL domain - company's live domain is frankrosspharmacy.com.</t>
+        </is>
+      </c>
+      <c r="Z47" s="4" t="inlineStr">
+        <is>
+          <t>Shivani Marda | Company Secretary &amp; Compliance Officer | General company line 033-2228 6042 / 0066 / 0067; frankrosspharmacy.com  (LOW)
+Investor Relations / Share Registrar desk (RTA) | mdpldc@yahoo.com / info@mdpl.in | 033-2248 2248 / 033-2243 5029, 23 R.N. Mukherjee Road, Kolkata - 700001  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA47" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5786,16 +5819,50 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R48" s="4" t="n"/>
-      <c r="S48" s="4" t="n"/>
-      <c r="T48" s="4" t="n"/>
-      <c r="U48" s="4" t="n"/>
-      <c r="V48" s="4" t="n"/>
-      <c r="W48" s="4" t="n"/>
-      <c r="X48" s="4" t="n"/>
-      <c r="Y48" s="4" t="n"/>
-      <c r="Z48" s="4" t="n"/>
-      <c r="AA48" s="4" t="n"/>
+      <c r="R48" s="3" t="inlineStr">
+        <is>
+          <t>Sanjay Kumar Bansal</t>
+        </is>
+      </c>
+      <c r="S48" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (Finance &amp; Accounts)</t>
+        </is>
+      </c>
+      <c r="T48" s="3" t="n"/>
+      <c r="U48" s="3" t="n"/>
+      <c r="V48" s="3" t="inlineStr">
+        <is>
+          <t>investor@dilipbuildcon.co.in / +91-755-4029999 (registered office / IR desk, matches existing on-file phone)</t>
+        </is>
+      </c>
+      <c r="W48" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X48" s="3" t="inlineStr">
+        <is>
+          <t>Official BSE board-meeting outcome filing dated 30-May-2022 confirming appointment as CFO/KMP effective 31-May-2022, corroborated by Trendlyne, TheOrg, Bloomberg Markets, MarketScreener</t>
+        </is>
+      </c>
+      <c r="Y48" s="3" t="inlineStr">
+        <is>
+          <t>Confirms he is still CFO of Dilip Buildcon Ltd itself (not just the DBL Infra Assets SPV). Data brokers list an email on the .com TLD, but the company's actual verified domain is dilipbuildcon.co.in - broker-suggested address is suspect, NOT used.</t>
+        </is>
+      </c>
+      <c r="Z48" s="4" t="inlineStr">
+        <is>
+          <t>Abhishek Shrivastava | Head - Company Secretary | +91-755-4029999 | investor@dilipbuildcon.co.in  (MEDIUM)
+Gautam Jain | Head of Investor Relations  (MEDIUM)
+Radhey Shyam Garg | President - Finance | investor@dilipbuildcon.co.in / +91-755-4029999  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA48" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5881,16 +5948,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R49" s="4" t="n"/>
-      <c r="S49" s="4" t="n"/>
-      <c r="T49" s="4" t="n"/>
-      <c r="U49" s="4" t="n"/>
-      <c r="V49" s="4" t="n"/>
-      <c r="W49" s="4" t="n"/>
-      <c r="X49" s="4" t="n"/>
-      <c r="Y49" s="4" t="n"/>
-      <c r="Z49" s="4" t="n"/>
-      <c r="AA49" s="4" t="n"/>
+      <c r="R49" s="3" t="inlineStr">
+        <is>
+          <t>Deepak Madnani</t>
+        </is>
+      </c>
+      <c r="S49" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T49" s="3" t="n"/>
+      <c r="U49" s="3" t="inlineStr">
+        <is>
+          <t>DMadnani@wockhardt.com</t>
+        </is>
+      </c>
+      <c r="V49" s="3" t="inlineStr">
+        <is>
+          <t>investorrelations@wockhardt.com / 022-2653 4444 (matches existing on-file phone)</t>
+        </is>
+      </c>
+      <c r="W49" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X49" s="3" t="inlineStr">
+        <is>
+          <t>Email/name directly quoted in Wockhardt's official 'Stakeholders Relationship Policy' PDF, naming him the designated stakeholder contact with this exact email; appointment as CFO (effective 7-June-2022) independently reported by IndiaInfoline, HRNxt</t>
+        </is>
+      </c>
+      <c r="Y49" s="3" t="inlineStr">
+        <is>
+          <t>Verified official-document email, not inferred/guessed. Prior CFO Pramod Gupta and Manas Datta are outdated/former.</t>
+        </is>
+      </c>
+      <c r="Z49" s="4" t="inlineStr">
+        <is>
+          <t>Rashmi Dinesh Mamtura | Company Secretary &amp; Compliance Officer | RashmiM@wockhardt.com | 022-2653 4444, Wockhardt Towers, Bandra Kurla Complex, Mumbai 400051  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA49" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5971,16 +6074,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R50" s="4" t="n"/>
-      <c r="S50" s="4" t="n"/>
-      <c r="T50" s="4" t="n"/>
-      <c r="U50" s="4" t="n"/>
-      <c r="V50" s="4" t="n"/>
-      <c r="W50" s="4" t="n"/>
-      <c r="X50" s="4" t="n"/>
-      <c r="Y50" s="4" t="n"/>
-      <c r="Z50" s="4" t="n"/>
-      <c r="AA50" s="4" t="n"/>
+      <c r="R50" s="3" t="inlineStr">
+        <is>
+          <t>Nikhila Ramesh</t>
+        </is>
+      </c>
+      <c r="S50" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T50" s="3" t="n"/>
+      <c r="U50" s="3" t="n"/>
+      <c r="V50" s="3" t="inlineStr">
+        <is>
+          <t>cg.ird@swelectes.com / 91-44-24993266</t>
+        </is>
+      </c>
+      <c r="W50" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X50" s="3" t="inlineStr">
+        <is>
+          <t>BSE Regulation-30 disclosure 'Appointment of Chief Financial Officer' (12-Nov-2020), corroborated by Bloomberg Markets profile, MarketScreener insider profile, and LinkedIn</t>
+        </is>
+      </c>
+      <c r="Y50" s="3" t="inlineStr">
+        <is>
+          <t>Direct personal email/mobile not verifiable - ZoomInfo shows only a masked address; NOT used. Used the company's verified investor-grievance email/landline as fallback.</t>
+        </is>
+      </c>
+      <c r="Z50" s="4" t="inlineStr">
+        <is>
+          <t>J. Bhuvaneswari | Company Secretary &amp; Compliance Officer (current, since 28-Aug-2024) | company.secy@swelectes.com | cg.ird@swelectes.com / 91-44-24993266  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA50" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6051,16 +6186,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R51" s="4" t="n"/>
-      <c r="S51" s="4" t="n"/>
-      <c r="T51" s="4" t="n"/>
-      <c r="U51" s="4" t="n"/>
-      <c r="V51" s="4" t="n"/>
-      <c r="W51" s="4" t="n"/>
-      <c r="X51" s="4" t="n"/>
-      <c r="Y51" s="4" t="n"/>
-      <c r="Z51" s="4" t="n"/>
-      <c r="AA51" s="4" t="n"/>
+      <c r="R51" s="3" t="inlineStr">
+        <is>
+          <t>Venkatesh Ramachandran</t>
+        </is>
+      </c>
+      <c r="S51" s="3" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer (effective 18-May-2026)</t>
+        </is>
+      </c>
+      <c r="T51" s="3" t="n"/>
+      <c r="U51" s="3" t="n"/>
+      <c r="V51" s="3" t="inlineStr">
+        <is>
+          <t>+91 40 2311 9049 (Zaggle registered office / KMP contact line, Hyderabad)</t>
+        </is>
+      </c>
+      <c r="W51" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X51" s="3" t="inlineStr">
+        <is>
+          <t>Board-approved appointment (13-May-2026) reported via TradingView/Reuters, medianews4u, mediabrief, adgully, passionateinmarketing, scanx.trade; succeeds interim CFO Rajesh Tummalaganti</t>
+        </is>
+      </c>
+      <c r="Y51" s="3" t="inlineStr">
+        <is>
+          <t>Personal email/mobile not verifiable. Zaggle's KMP-contact filing shows inconsistent email conventions across KMPs, so a firstname.lastname@zaggle.in guess was NOT made. Registered-office number used as real fallback only.</t>
+        </is>
+      </c>
+      <c r="Z51" s="4" t="inlineStr">
+        <is>
+          <t>Rajesh Tummalaganti | Deputy Chief Financial Officer (was Interim CFO Apr-May 2026) | +91 40 2311 9049  (HIGH)
+Haripriya Singh | Company Secretary &amp; Compliance Officer (NOT finance leadership - verified) | haripriya.singh@zaggle.in | +91 40 2311 9049  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA51" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6141,16 +6309,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R52" s="4" t="n"/>
-      <c r="S52" s="4" t="n"/>
-      <c r="T52" s="4" t="n"/>
-      <c r="U52" s="4" t="n"/>
-      <c r="V52" s="4" t="n"/>
-      <c r="W52" s="4" t="n"/>
-      <c r="X52" s="4" t="n"/>
-      <c r="Y52" s="4" t="n"/>
-      <c r="Z52" s="4" t="n"/>
-      <c r="AA52" s="4" t="n"/>
+      <c r="R52" s="5" t="inlineStr">
+        <is>
+          <t>Rambabu Harinath Yadav</t>
+        </is>
+      </c>
+      <c r="S52" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (appointed 27-Oct-2025)</t>
+        </is>
+      </c>
+      <c r="T52" s="5" t="n"/>
+      <c r="U52" s="5" t="n"/>
+      <c r="V52" s="5" t="inlineStr">
+        <is>
+          <t>dipti@ochfl.com / 91-22-44554877</t>
+        </is>
+      </c>
+      <c r="W52" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X52" s="5" t="inlineStr">
+        <is>
+          <t>thecompanycheck.com company profile - appears consistently across repeat searches but traces to a single aggregator source, not independently corroborated by a second outlet</t>
+        </is>
+      </c>
+      <c r="Y52" s="5" t="inlineStr">
+        <is>
+          <t>Source page's CIN suffix reads 'PLC130664' while company on file uses 'PTC130664' - mismatch could not be reconciled, capped at medium. No personal email/mobile found; used existing verified registered email/phone as fallback.</t>
+        </is>
+      </c>
+      <c r="Z52" s="4" t="inlineStr">
+        <is>
+          <t>Dipti Andhare | Assistant General Manager | dipti@ochfl.com | 91-22-44554877  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA52" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6211,16 +6411,52 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R53" s="4" t="n"/>
-      <c r="S53" s="4" t="n"/>
-      <c r="T53" s="4" t="n"/>
-      <c r="U53" s="4" t="n"/>
-      <c r="V53" s="4" t="n"/>
-      <c r="W53" s="4" t="n"/>
-      <c r="X53" s="4" t="n"/>
-      <c r="Y53" s="4" t="n"/>
-      <c r="Z53" s="4" t="n"/>
-      <c r="AA53" s="4" t="n"/>
+      <c r="R53" s="5" t="inlineStr">
+        <is>
+          <t>Niraj Kumar Gautam (Neeraj Gautam)</t>
+        </is>
+      </c>
+      <c r="S53" s="5" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer, Puravankara Ltd (parent company); listed Director, T-Hills Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="T53" s="5" t="n"/>
+      <c r="U53" s="5" t="inlineStr">
+        <is>
+          <t>neeraj.gautam@puravankara.com</t>
+        </is>
+      </c>
+      <c r="V53" s="5" t="inlineStr">
+        <is>
+          <t>bindu.d@puravankara.com (existing on-file registered email for Puravankara/T-Hills filings)</t>
+        </is>
+      </c>
+      <c r="W53" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X53" s="5" t="inlineStr">
+        <is>
+          <t>MarketScreener, RP Realty Plus, boardstewardship.com, puravankara.com/leadership/neeraj-gautam; Zauba Corp/Tofler MCA-sourced director listing for T-Hills Private Limited</t>
+        </is>
+      </c>
+      <c r="Y53" s="5" t="inlineStr">
+        <is>
+          <t>Elevated from Deputy-CFO to Group CFO effective 24-Sep-2025. Zauba Corp/Tofler director records for T-Hills list him as one of five directors, confirming he is genuinely finance-relevant for this specific SPV. Email appears on aggregator sites matching the confirmed @puravankara.com domain but not found on an official document itself - capped at medium.</t>
+        </is>
+      </c>
+      <c r="Z53" s="4" t="inlineStr">
+        <is>
+          <t>Sudip Chatterjee | Group Head - Company Secretary &amp; Compliance Officer, Puravankara Ltd; listed Director, T-Hills Pvt Ltd | puravankara.com domain (exact address masked, not independently confirmed)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA53" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6271,16 +6507,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R54" s="4" t="n"/>
-      <c r="S54" s="4" t="n"/>
-      <c r="T54" s="4" t="n"/>
-      <c r="U54" s="4" t="n"/>
-      <c r="V54" s="4" t="n"/>
-      <c r="W54" s="4" t="n"/>
-      <c r="X54" s="4" t="n"/>
-      <c r="Y54" s="4" t="n"/>
-      <c r="Z54" s="4" t="n"/>
-      <c r="AA54" s="4" t="n"/>
+      <c r="R54" s="3" t="inlineStr">
+        <is>
+          <t>Chintan Pandya (CA)</t>
+        </is>
+      </c>
+      <c r="S54" s="3" t="inlineStr">
+        <is>
+          <t>Chief Operating Officer &amp; Chief Financial Officer, MAS Rural Housing &amp; Mortgage Finance Ltd</t>
+        </is>
+      </c>
+      <c r="T54" s="3" t="n"/>
+      <c r="U54" s="3" t="n"/>
+      <c r="V54" s="3" t="inlineStr">
+        <is>
+          <t>+91-79-4110-6500 (company HQ landline, Navrangpura, Ahmedabad)</t>
+        </is>
+      </c>
+      <c r="W54" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X54" s="3" t="inlineStr">
+        <is>
+          <t>ZoomInfo, LinkedIn, RocketReach management listing; MAS Rural Housing &amp; Mortgage Finance Annual Report 2024-25</t>
+        </is>
+      </c>
+      <c r="Y54" s="3" t="inlineStr">
+        <is>
+          <t>Combined COO &amp; CFO role confirmed across multiple sources. Personal email masked on aggregators, not independently confirmed, left null; verified company landline offered as fallback.</t>
+        </is>
+      </c>
+      <c r="Z54" s="4" t="inlineStr">
+        <is>
+          <t>Darshil Hiranandani | Company Secretary, MAS Rural Housing &amp; Mortgage Finance Ltd | darshil_hiranandani@mas.co.in  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA54" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6361,16 +6629,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R55" s="4" t="n"/>
-      <c r="S55" s="4" t="n"/>
-      <c r="T55" s="4" t="n"/>
-      <c r="U55" s="4" t="n"/>
-      <c r="V55" s="4" t="n"/>
-      <c r="W55" s="4" t="n"/>
-      <c r="X55" s="4" t="n"/>
-      <c r="Y55" s="4" t="n"/>
-      <c r="Z55" s="4" t="n"/>
-      <c r="AA55" s="4" t="n"/>
+      <c r="R55" s="3" t="inlineStr">
+        <is>
+          <t>Arun Kumar Agarwal</t>
+        </is>
+      </c>
+      <c r="S55" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer &amp; Key Managerial Personnel, Prism Johnson Ltd</t>
+        </is>
+      </c>
+      <c r="T55" s="3" t="n"/>
+      <c r="U55" s="3" t="n"/>
+      <c r="V55" s="3" t="inlineStr">
+        <is>
+          <t>investor@prismjohnson.in / +91-22-66754142 (existing IR desk contact on file)</t>
+        </is>
+      </c>
+      <c r="W55" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X55" s="3" t="inlineStr">
+        <is>
+          <t>Free Press Journal, boardstewardship.com, LinkedIn, MarketScreener</t>
+        </is>
+      </c>
+      <c r="Y55" s="3" t="inlineStr">
+        <is>
+          <t>Appointed CFO &amp; KMP effective 26-Nov-2023, succeeding Manish Bhatia. No direct personal email/mobile found; using verified IR email/landline as fallback.</t>
+        </is>
+      </c>
+      <c r="Z55" s="4" t="inlineStr">
+        <is>
+          <t>Ashish Samal | Chief Investor Relations Officer, Prism Johnson Ltd - RMC (India) Division | investor@prismjohnson.in  (MEDIUM)
+Shailesh Nagindas Dholakia | Company Secretary &amp; Compliance Officer, Prism Johnson Ltd | +91-40-23400218 (registered office landline, Hyderabad; fax 23402249) | investor@prismjohnson.in  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA55" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6431,16 +6732,53 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R56" s="4" t="n"/>
-      <c r="S56" s="4" t="n"/>
-      <c r="T56" s="4" t="n"/>
-      <c r="U56" s="4" t="n"/>
-      <c r="V56" s="4" t="n"/>
-      <c r="W56" s="4" t="n"/>
-      <c r="X56" s="4" t="n"/>
-      <c r="Y56" s="4" t="n"/>
-      <c r="Z56" s="4" t="n"/>
-      <c r="AA56" s="4" t="n"/>
+      <c r="R56" s="5" t="inlineStr">
+        <is>
+          <t>Kaivan Vora</t>
+        </is>
+      </c>
+      <c r="S56" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Sadbhav Infrastructure Project Ltd. (SIPL) - the group holding/BOT-HAM company that Sadbhav Gadag Highway Pvt. Ltd. sits under</t>
+        </is>
+      </c>
+      <c r="T56" s="5" t="n"/>
+      <c r="U56" s="5" t="inlineStr">
+        <is>
+          <t>kaivan.vora@sadbhav.co.in</t>
+        </is>
+      </c>
+      <c r="V56" s="5" t="inlineStr">
+        <is>
+          <t>investor@sadbhav.co.in / +91 79-26463384 (Sadbhav Group Investor Relations)</t>
+        </is>
+      </c>
+      <c r="W56" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X56" s="5" t="inlineStr">
+        <is>
+          <t>TipRanks/scanx.trade confirming Kaivan Vora appointed CFO of SIPL effective 27-May-2026 as KMP; email is an INFERRED pattern based on the company's confirmed email format, matching the existing on-file address style</t>
+        </is>
+      </c>
+      <c r="Y56" s="5" t="inlineStr">
+        <is>
+          <t>Sadbhav Gadag Highway Pvt Ltd is an SPV with no standalone CFO; finance handled at SIPL group level. Could NOT verify that tushar.shah@sadbhav.co.in (existing on-file) is a current/finance-relevant employee - no match found, recommend internal verification. High CFO churn at both Sadbhav Engineering and SIPL in 2025-2026.</t>
+        </is>
+      </c>
+      <c r="Z56" s="4" t="inlineStr">
+        <is>
+          <t>Hitesh Chelani | Chief Financial Officer, Sadbhav Engineering Ltd. (ultimate listed parent), effective 30-May-2026 | hitesh.chelani@sadbhav.co.in | selinfo@sadbhav.co.in / +91 79-26463384  (MEDIUM)
+Kedar Pandya | Company Secretary &amp; Compliance Officer, Sadbhav Infrastructure Project Ltd. | investor@sadbhav.co.in  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA56" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6521,16 +6859,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R57" s="4" t="n"/>
-      <c r="S57" s="4" t="n"/>
-      <c r="T57" s="4" t="n"/>
-      <c r="U57" s="4" t="n"/>
-      <c r="V57" s="4" t="n"/>
-      <c r="W57" s="4" t="n"/>
-      <c r="X57" s="4" t="n"/>
-      <c r="Y57" s="4" t="n"/>
-      <c r="Z57" s="4" t="n"/>
-      <c r="AA57" s="4" t="n"/>
+      <c r="R57" s="3" t="inlineStr">
+        <is>
+          <t>Sunil Ranka</t>
+        </is>
+      </c>
+      <c r="S57" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Shree Renuka Sugars Ltd. (CFO since May 2018)</t>
+        </is>
+      </c>
+      <c r="T57" s="3" t="n"/>
+      <c r="U57" s="3" t="inlineStr">
+        <is>
+          <t>sunil.ranka@renukasugars.com</t>
+        </is>
+      </c>
+      <c r="V57" s="3" t="inlineStr">
+        <is>
+          <t>info@renukasugars.com / +91-22-2497 7744 (existing on-file company line, confirmed current)</t>
+        </is>
+      </c>
+      <c r="W57" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X57" s="3" t="inlineStr">
+        <is>
+          <t>FY2024-25 Annual Report / Directors Report confirming no change in KMP; corroborated by ZoomInfo, RocketReach, SignalHire, Bloomberg Markets, MarketScreener</t>
+        </is>
+      </c>
+      <c r="Y57" s="3" t="inlineStr">
+        <is>
+          <t>IMPORTANT: existing on-file contact iyer.dv@renukasugars.com belongs to D.V. Iyer, who resigned as CS effective 17-Jul-2015 - an 11-year-stale contact, should be replaced/flagged. Wilmar (Singapore) is majority owner post-2020; no separate Wilmar-appointed CFO found.</t>
+        </is>
+      </c>
+      <c r="Z57" s="4" t="inlineStr">
+        <is>
+          <t>Deepak Manerikar | Company Secretary &amp; Compliance Officer, Shree Renuka Sugars Ltd. (current, per Sept-2025 filing) | info@renukasugars.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA57" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6611,16 +6985,36 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R58" s="4" t="n"/>
-      <c r="S58" s="4" t="n"/>
-      <c r="T58" s="4" t="n"/>
-      <c r="U58" s="4" t="n"/>
-      <c r="V58" s="4" t="n"/>
-      <c r="W58" s="4" t="n"/>
-      <c r="X58" s="4" t="n"/>
-      <c r="Y58" s="4" t="n"/>
+      <c r="R58" s="6" t="n"/>
+      <c r="S58" s="6" t="n"/>
+      <c r="T58" s="6" t="n"/>
+      <c r="U58" s="6" t="n"/>
+      <c r="V58" s="6" t="inlineStr">
+        <is>
+          <t>inquiry@marwadionline.in / +91-281-6192000 or 7174000 (Corporate Office, Rajkot) - matches existing on-file phone</t>
+        </is>
+      </c>
+      <c r="W58" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X58" s="6" t="inlineStr">
+        <is>
+          <t>marwadionline.com/investor-relations/ page content (via search snippet, direct page fetch blocked by network egress)</t>
+        </is>
+      </c>
+      <c r="Y58" s="6" t="inlineStr">
+        <is>
+          <t>Extensive search found NO named CFO, Treasury Head, or dedicated Finance Head for Marwadi Shares &amp; Finance Ltd. Top named executives are Ketan H. Marwadi (Chairman/MD) and a CEO (sources conflict on name). An active LinkedIn job posting for 'Company Secretary' suggests that role may be currently vacant. Recommend using existing on-file registered email/phone until a named contact can be confirmed directly.</t>
+        </is>
+      </c>
       <c r="Z58" s="4" t="n"/>
-      <c r="AA58" s="4" t="n"/>
+      <c r="AA58" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6671,16 +7065,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R59" s="4" t="n"/>
-      <c r="S59" s="4" t="n"/>
-      <c r="T59" s="4" t="n"/>
-      <c r="U59" s="4" t="n"/>
-      <c r="V59" s="4" t="n"/>
-      <c r="W59" s="4" t="n"/>
-      <c r="X59" s="4" t="n"/>
-      <c r="Y59" s="4" t="n"/>
-      <c r="Z59" s="4" t="n"/>
-      <c r="AA59" s="4" t="n"/>
+      <c r="R59" s="5" t="inlineStr">
+        <is>
+          <t>Niraj Kumar Gautam (bylined in press as "Neeraj Gautam")</t>
+        </is>
+      </c>
+      <c r="S59" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Puravankara Group (also a Director of Purva Sapphire Land Pvt. Ltd.)</t>
+        </is>
+      </c>
+      <c r="T59" s="5" t="n"/>
+      <c r="U59" s="5" t="inlineStr">
+        <is>
+          <t>neeraj.gautam@puravankara.com</t>
+        </is>
+      </c>
+      <c r="V59" s="5" t="inlineStr">
+        <is>
+          <t>investors@puravankara.com / +91-80-2559-9000 (Puravankara Group registered office &amp; IR desk)</t>
+        </is>
+      </c>
+      <c r="W59" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X59" s="5" t="inlineStr">
+        <is>
+          <t>ZaubaCorp/MCA director listing for Purva Sapphire Land Pvt. Ltd. lists directors including Niraj Kumar Gautam; RPRealtyPlus/MarketScreener/HRToday news confirming elevation to Group CFO effective 24-Sep-2025</t>
+        </is>
+      </c>
+      <c r="Y59" s="5" t="inlineStr">
+        <is>
+          <t>He sits on this SPV's board AND is the Puravankara Group CFO, independently corroborating prior research. Email is aggregator-sourced, matches the same pattern as on-file ravikumar.reddy@puravankara.com contact, flagged medium rather than high.</t>
+        </is>
+      </c>
+      <c r="Z59" s="4" t="inlineStr">
+        <is>
+          <t>Sudip Chatterjee | Company Secretary &amp; Compliance Officer, Puravankara Limited | investors@puravankara.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA59" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6761,16 +7191,50 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R60" s="4" t="n"/>
-      <c r="S60" s="4" t="n"/>
-      <c r="T60" s="4" t="n"/>
-      <c r="U60" s="4" t="n"/>
-      <c r="V60" s="4" t="n"/>
-      <c r="W60" s="4" t="n"/>
-      <c r="X60" s="4" t="n"/>
-      <c r="Y60" s="4" t="n"/>
-      <c r="Z60" s="4" t="n"/>
-      <c r="AA60" s="4" t="n"/>
+      <c r="R60" s="3" t="inlineStr">
+        <is>
+          <t>Vishal Kanodia</t>
+        </is>
+      </c>
+      <c r="S60" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Shubham Housing Development Finance Company Ltd.</t>
+        </is>
+      </c>
+      <c r="T60" s="3" t="n"/>
+      <c r="U60" s="3" t="n"/>
+      <c r="V60" s="3" t="inlineStr">
+        <is>
+          <t>compliance@shubham.co / +91-124-4762545 (Compliance Dept for debenture/NCD holder queries); general board line 91-124-4212531</t>
+        </is>
+      </c>
+      <c r="W60" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X60" s="3" t="inlineStr">
+        <is>
+          <t>The Org, ZoomInfo, RocketReach, TheOfficialBoard, Bloomberg Markets profile - multiple independent sources concur</t>
+        </is>
+      </c>
+      <c r="Y60" s="3" t="inlineStr">
+        <is>
+          <t>IMPORTANT CORRECTION: existing on-file contact sanjay.chaturvedi@shubham.co is NOT the CFO - Sanjay Chaturvedi is Co-Promoter &amp; CEO. Vishal Kanodia's direct email/mobile is masked across all aggregators; no primary-source contact page reachable, so left null.</t>
+        </is>
+      </c>
+      <c r="Z60" s="4" t="inlineStr">
+        <is>
+          <t>Sanjay Chaturvedi | Co-Promoter &amp; CEO (existing on-file contact - role correction: he is CEO, not CFO) | sanjay.chaturvedi@shubham.co | 91-124-4212531  (HIGH)
+Anuj Aggarwal | Head - Finance, Accounts &amp; Tax  (MEDIUM)
+Kanika Sharma | NHB-registered Nodal Officer / Sr. Manager - Customer Service (statutory point of contact, not finance leadership) | 9818412207 | kanika.sharma1@shubham.co  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA60" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6831,16 +7295,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R61" s="4" t="n"/>
-      <c r="S61" s="4" t="n"/>
-      <c r="T61" s="4" t="n"/>
-      <c r="U61" s="4" t="n"/>
-      <c r="V61" s="4" t="n"/>
-      <c r="W61" s="4" t="n"/>
-      <c r="X61" s="4" t="n"/>
-      <c r="Y61" s="4" t="n"/>
-      <c r="Z61" s="4" t="n"/>
-      <c r="AA61" s="4" t="n"/>
+      <c r="R61" s="3" t="inlineStr">
+        <is>
+          <t>Sanjay Mehrotra (DIN 02263323)</t>
+        </is>
+      </c>
+      <c r="S61" s="3" t="inlineStr">
+        <is>
+          <t>Director (Finance), U.P. Power Corporation Ltd. (UPPCL) - holding additional charge</t>
+        </is>
+      </c>
+      <c r="T61" s="3" t="n"/>
+      <c r="U61" s="3" t="n"/>
+      <c r="V61" s="3" t="inlineStr">
+        <is>
+          <t>mduppcl12@gmail.com / +91-522-2287525 (UPPCL Head Office, Shakti Bhawan, Lucknow); companysecretary@uppcl.org</t>
+        </is>
+      </c>
+      <c r="W61" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X61" s="3" t="inlineStr">
+        <is>
+          <t>UPPCL Annual Report 2024-25 / 'List of Directors_Annexure-I' - Board Meeting No. 215 letter dated 09.09.2025 giving him additional charge of Director (Finance); DIN corroborated independently by FileSure director-profile database</t>
+        </is>
+      </c>
+      <c r="Y61" s="3" t="inlineStr">
+        <is>
+          <t>UPPCL confirmed as a distinct sister entity to UP Power Transmission Corp. Predecessor Nidhi Kumar Narang was Director (Finance) Jun-2022 to 17-Aug-2025; Sanjay Mehrotra took over on additional-charge basis Sept-2025 - may not be a permanent/sole appointment. No verified personal email/mobile found; a pattern-guessed email was excluded per no-fabrication rule. Existing on-file contact could not be tied to any current UPPCL finance role.</t>
+        </is>
+      </c>
+      <c r="Z61" s="4" t="inlineStr">
+        <is>
+          <t>Prashant Verma | Director (Commercial), UPPCL (since April 2025); previously Director (Finance) &amp; CFO at Grid Controller of India Ltd.  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA61" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">

</xml_diff>

<commit_message>
enrich batch (9PM pass): rows 60-74
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -7387,16 +7387,53 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R62" s="4" t="n"/>
-      <c r="S62" s="4" t="n"/>
-      <c r="T62" s="4" t="n"/>
-      <c r="U62" s="4" t="n"/>
-      <c r="V62" s="4" t="n"/>
-      <c r="W62" s="4" t="n"/>
-      <c r="X62" s="4" t="n"/>
-      <c r="Y62" s="4" t="n"/>
-      <c r="Z62" s="4" t="n"/>
-      <c r="AA62" s="4" t="n"/>
+      <c r="R62" s="5" t="inlineStr">
+        <is>
+          <t>Shikha Gupta</t>
+        </is>
+      </c>
+      <c r="S62" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, IFCI Factors Ltd.</t>
+        </is>
+      </c>
+      <c r="T62" s="5" t="n"/>
+      <c r="U62" s="5" t="inlineStr">
+        <is>
+          <t>shikhagupta@ifcifactors.com</t>
+        </is>
+      </c>
+      <c r="V62" s="5" t="inlineStr">
+        <is>
+          <t>011-4173 2000 (IFCI Factors registered office board line, IFCI Tower, 61 Nehru Place, New Delhi)</t>
+        </is>
+      </c>
+      <c r="W62" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X62" s="5" t="inlineStr">
+        <is>
+          <t>ifcifactors.com 'Key Managerial Personnel' page naming Shikha Gupta as CFO, CA/M.Com/JAIIB-CAIIB, heading Integrated Treasury &amp; Investment and Resources Dept</t>
+        </is>
+      </c>
+      <c r="Y62" s="5" t="inlineStr">
+        <is>
+          <t>Role/identity confirmed on the company's own KMP page. Email is INFERRED from the confirmed company address pattern, NOT independently verified - medium confidence only. A conflicting single-source ZoomInfo record names a 'Manish Jain' as CFO - likely outdated, not used given it contradicts the official KMP page.</t>
+        </is>
+      </c>
+      <c r="Z62" s="4" t="inlineStr">
+        <is>
+          <t>Smit Kumar | Company Secretary, IFCI Factors Ltd. | smitkumar@ifcifactors.com  (HIGH)
+Prafulla Sharma | Sr. AVP &amp; Secretary to the Board (also cited as Head-HR / President in different sources) | +91-9958807392 | prafullasharma@ifcifactors.com | +91-11-46412863  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA62" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7447,16 +7484,52 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R63" s="4" t="n"/>
-      <c r="S63" s="4" t="n"/>
-      <c r="T63" s="4" t="n"/>
-      <c r="U63" s="4" t="n"/>
-      <c r="V63" s="4" t="n"/>
-      <c r="W63" s="4" t="n"/>
-      <c r="X63" s="4" t="n"/>
-      <c r="Y63" s="4" t="n"/>
-      <c r="Z63" s="4" t="n"/>
-      <c r="AA63" s="4" t="n"/>
+      <c r="R63" s="5" t="inlineStr">
+        <is>
+          <t>Niraj Kumar Gautam (also styled Neeraj Gautam)</t>
+        </is>
+      </c>
+      <c r="S63" s="5" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer, Puravankara Ltd. (parent of Varishtha Property Developers Pvt. Ltd., a wholly-owned SPV)</t>
+        </is>
+      </c>
+      <c r="T63" s="5" t="n"/>
+      <c r="U63" s="5" t="inlineStr">
+        <is>
+          <t>neeraj.gautam@puravankara.com</t>
+        </is>
+      </c>
+      <c r="V63" s="5" t="inlineStr">
+        <is>
+          <t>+91-80-4343 9794</t>
+        </is>
+      </c>
+      <c r="W63" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X63" s="5" t="inlineStr">
+        <is>
+          <t>puravankara.com/leadership/neeraj-gautam; MarketScreener, boardstewardship.com and rprealtyplus.com news coverage of Sept 2025 CFO appointment; email/phone via RocketReach aggregator</t>
+        </is>
+      </c>
+      <c r="Y63" s="5" t="inlineStr">
+        <is>
+          <t>Varishtha Property Developers is a Puravankara Group SPV with no separate finance leadership found. Deepak Rastogi resigned as Group CFO effective 23-Sep-2025; Niraj Kumar Gautam elevated effective 24-Sep-2025, formally approved 07-Nov-2025 - current CFO as of Aug 2026. Email/phone come only from an aggregator listing, pegged to medium confidence.</t>
+        </is>
+      </c>
+      <c r="Z63" s="4" t="inlineStr">
+        <is>
+          <t>Sudip Chatterjee | Company Secretary &amp; Compliance Officer, Puravankara Ltd.  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA63" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7532,16 +7605,48 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R64" s="4" t="n"/>
-      <c r="S64" s="4" t="n"/>
-      <c r="T64" s="4" t="n"/>
-      <c r="U64" s="4" t="n"/>
-      <c r="V64" s="4" t="n"/>
-      <c r="W64" s="4" t="n"/>
-      <c r="X64" s="4" t="n"/>
-      <c r="Y64" s="4" t="n"/>
-      <c r="Z64" s="4" t="n"/>
-      <c r="AA64" s="4" t="n"/>
+      <c r="R64" s="5" t="inlineStr">
+        <is>
+          <t>Vishal Anand</t>
+        </is>
+      </c>
+      <c r="S64" s="5" t="inlineStr">
+        <is>
+          <t>Chief Finance Officer, TVS Emerald Ltd. / Emerald Haven Realty Ltd.</t>
+        </is>
+      </c>
+      <c r="T64" s="5" t="n"/>
+      <c r="U64" s="5" t="n"/>
+      <c r="V64" s="5" t="inlineStr">
+        <is>
+          <t>contactus@tvsemerald.com / +91 80621 95010 (general company contact line, Chennai)</t>
+        </is>
+      </c>
+      <c r="W64" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X64" s="5" t="inlineStr">
+        <is>
+          <t>tvsemerald.com/staff-view/vishal-anand (company staff bio page); ZoomInfo and RocketReach profiles listing him as CFO</t>
+        </is>
+      </c>
+      <c r="Y64" s="5" t="inlineStr">
+        <is>
+          <t>TVS Emerald Ltd was formerly named Emerald Haven Realty Ltd (same CIN) - part of TVS Group's real estate arm. Direct email/phone could not be independently verified (masked on ZoomInfo), left blank; use verified general contact as fallback.</t>
+        </is>
+      </c>
+      <c r="Z64" s="4" t="inlineStr">
+        <is>
+          <t>Roshni K Sheth | Company Secretary, TVS Emerald / Emerald Haven Realty group entities | corpsec@tvsemerald.com  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA64" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7622,16 +7727,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R65" s="4" t="n"/>
-      <c r="S65" s="4" t="n"/>
-      <c r="T65" s="4" t="n"/>
-      <c r="U65" s="4" t="n"/>
-      <c r="V65" s="4" t="n"/>
-      <c r="W65" s="4" t="n"/>
-      <c r="X65" s="4" t="n"/>
-      <c r="Y65" s="4" t="n"/>
-      <c r="Z65" s="4" t="n"/>
-      <c r="AA65" s="4" t="n"/>
+      <c r="R65" s="3" t="inlineStr">
+        <is>
+          <t>Parv Jain</t>
+        </is>
+      </c>
+      <c r="S65" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T65" s="3" t="n"/>
+      <c r="U65" s="3" t="n"/>
+      <c r="V65" s="3" t="inlineStr">
+        <is>
+          <t>info@magnumventures.in / +91-11-42420015 (company corporate office, New Delhi)</t>
+        </is>
+      </c>
+      <c r="W65" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X65" s="3" t="inlineStr">
+        <is>
+          <t>Magnum Ventures Ltd. official website management-team page; corroborated by Bloomberg Markets profile and MarketScreener insider record</t>
+        </is>
+      </c>
+      <c r="Y65" s="3" t="inlineStr">
+        <is>
+          <t>CFO since Sep 2016 (joined co. 2010). No verified direct personal email or mobile found. Delhi corporate-office landline found here differs from the Noida-area number already on file; both may be valid (different offices/lines).</t>
+        </is>
+      </c>
+      <c r="Z65" s="4" t="inlineStr">
+        <is>
+          <t>Aaina Gupta | Company Secretary &amp; Compliance Officer | 7042593791 | cs_mvl@cissahibabad.in | info@magnumventures.in  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA65" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7692,16 +7829,40 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R66" s="4" t="n"/>
-      <c r="S66" s="4" t="n"/>
-      <c r="T66" s="4" t="n"/>
-      <c r="U66" s="4" t="n"/>
-      <c r="V66" s="4" t="n"/>
-      <c r="W66" s="4" t="n"/>
-      <c r="X66" s="4" t="n"/>
-      <c r="Y66" s="4" t="n"/>
-      <c r="Z66" s="4" t="n"/>
-      <c r="AA66" s="4" t="n"/>
+      <c r="R66" s="6" t="n"/>
+      <c r="S66" s="6" t="n"/>
+      <c r="T66" s="6" t="n"/>
+      <c r="U66" s="6" t="n"/>
+      <c r="V66" s="6" t="inlineStr">
+        <is>
+          <t>lumbinieducationpvtltd@gmail.com (registered email on file)</t>
+        </is>
+      </c>
+      <c r="W66" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X66" s="6" t="inlineStr">
+        <is>
+          <t>MCA-sourced director records via Tofler, Tracxn and TheCompanyCheck company profiles for CIN U85500RJ2023PTC086224</t>
+        </is>
+      </c>
+      <c r="Y66" s="6" t="inlineStr">
+        <is>
+          <t>Very small entity (incorporated Mar 2023, Jaipur; paid-up capital ~1 lakh) functioning as an SPV-like structure for education-linked NCDs. Only two directors on record - Sushil Kumar Agarwal and Jayant Kumar Agarwal - and no separate CFO/Head-Finance title found. A well-known same-named finance professional (ex-Aavas Financiers) surfaced but could NOT be confirmed as the same individual - not conflated. No verified personal phone/email for either director found.</t>
+        </is>
+      </c>
+      <c r="Z66" s="4" t="inlineStr">
+        <is>
+          <t>Jayant Kumar Agarwal | Director (Promoter) | lumbinieducationpvtltd@gmail.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA66" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7782,16 +7943,44 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R67" s="4" t="n"/>
-      <c r="S67" s="4" t="n"/>
-      <c r="T67" s="4" t="n"/>
-      <c r="U67" s="4" t="n"/>
-      <c r="V67" s="4" t="n"/>
-      <c r="W67" s="4" t="n"/>
-      <c r="X67" s="4" t="n"/>
-      <c r="Y67" s="4" t="n"/>
+      <c r="R67" s="3" t="inlineStr">
+        <is>
+          <t>Santosh Agarwal</t>
+        </is>
+      </c>
+      <c r="S67" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer &amp; Executive Director</t>
+        </is>
+      </c>
+      <c r="T67" s="3" t="n"/>
+      <c r="U67" s="3" t="n"/>
+      <c r="V67" s="3" t="inlineStr">
+        <is>
+          <t>info@alphacorp.in / 91-124-4831111 (company registered contact on file)</t>
+        </is>
+      </c>
+      <c r="W67" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X67" s="3" t="inlineStr">
+        <is>
+          <t>Alpha Corp official website leadership page; LinkedIn; TheOrg org chart; GRI Institute member profile; company's own Facebook posts naming him CFO &amp; Executive Director</t>
+        </is>
+      </c>
+      <c r="Y67" s="3" t="inlineStr">
+        <is>
+          <t>CA with 20+ years' experience, CFO since 2014 - corroborated by 4+ independent sources. Personal email/mobile could not be verified from a primary source, left blank per no-fabrication rule.</t>
+        </is>
+      </c>
       <c r="Z67" s="4" t="n"/>
-      <c r="AA67" s="4" t="n"/>
+      <c r="AA67" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7872,16 +8061,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R68" s="4" t="n"/>
-      <c r="S68" s="4" t="n"/>
-      <c r="T68" s="4" t="n"/>
-      <c r="U68" s="4" t="n"/>
-      <c r="V68" s="4" t="n"/>
-      <c r="W68" s="4" t="n"/>
-      <c r="X68" s="4" t="n"/>
-      <c r="Y68" s="4" t="n"/>
-      <c r="Z68" s="4" t="n"/>
-      <c r="AA68" s="4" t="n"/>
+      <c r="R68" s="5" t="inlineStr">
+        <is>
+          <t>Sachin Sharma</t>
+        </is>
+      </c>
+      <c r="S68" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Satin Housing Finance Limited</t>
+        </is>
+      </c>
+      <c r="T68" s="5" t="n"/>
+      <c r="U68" s="5" t="inlineStr">
+        <is>
+          <t>sachin.sharma@satinhousingfinance.com</t>
+        </is>
+      </c>
+      <c r="V68" s="5" t="inlineStr">
+        <is>
+          <t>91-124-4346200</t>
+        </is>
+      </c>
+      <c r="W68" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X68" s="5" t="inlineStr">
+        <is>
+          <t>ZoomInfo profile + TheOfficialBoard bio; LinkedIn profile lists him at Satin Housing Finance</t>
+        </is>
+      </c>
+      <c r="Y68" s="5" t="inlineStr">
+        <is>
+          <t>Name/designation confirmed as CFO via 2 independent sources plus matching LinkedIn. Email is an INFERRED guess following the confirmed firstname.lastname pattern from the on-file address - not verified, treat as medium confidence only.</t>
+        </is>
+      </c>
+      <c r="Z68" s="4" t="inlineStr">
+        <is>
+          <t>Kuldeep Singh Yadav | Former Director / former Company Secretary (Satin group entities) - likely outdated contact | kuldeep.yadav@satinhousingfinance.com | 91-124-4346200  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA68" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7957,16 +8182,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R69" s="4" t="n"/>
-      <c r="S69" s="4" t="n"/>
-      <c r="T69" s="4" t="n"/>
-      <c r="U69" s="4" t="n"/>
-      <c r="V69" s="4" t="n"/>
-      <c r="W69" s="4" t="n"/>
-      <c r="X69" s="4" t="n"/>
-      <c r="Y69" s="4" t="n"/>
-      <c r="Z69" s="4" t="n"/>
-      <c r="AA69" s="4" t="n"/>
+      <c r="R69" s="5" t="inlineStr">
+        <is>
+          <t>Rajat Mehra</t>
+        </is>
+      </c>
+      <c r="S69" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, SAMHI Hotels Limited (parent); also Director of SAMHI Hotels (Ahmedabad) Private Limited (this SPV)</t>
+        </is>
+      </c>
+      <c r="T69" s="5" t="n"/>
+      <c r="U69" s="5" t="inlineStr">
+        <is>
+          <t>rajat.mehra@samhi.co.in</t>
+        </is>
+      </c>
+      <c r="V69" s="5" t="inlineStr">
+        <is>
+          <t>91-124-4910100</t>
+        </is>
+      </c>
+      <c r="W69" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X69" s="5" t="inlineStr">
+        <is>
+          <t>ZoomInfo, RocketReach, TheOrg, Bloomberg, Crunchbase, LinkedIn all identify him as CFO of SAMHI Hotels; Tofler company-filing data for this SPV lists him as Director/authorized signatory</t>
+        </is>
+      </c>
+      <c r="Y69" s="5" t="inlineStr">
+        <is>
+          <t>5+ sources agree on parent-company CFO role, and registry data confirms he is also director/signatory of this specific SPV. Email is INFERRED from the confirmed firstname.lastname@samhi.co.in domain pattern - not independently verified, capped at medium.</t>
+        </is>
+      </c>
+      <c r="Z69" s="4" t="inlineStr">
+        <is>
+          <t>Sanjay Jain | Senior Director - Corporate Affairs, Company Secretary &amp; Compliance Officer, SAMHI Hotels Limited | sanjay.jain@samhi.co.in | 91-124-4910100  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA69" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8047,16 +8308,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R70" s="4" t="n"/>
-      <c r="S70" s="4" t="n"/>
-      <c r="T70" s="4" t="n"/>
-      <c r="U70" s="4" t="n"/>
-      <c r="V70" s="4" t="n"/>
-      <c r="W70" s="4" t="n"/>
-      <c r="X70" s="4" t="n"/>
-      <c r="Y70" s="4" t="n"/>
-      <c r="Z70" s="4" t="n"/>
-      <c r="AA70" s="4" t="n"/>
+      <c r="R70" s="3" t="inlineStr">
+        <is>
+          <t>Ashish Vinay Deshpande</t>
+        </is>
+      </c>
+      <c r="S70" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, GMR Warora Energy Limited</t>
+        </is>
+      </c>
+      <c r="T70" s="3" t="n"/>
+      <c r="U70" s="3" t="n"/>
+      <c r="V70" s="3" t="inlineStr">
+        <is>
+          <t>energy-secretarial@gmrgroup.in / 91-22-40404500</t>
+        </is>
+      </c>
+      <c r="W70" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X70" s="3" t="inlineStr">
+        <is>
+          <t>GMR Warora Energy Limited Annual Report FY2023-24 corporate-information section; corroborated via Zaubacorp/Tofler/IndiaFilings</t>
+        </is>
+      </c>
+      <c r="Y70" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed via the company's own FY2023-24 annual report. No personal email or mobile found or verified anywhere. GMR's email convention for this entity is functional/departmental, not firstname.lastname, so no personal email inferred.</t>
+        </is>
+      </c>
+      <c r="Z70" s="4" t="inlineStr">
+        <is>
+          <t>Sanjay Kumar Babu | Company Secretary, GMR Warora Energy Limited (FCS 8649) | energy-secretarial@gmrgroup.in / 91-22-40404500  (MEDIUM)
+Suresh Bagrodia | Group Chief Financial Officer, GMR Power and Urban Infra Limited (GWEL's listed holding company) | GPUIL.CS@gmrgroup.in  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA70" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8137,16 +8431,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R71" s="4" t="n"/>
-      <c r="S71" s="4" t="n"/>
-      <c r="T71" s="4" t="n"/>
-      <c r="U71" s="4" t="n"/>
-      <c r="V71" s="4" t="n"/>
-      <c r="W71" s="4" t="n"/>
-      <c r="X71" s="4" t="n"/>
-      <c r="Y71" s="4" t="n"/>
-      <c r="Z71" s="4" t="n"/>
-      <c r="AA71" s="4" t="n"/>
+      <c r="R71" s="3" t="inlineStr">
+        <is>
+          <t>Jugeshinder "Robbie" Singh</t>
+        </is>
+      </c>
+      <c r="S71" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO), Adani Enterprises Ltd</t>
+        </is>
+      </c>
+      <c r="T71" s="3" t="n"/>
+      <c r="U71" s="3" t="n"/>
+      <c r="V71" s="3" t="inlineStr">
+        <is>
+          <t>investor.ael@adani.com / +91-79-26565555 (registered office)</t>
+        </is>
+      </c>
+      <c r="W71" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X71" s="3" t="inlineStr">
+        <is>
+          <t>Adani Enterprises Integrated Annual Report 2024-25 (KMP disclosure); adanienterprises.com/investors KMP page; multiple news sources confirming role since 2019</t>
+        </is>
+      </c>
+      <c r="Y71" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed as CFO of Adani Enterprises Ltd specifically per FY24-25 annual report KMP list. No direct personal email/phone publicly available; used verified official IR desk contact as fallback.</t>
+        </is>
+      </c>
+      <c r="Z71" s="4" t="inlineStr">
+        <is>
+          <t>Jatin Jalundhwala | Company Secretary &amp; Joint President (Legal) | jatin.jalundhwala@adani.in | 91-79-25555286  (HIGH)
+Manan Vakharia | Head of Finance / Investor Relations | mananj.vakharia@adani.com | +91-79-25556140  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA71" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8227,16 +8554,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R72" s="4" t="n"/>
-      <c r="S72" s="4" t="n"/>
-      <c r="T72" s="4" t="n"/>
-      <c r="U72" s="4" t="n"/>
-      <c r="V72" s="4" t="n"/>
-      <c r="W72" s="4" t="n"/>
-      <c r="X72" s="4" t="n"/>
-      <c r="Y72" s="4" t="n"/>
-      <c r="Z72" s="4" t="n"/>
-      <c r="AA72" s="4" t="n"/>
+      <c r="R72" s="5" t="inlineStr">
+        <is>
+          <t>CA R R Jhunjhunwala</t>
+        </is>
+      </c>
+      <c r="S72" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO), Corrtech International Ltd</t>
+        </is>
+      </c>
+      <c r="T72" s="5" t="n"/>
+      <c r="U72" s="5" t="n"/>
+      <c r="V72" s="5" t="inlineStr">
+        <is>
+          <t>compliance@corrtech.in / +91-79-26313138 (registered office / compliance desk)</t>
+        </is>
+      </c>
+      <c r="W72" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X72" s="5" t="inlineStr">
+        <is>
+          <t>Multiple LinkedIn posts (CXO Tech Bot, CEO Review Magazine India, BharatCXO, CXO Chapter) announcing the appointment around early August 2026</t>
+        </is>
+      </c>
+      <c r="Y72" s="5" t="inlineStr">
+        <is>
+          <t>Very recent appointment (~Aug 6, 2026). All corroborating sources appear to stem from one underlying announcement, capped at medium; no official BSE/NSE filing located. No personal email/phone found. Other CFO filings found (Ramesh Goel, Sandhya Gulhane) could not be confirmed as this specific company - excluded to avoid misattribution.</t>
+        </is>
+      </c>
+      <c r="Z72" s="4" t="inlineStr">
+        <is>
+          <t>Anita Chellani | Compliance Officer, Corrtech International | anita.chellani@corrtech.in  (MEDIUM)
+General Compliance / Registered Office Desk | compliance@corrtech.in | 079-26313138  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA72" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8297,16 +8657,53 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R73" s="4" t="n"/>
-      <c r="S73" s="4" t="n"/>
-      <c r="T73" s="4" t="n"/>
-      <c r="U73" s="4" t="n"/>
-      <c r="V73" s="4" t="n"/>
-      <c r="W73" s="4" t="n"/>
-      <c r="X73" s="4" t="n"/>
-      <c r="Y73" s="4" t="n"/>
-      <c r="Z73" s="4" t="n"/>
-      <c r="AA73" s="4" t="n"/>
+      <c r="R73" s="5" t="inlineStr">
+        <is>
+          <t>Rahul Shashikant Ganu</t>
+        </is>
+      </c>
+      <c r="S73" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO), Belrise Industries Ltd</t>
+        </is>
+      </c>
+      <c r="T73" s="5" t="n"/>
+      <c r="U73" s="5" t="inlineStr">
+        <is>
+          <t>rsganu@belriseindustries.com</t>
+        </is>
+      </c>
+      <c r="V73" s="5" t="inlineStr">
+        <is>
+          <t>+91 (240) 2555186 / 2555187 (corporate office landline)</t>
+        </is>
+      </c>
+      <c r="W73" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X73" s="5" t="inlineStr">
+        <is>
+          <t>Bloomberg Markets profile; LinkedIn; Belrise BSE Reg 30(5) intimation dated May 28, 2025; ZoomInfo/Datanyze listings</t>
+        </is>
+      </c>
+      <c r="Y73" s="5" t="inlineStr">
+        <is>
+          <t>Identity/role confirmed by Bloomberg + LinkedIn + official BSE filing (high confidence). Email only appears in secondary aggregator sources consistent with the pattern, treat as medium-confidence until verified. Company recently IPO'd (May 2025) as rebrand of Badve Engineering/Autoline-linked entity - existing on-file email is a stale legacy address.</t>
+        </is>
+      </c>
+      <c r="Z73" s="4" t="inlineStr">
+        <is>
+          <t>Siddhesh Mandke | Company Secretary &amp; Compliance Officer (KMP) and Head of Legal | +91 0240 2555186/87  (HIGH)
+Manish Kumar | Former Company Secretary &amp; Compliance Officer | complianceofficer@belriseindustries.com | +91 (240) 2551206  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA73" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8387,16 +8784,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R74" s="4" t="n"/>
-      <c r="S74" s="4" t="n"/>
-      <c r="T74" s="4" t="n"/>
-      <c r="U74" s="4" t="n"/>
-      <c r="V74" s="4" t="n"/>
-      <c r="W74" s="4" t="n"/>
-      <c r="X74" s="4" t="n"/>
-      <c r="Y74" s="4" t="n"/>
-      <c r="Z74" s="4" t="n"/>
-      <c r="AA74" s="4" t="n"/>
+      <c r="R74" s="3" t="inlineStr">
+        <is>
+          <t>Gourav Munjal</t>
+        </is>
+      </c>
+      <c r="S74" s="3" t="inlineStr">
+        <is>
+          <t>Whole-Time Director &amp; Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T74" s="3" t="n"/>
+      <c r="U74" s="3" t="n"/>
+      <c r="V74" s="3" t="inlineStr">
+        <is>
+          <t>csteam@5paisa.com</t>
+        </is>
+      </c>
+      <c r="W74" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X74" s="3" t="inlineStr">
+        <is>
+          <t>Bloomberg Markets profile, ZoomInfo, MarketScreener India, TheOrg org-chart, and 5paisa's own 'Names and Contact Details of KMPs' disclosure page plus BSE filings signed by him</t>
+        </is>
+      </c>
+      <c r="Y74" s="3" t="inlineStr">
+        <is>
+          <t>Identity/role (CA/CS, ~13 yrs finance/treasury experience) confirmed by 4+ sources. Direct personal email is masked on aggregators, left null. csteam@5paisa.com is the company's own listed KMP/CS contact channel (existing on file) - safest verified fallback.</t>
+        </is>
+      </c>
+      <c r="Z74" s="4" t="inlineStr">
+        <is>
+          <t>Investor Relations desk | ir@5paisa.com | +91 89766 89766 (general corporate) / registered office: IIFL House, Thane  (MEDIUM)
+Registrar &amp; Share Transfer Agent (MUFG Intime India) - shareholder/investor queries | investor.helpdesk@in.mpms.mufg.com | 022-49186000  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA74" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8457,16 +8887,52 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R75" s="4" t="n"/>
-      <c r="S75" s="4" t="n"/>
-      <c r="T75" s="4" t="n"/>
-      <c r="U75" s="4" t="n"/>
-      <c r="V75" s="4" t="n"/>
-      <c r="W75" s="4" t="n"/>
-      <c r="X75" s="4" t="n"/>
-      <c r="Y75" s="4" t="n"/>
-      <c r="Z75" s="4" t="n"/>
-      <c r="AA75" s="4" t="n"/>
+      <c r="R75" s="5" t="inlineStr">
+        <is>
+          <t>R. Santhosh</t>
+        </is>
+      </c>
+      <c r="S75" s="5" t="inlineStr">
+        <is>
+          <t>VP - Shared Services &amp; Company Secretary, RMZ Corp (parent/promoter group of Millennia Realtors Pvt. Ltd.)</t>
+        </is>
+      </c>
+      <c r="T75" s="5" t="n"/>
+      <c r="U75" s="5" t="inlineStr">
+        <is>
+          <t>r.santhosh@rmzcorp.com</t>
+        </is>
+      </c>
+      <c r="V75" s="5" t="inlineStr">
+        <is>
+          <t>corpsec@rmzcorp.com</t>
+        </is>
+      </c>
+      <c r="W75" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X75" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn profile 'Santhosh Raja - Sr VP &amp; Company Secretary', corroborated by aggregator email-format listings for RMZ Corp / Millennia Realtors Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="Y75" s="5" t="inlineStr">
+        <is>
+          <t>Millennia Realtors Pvt. Ltd. is a project SPV of the Menda family's RMZ Corp group. No SPV-specific CFO/finance officer found; ICRA rating rationale could not be fetched to cross-check. R. Santhosh is the named group-level CS/Shared-Services contact, best verifiable point of contact. Existing on-file email (millenia@vsnl.com) confirmed stale.</t>
+        </is>
+      </c>
+      <c r="Z75" s="4" t="inlineStr">
+        <is>
+          <t>Raj Menda, Manoj Menda, Arjunlal Menda | Directors / Promoters, Millennia Realtors Pvt. Ltd. (RMZ Corp founding family)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA75" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -8517,16 +8983,51 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R76" s="4" t="n"/>
-      <c r="S76" s="4" t="n"/>
-      <c r="T76" s="4" t="n"/>
-      <c r="U76" s="4" t="n"/>
-      <c r="V76" s="4" t="n"/>
-      <c r="W76" s="4" t="n"/>
-      <c r="X76" s="4" t="n"/>
-      <c r="Y76" s="4" t="n"/>
-      <c r="Z76" s="4" t="n"/>
-      <c r="AA76" s="4" t="n"/>
+      <c r="R76" s="5" t="inlineStr">
+        <is>
+          <t>Smt. Hem Prabha</t>
+        </is>
+      </c>
+      <c r="S76" s="5" t="inlineStr">
+        <is>
+          <t>Director (Finance) &amp; CFO, Rajasthan Rajya Vidyut Prasaran Nigam Ltd. (RVPN)</t>
+        </is>
+      </c>
+      <c r="T76" s="5" t="n"/>
+      <c r="U76" s="5" t="n"/>
+      <c r="V76" s="5" t="inlineStr">
+        <is>
+          <t>0141-2740116 (office landline)</t>
+        </is>
+      </c>
+      <c r="W76" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X76" s="5" t="inlineStr">
+        <is>
+          <t>RVPN Contact List / Diary Contact List directory (via scribd aggregation), corroborated by RocketReach RVPN management/org-chart listing</t>
+        </is>
+      </c>
+      <c r="Y76" s="5" t="inlineStr">
+        <is>
+          <t>RVPN's Director (Finance) is typically a Rajasthan state-cadre officer and the post rotates periodically. Sourced from a public contact-directory aggregation, not RVPN's own current website - could not independently re-verify as still current for 2026. Recommend phone/email confirmation before outreach. No email found for Hem Prabha.</t>
+        </is>
+      </c>
+      <c r="Z76" s="4" t="inlineStr">
+        <is>
+          <t>Sh. Alok | Chairman, RVPN | 9413311300 | cmd.rvpn@rvpn.co.in | 0141-2740118 / cmd.rvpn@gmail.com  (MEDIUM)
+Sh. Nathmal Didel | Managing Director, RVPN | 8875777470 | 0141-2741134  (MEDIUM)
+Sourabh Bhatt | Chief Accounts Officer (P&amp;F), RVPN | 9413382018 | 0141-2740018  (MEDIUM)
+Company Secretary desk, RVPN | comp.sec@rvpn.co.in | 0141-2740894 (RVPN general/board line)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA76" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-13-2100</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">

</xml_diff>

<commit_message>
enrich batch (1AM pass): rows 4,56,64,75-86
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -1188,7 +1188,7 @@
       <c r="U6" s="6" t="n"/>
       <c r="V6" s="6" t="inlineStr">
         <is>
-          <t>Registered office: Shakti Bhawan, 14 Ashok Marg, Lucknow (UPPTCL headquarters)</t>
+          <t>UPPTCL Head Office, Shakti Bhawan, 14 Ashok Marg, Lucknow — Phone: +91-522-2287874 (Accounts: 0522-2287701); Fax: 0522-2286476</t>
         </is>
       </c>
       <c r="W6" s="6" t="inlineStr">
@@ -1198,18 +1198,18 @@
       </c>
       <c r="X6" s="6" t="inlineStr">
         <is>
-          <t>upptcl.org Corporate Directory page, via search snippet - direct WebFetch to upptcl.org was blocked by network egress so could not be independently confirmed</t>
+          <t>Search aggregation of upptcl.org corporate directory pages, indiacustomercare.com, ZoomInfo listing for an Accounts Officer at UPPTCL</t>
         </is>
       </c>
       <c r="Y6" s="6" t="inlineStr">
         <is>
-          <t>UPPTCL is a UP state-government transmission utility. Extensive search did not turn up a distinctly named CFO/Director(Finance)/Finance Controller for UPPTCL specifically - most 'Director (Finance)' hits found (e.g. Nidhi Narang, Sanjay Mehrotra) belong to the separate sister entity UPPCL and must NOT be used for this row. MD Mayur Maheshwari, IAS is the best-verified named senior contact but is not a finance-specific role, so omitted from contact and left as fallback-only. Existing on-file contact (hem.kumar.agrawar@gmail.com) was not re-verified.</t>
+          <t>Could not confirm a current named CFO/Director(Finance)/GM(Finance) for UPPTCL specifically. Confirmed top leadership only: Dr. Ashish Kumar Goel IAS (Chairman), Mayur Maheshwari IAS (MD) — not finance-specific. Recommend outreach via head office number/registered email with follow-up ask for Director(Finance)/FA&amp;CAO by designation.</t>
         </is>
       </c>
       <c r="Z6" s="4" t="n"/>
       <c r="AA6" s="6" t="inlineStr">
         <is>
-          <t>2026-08-13-2100</t>
+          <t>2026-08-14-0100</t>
         </is>
       </c>
     </row>
@@ -6985,34 +6985,47 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R58" s="6" t="n"/>
-      <c r="S58" s="6" t="n"/>
-      <c r="T58" s="6" t="n"/>
-      <c r="U58" s="6" t="n"/>
-      <c r="V58" s="6" t="inlineStr">
-        <is>
-          <t>inquiry@marwadionline.in / +91-281-6192000 or 7174000 (Corporate Office, Rajkot) - matches existing on-file phone</t>
-        </is>
-      </c>
-      <c r="W58" s="6" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="X58" s="6" t="inlineStr">
-        <is>
-          <t>marwadionline.com/investor-relations/ page content (via search snippet, direct page fetch blocked by network egress)</t>
-        </is>
-      </c>
-      <c r="Y58" s="6" t="inlineStr">
-        <is>
-          <t>Extensive search found NO named CFO, Treasury Head, or dedicated Finance Head for Marwadi Shares &amp; Finance Ltd. Top named executives are Ketan H. Marwadi (Chairman/MD) and a CEO (sources conflict on name). An active LinkedIn job posting for 'Company Secretary' suggests that role may be currently vacant. Recommend using existing on-file registered email/phone until a named contact can be confirmed directly.</t>
-        </is>
-      </c>
-      <c r="Z58" s="4" t="n"/>
-      <c r="AA58" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-13-2100</t>
+      <c r="R58" s="3" t="inlineStr">
+        <is>
+          <t>Sanjay H. Thakrar</t>
+        </is>
+      </c>
+      <c r="S58" s="3" t="inlineStr">
+        <is>
+          <t>Senior VP - Accounts &amp; Finance</t>
+        </is>
+      </c>
+      <c r="T58" s="3" t="n"/>
+      <c r="U58" s="3" t="n"/>
+      <c r="V58" s="3" t="inlineStr">
+        <is>
+          <t>msfl@marwadigroup.in / inquiry@marwadionline.in; Phone: 0281-6192000 / 0281-7174000</t>
+        </is>
+      </c>
+      <c r="W58" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X58" s="3" t="inlineStr">
+        <is>
+          <t>Official company Leadership page marwadionline.com/leadership; corroborated by ZoomInfo listing (title: Senior VP, Accounts &amp; Finance at Marwadi Shares &amp; Finance)</t>
+        </is>
+      </c>
+      <c r="Y58" s="3" t="inlineStr">
+        <is>
+          <t>No 'CFO' title used by company; Thakrar is the de facto senior finance executive per official leadership page. Personal direct email/mobile not published (ZoomInfo shows masked address), left null rather than guessed.</t>
+        </is>
+      </c>
+      <c r="Z58" s="4" t="inlineStr">
+        <is>
+          <t>Mira D. Marwadi | Whole Time Director (promoter family) | msfl@marwadigroup.in; 0281-7174000  (MEDIUM)
+Company Secretary / Compliance Officer | msfl@marwadigroup.in; 0281-7174000  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA58" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
         </is>
       </c>
     </row>
@@ -7829,38 +7842,46 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R66" s="6" t="n"/>
-      <c r="S66" s="6" t="n"/>
-      <c r="T66" s="6" t="n"/>
-      <c r="U66" s="6" t="n"/>
-      <c r="V66" s="6" t="inlineStr">
-        <is>
-          <t>lumbinieducationpvtltd@gmail.com (registered email on file)</t>
-        </is>
-      </c>
-      <c r="W66" s="6" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="X66" s="6" t="inlineStr">
-        <is>
-          <t>MCA-sourced director records via Tofler, Tracxn and TheCompanyCheck company profiles for CIN U85500RJ2023PTC086224</t>
-        </is>
-      </c>
-      <c r="Y66" s="6" t="inlineStr">
-        <is>
-          <t>Very small entity (incorporated Mar 2023, Jaipur; paid-up capital ~1 lakh) functioning as an SPV-like structure for education-linked NCDs. Only two directors on record - Sushil Kumar Agarwal and Jayant Kumar Agarwal - and no separate CFO/Head-Finance title found. A well-known same-named finance professional (ex-Aavas Financiers) surfaced but could NOT be confirmed as the same individual - not conflated. No verified personal phone/email for either director found.</t>
+      <c r="R66" s="5" t="inlineStr">
+        <is>
+          <t>Sushil Kumar Agarwal</t>
+        </is>
+      </c>
+      <c r="S66" s="5" t="inlineStr">
+        <is>
+          <t>Director (small private company, no distinct CFO role; finance handled at director level)</t>
+        </is>
+      </c>
+      <c r="T66" s="5" t="n"/>
+      <c r="U66" s="5" t="n"/>
+      <c r="V66" s="5" t="inlineStr">
+        <is>
+          <t>lumbinieducationpvtltd@gmail.com / info@lumbinieducation.com; Phone: +91-8529758464</t>
+        </is>
+      </c>
+      <c r="W66" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X66" s="5" t="inlineStr">
+        <is>
+          <t>MCA-derived company/director records via Tofler, TheCompanyCheck, and search consensus (CIN U85500RJ2023PTC086224); company website lumbinieducation.com</t>
+        </is>
+      </c>
+      <c r="Y66" s="5" t="inlineStr">
+        <is>
+          <t>Company is small (Rs 1 lakh paid-up capital), recently incorporated (March 2023), only two directors, no separate finance department. DIN cross-check to other directorships couldn't be fully confirmed as same individual — flagged as inference hence medium not high.</t>
         </is>
       </c>
       <c r="Z66" s="4" t="inlineStr">
         <is>
-          <t>Jayant Kumar Agarwal | Director (Promoter) | lumbinieducationpvtltd@gmail.com  (LOW)</t>
-        </is>
-      </c>
-      <c r="AA66" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-13-2100</t>
+          <t>Jayant Agarwal (also cited as Jayant Kumar Agarwal) | Director | lumbinieducationpvtltd@gmail.com / info@lumbinieducation.com; +91-8529758464  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA66" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
         </is>
       </c>
     </row>
@@ -9088,16 +9109,40 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R77" s="4" t="n"/>
-      <c r="S77" s="4" t="n"/>
-      <c r="T77" s="4" t="n"/>
-      <c r="U77" s="4" t="n"/>
-      <c r="V77" s="4" t="n"/>
-      <c r="W77" s="4" t="n"/>
-      <c r="X77" s="4" t="n"/>
-      <c r="Y77" s="4" t="n"/>
-      <c r="Z77" s="4" t="n"/>
-      <c r="AA77" s="4" t="n"/>
+      <c r="R77" s="6" t="n"/>
+      <c r="S77" s="6" t="n"/>
+      <c r="T77" s="6" t="n"/>
+      <c r="U77" s="6" t="n"/>
+      <c r="V77" s="6" t="inlineStr">
+        <is>
+          <t>roc.efiling2014@gmail.com</t>
+        </is>
+      </c>
+      <c r="W77" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X77" s="6" t="inlineStr">
+        <is>
+          <t>MCA/ROC filing email as listed on ZaubaCorp/Tofler/IndiaFilings company profile pages for CIN U70109WB2006PTC165835</t>
+        </is>
+      </c>
+      <c r="Y77" s="6" t="inlineStr">
+        <is>
+          <t>No named CFO, Treasury head, or finance controller could be identified for this company via MCA, company website, LinkedIn, or news search. CARE Ratings' latest press release (Nov 2025) marks the company's rating as 'ISSUER NOT COOPERATING'. Fallback is the generic ROC filing email already on file, unverified as a live monitored inbox.</t>
+        </is>
+      </c>
+      <c r="Z77" s="4" t="inlineStr">
+        <is>
+          <t>Pallab Das, Sanjay Jhunjhunwala, Minu Tulsian, Prithiwiraj Mukherjee, Vinod Kejriwal, Suresh Kumar Kedia | Directors (MCA record) — finance-specific role not specified  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA77" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -9173,16 +9218,40 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R78" s="4" t="n"/>
-      <c r="S78" s="4" t="n"/>
-      <c r="T78" s="4" t="n"/>
-      <c r="U78" s="4" t="n"/>
-      <c r="V78" s="4" t="n"/>
-      <c r="W78" s="4" t="n"/>
-      <c r="X78" s="4" t="n"/>
-      <c r="Y78" s="4" t="n"/>
-      <c r="Z78" s="4" t="n"/>
-      <c r="AA78" s="4" t="n"/>
+      <c r="R78" s="6" t="n"/>
+      <c r="S78" s="6" t="n"/>
+      <c r="T78" s="6" t="n"/>
+      <c r="U78" s="6" t="n"/>
+      <c r="V78" s="6" t="inlineStr">
+        <is>
+          <t>lavishbuildmart@gmail.com</t>
+        </is>
+      </c>
+      <c r="W78" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X78" s="6" t="inlineStr">
+        <is>
+          <t>MCA/ROC registered email as listed on ZaubaCorp, Tofler, CleartTax, TheCompanyCheck for CIN U45300HR2007PTC056065</t>
+        </is>
+      </c>
+      <c r="Y78" s="6" t="inlineStr">
+        <is>
+          <t>No named CFO or finance officer found for the SPV entity itself. Confirmed Lavish Buildmart is a 100%-owned subsidiary of M3M India Private Limited (M3M Group) per CARE Ratings press release (Feb 2024). No single current named Group CFO could be confidently verified. Registered company email is the only verifiable fallback.</t>
+        </is>
+      </c>
+      <c r="Z78" s="4" t="inlineStr">
+        <is>
+          <t>Vijay Kumar Aggarwal / Anuj Kumar Tiwari | Directors (MCA record) — finance-specific role not specified  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA78" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -9263,16 +9332,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R79" s="4" t="n"/>
-      <c r="S79" s="4" t="n"/>
-      <c r="T79" s="4" t="n"/>
-      <c r="U79" s="4" t="n"/>
-      <c r="V79" s="4" t="n"/>
-      <c r="W79" s="4" t="n"/>
-      <c r="X79" s="4" t="n"/>
-      <c r="Y79" s="4" t="n"/>
-      <c r="Z79" s="4" t="n"/>
-      <c r="AA79" s="4" t="n"/>
+      <c r="R79" s="3" t="inlineStr">
+        <is>
+          <t>Amit Mor</t>
+        </is>
+      </c>
+      <c r="S79" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Prestige Group / Prestige Estates Projects Ltd.</t>
+        </is>
+      </c>
+      <c r="T79" s="3" t="n"/>
+      <c r="U79" s="3" t="n"/>
+      <c r="V79" s="3" t="inlineStr">
+        <is>
+          <t>investors@prestigeconstructions.com; +91 80 2559 1080 / 2559 1945</t>
+        </is>
+      </c>
+      <c r="W79" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X79" s="3" t="inlineStr">
+        <is>
+          <t>Official bio page prestigeconstructions.com/about-us/cfo/amit-mor; corroborated by Trendlyne (executive remuneration disclosure filed with BSE/NSE annual report), Crunchbase, and LinkedIn (in.linkedin.com/in/amit-mor-006a382a8) — 3+ independent sources agree on name, title, and tenure since June 2021</t>
+        </is>
+      </c>
+      <c r="Y79" s="3" t="inlineStr">
+        <is>
+          <t>No direct personal email or mobile number for Amit Mor is published on any public source; only the general company investor-relations email/landline is available as fallback contact route. His stated remit explicitly covers Corporate Finance, Fund Raising, and Treasury.</t>
+        </is>
+      </c>
+      <c r="Z79" s="4" t="inlineStr">
+        <is>
+          <t>Manoj Krishna J V | Company Secretary &amp; Compliance Officer | investors@prestigeconstructions.com  (HIGH)
+Investor Relations Desk | investors@prestigeconstructions.com | +91 80 2559 1080  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA79" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -9343,16 +9445,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R80" s="4" t="n"/>
-      <c r="S80" s="4" t="n"/>
-      <c r="T80" s="4" t="n"/>
-      <c r="U80" s="4" t="n"/>
-      <c r="V80" s="4" t="n"/>
-      <c r="W80" s="4" t="n"/>
-      <c r="X80" s="4" t="n"/>
-      <c r="Y80" s="4" t="n"/>
-      <c r="Z80" s="4" t="n"/>
-      <c r="AA80" s="4" t="n"/>
+      <c r="R80" s="5" t="inlineStr">
+        <is>
+          <t>Suyash Bhise</t>
+        </is>
+      </c>
+      <c r="S80" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T80" s="5" t="n"/>
+      <c r="U80" s="5" t="n"/>
+      <c r="V80" s="5" t="inlineStr">
+        <is>
+          <t>cs@marathonrealty.com / yogesh.patole@marathonrealty.com (Company Secretary desk), landline +91-22-6772 8484</t>
+        </is>
+      </c>
+      <c r="W80" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X80" s="5" t="inlineStr">
+        <is>
+          <t>CFO appointment: Marathon Nextgen Realty board meeting outcome filing dated 21-Jun-2024, corroborated by boardstewardship.com and ZoomInfo/Bloomberg profile pages. Fallback via NSE filing signed by Yogesh Ashok Patole, Company Secretary &amp; Compliance Officer</t>
+        </is>
+      </c>
+      <c r="Y80" s="5" t="inlineStr">
+        <is>
+          <t>CFO identity/appointment confirmed via official filing but no personal email/mobile found (ZoomInfo masks it, not reproduced). Fallback is CS contact, independently verified via NSE filing.</t>
+        </is>
+      </c>
+      <c r="Z80" s="4" t="inlineStr">
+        <is>
+          <t>Yogesh Ashok Patole | Company Secretary &amp; Compliance Officer | cs@marathonrealty.com | +91-22-6772 8484  (HIGH)
+Investor/Shares desk | shares@marathonnextgen.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA80" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -9433,16 +9568,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R81" s="4" t="n"/>
-      <c r="S81" s="4" t="n"/>
-      <c r="T81" s="4" t="n"/>
-      <c r="U81" s="4" t="n"/>
-      <c r="V81" s="4" t="n"/>
-      <c r="W81" s="4" t="n"/>
-      <c r="X81" s="4" t="n"/>
-      <c r="Y81" s="4" t="n"/>
-      <c r="Z81" s="4" t="n"/>
-      <c r="AA81" s="4" t="n"/>
+      <c r="R81" s="5" t="inlineStr">
+        <is>
+          <t>Rakesh Mitra</t>
+        </is>
+      </c>
+      <c r="S81" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T81" s="5" t="n"/>
+      <c r="U81" s="5" t="n"/>
+      <c r="V81" s="5" t="inlineStr">
+        <is>
+          <t>corporate@thelalit.com, landline +91-11-23411001 / +91-11-44447777</t>
+        </is>
+      </c>
+      <c r="W81" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X81" s="5" t="inlineStr">
+        <is>
+          <t>Bharat Hotels Ltd Annual Report 2023-24, corroborated by RocketReach profile and news search — Amit Gupta resigned as CFO effective 8-Nov-2023, Rakesh Mitra appointed CFO effective 7-Mar-2024 (with company since 17-May-2002)</t>
+        </is>
+      </c>
+      <c r="Y81" s="5" t="inlineStr">
+        <is>
+          <t>Name/designation corroborated by 2+ sources, but no direct personal email or mobile located. Fallback is general corporate email/landline, not independently re-confirmed as CFO's direct line.</t>
+        </is>
+      </c>
+      <c r="Z81" s="4" t="inlineStr">
+        <is>
+          <t>Himanshu Pandey | Company Secretary &amp; Head - Legal and Compliance (as of 2018 DRHP)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA81" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -9513,16 +9680,40 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R82" s="4" t="n"/>
-      <c r="S82" s="4" t="n"/>
-      <c r="T82" s="4" t="n"/>
-      <c r="U82" s="4" t="n"/>
-      <c r="V82" s="4" t="n"/>
-      <c r="W82" s="4" t="n"/>
-      <c r="X82" s="4" t="n"/>
-      <c r="Y82" s="4" t="n"/>
-      <c r="Z82" s="4" t="n"/>
-      <c r="AA82" s="4" t="n"/>
+      <c r="R82" s="6" t="n"/>
+      <c r="S82" s="6" t="n"/>
+      <c r="T82" s="6" t="n"/>
+      <c r="U82" s="6" t="n"/>
+      <c r="V82" s="6" t="inlineStr">
+        <is>
+          <t>india@asaindiaamf.com, phone 91-33-23358510 (existing registered contact, not independently re-verified); alt office number +91 (33) 2357 8508/18</t>
+        </is>
+      </c>
+      <c r="W82" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X82" s="6" t="inlineStr">
+        <is>
+          <t>Existing company registration hint; general office number from web-search summary</t>
+        </is>
+      </c>
+      <c r="Y82" s="6" t="inlineStr">
+        <is>
+          <t>No named CFO/Treasury Head/Finance Controller for the India entity could be found despite extensive searching. Parent group CFO (Geert Embrechts, Amsterdam) covers the whole group, not India specifically, so not listed as India contact. Several company sites were blocked by network egress proxy and could not be directly fetched, worth manual re-check.</t>
+        </is>
+      </c>
+      <c r="Z82" s="4" t="inlineStr">
+        <is>
+          <t>Anjan Dasgupta | Managing Director (finance &amp; banking background; oversees overall business including finance) | 8100065555 | anjan.dgupta@gmail.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA82" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -9583,16 +9774,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R83" s="4" t="n"/>
-      <c r="S83" s="4" t="n"/>
-      <c r="T83" s="4" t="n"/>
-      <c r="U83" s="4" t="n"/>
-      <c r="V83" s="4" t="n"/>
-      <c r="W83" s="4" t="n"/>
-      <c r="X83" s="4" t="n"/>
-      <c r="Y83" s="4" t="n"/>
-      <c r="Z83" s="4" t="n"/>
-      <c r="AA83" s="4" t="n"/>
+      <c r="R83" s="3" t="inlineStr">
+        <is>
+          <t>Chandrashekar S. (Chandrashekar Shriramulu)</t>
+        </is>
+      </c>
+      <c r="S83" s="3" t="inlineStr">
+        <is>
+          <t>Company Secretary, Bangalore Tower Pvt. Ltd. (Keppel Land group SPV)</t>
+        </is>
+      </c>
+      <c r="T83" s="3" t="n"/>
+      <c r="U83" s="3" t="inlineStr">
+        <is>
+          <t>chandrashekar.s@keppelland.com</t>
+        </is>
+      </c>
+      <c r="V83" s="3" t="inlineStr">
+        <is>
+          <t>+91 80 6949 555 (Keppel Real Estate India / BTPL office, The Cube, Karle Town Centre, Bengaluru)</t>
+        </is>
+      </c>
+      <c r="W83" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X83" s="3" t="inlineStr">
+        <is>
+          <t>Keppel's own Bangalore Tower/BTPL project pages list this contact email/phone; corporate-registry aggregator (thecompanycheck.com, CIN U45309KA2021PTC152825) independently names Chandrashekar Shriramulu as Company Secretary</t>
+        </is>
+      </c>
+      <c r="Y83" s="3" t="inlineStr">
+        <is>
+          <t>BTPL is a 100%-owned Keppel Land SPV (no independent CFO); Company Secretary is the closest named finance-adjacent contact found.</t>
+        </is>
+      </c>
+      <c r="Z83" s="4" t="inlineStr">
+        <is>
+          <t>Deepak T S | Senior Manager, Keppel Real Estate Division (India) - role not confirmed as finance-specific | deepak.s@keppelland.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA83" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -9643,16 +9870,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R84" s="4" t="n"/>
-      <c r="S84" s="4" t="n"/>
-      <c r="T84" s="4" t="n"/>
-      <c r="U84" s="4" t="n"/>
-      <c r="V84" s="4" t="n"/>
-      <c r="W84" s="4" t="n"/>
-      <c r="X84" s="4" t="n"/>
-      <c r="Y84" s="4" t="n"/>
-      <c r="Z84" s="4" t="n"/>
-      <c r="AA84" s="4" t="n"/>
+      <c r="R84" s="5" t="inlineStr">
+        <is>
+          <t>Chirag Parmar</t>
+        </is>
+      </c>
+      <c r="S84" s="5" t="inlineStr">
+        <is>
+          <t>Company Secretary &amp; Compliance Officer</t>
+        </is>
+      </c>
+      <c r="T84" s="5" t="n"/>
+      <c r="U84" s="5" t="n"/>
+      <c r="V84" s="5" t="inlineStr">
+        <is>
+          <t>moneymsecurities@gmail.com; phone +91 22 3304 3800 (registered office, Bandra West, Mumbai)</t>
+        </is>
+      </c>
+      <c r="W84" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X84" s="5" t="inlineStr">
+        <is>
+          <t>Company's own leadership page (moneymartspl.com/leaders.html via cached search snippets)</t>
+        </is>
+      </c>
+      <c r="Y84" s="5" t="inlineStr">
+        <is>
+          <t>Could not find personal/direct email or mobile for Chirag Parmar. Note: moneymartspl.com's contact page may indicate a lapsed/inactive domain - verify before relying on it.</t>
+        </is>
+      </c>
+      <c r="Z84" s="4" t="inlineStr">
+        <is>
+          <t>Sanjeev Gajanan Patil | Director (ex-CFO Epsilon Carbon Pvt Ltd, senior finance roles at Privi Speciality Chemicals, Asian Paints, 20th Century Finance)  (LOW)
+Gaurav Jeswani (IDBI Trusteeship Services Ltd - debenture trustee) | Debenture Trustee contact for Moneymart NCD issues | 022 4080 7000 | itsl@idbitrustee.com / response@idbitrustee.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA84" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -9728,16 +9988,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R85" s="4" t="n"/>
-      <c r="S85" s="4" t="n"/>
-      <c r="T85" s="4" t="n"/>
-      <c r="U85" s="4" t="n"/>
-      <c r="V85" s="4" t="n"/>
-      <c r="W85" s="4" t="n"/>
-      <c r="X85" s="4" t="n"/>
-      <c r="Y85" s="4" t="n"/>
-      <c r="Z85" s="4" t="n"/>
-      <c r="AA85" s="4" t="n"/>
+      <c r="R85" s="3" t="inlineStr">
+        <is>
+          <t>Ramya Bharathram</t>
+        </is>
+      </c>
+      <c r="S85" s="3" t="inlineStr">
+        <is>
+          <t>Managing Director &amp; Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T85" s="3" t="n"/>
+      <c r="U85" s="3" t="n"/>
+      <c r="V85" s="3" t="inlineStr">
+        <is>
+          <t>investorinfo@thirumalaichemicals.com; +91 44 6605 7700/7736 (Chennai corporate office, Spic House, Guindy) - note existing on-file number 91-22-24017841 appears to be an older Mumbai line, should be re-verified</t>
+        </is>
+      </c>
+      <c r="W85" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X85" s="3" t="inlineStr">
+        <is>
+          <t>Company's own Board of Directors page, Business Standard (2021 appointment article), MarketScreener, Bloomberg, LinkedIn; confirmed current via reappointment at 53rd AGM Aug 2026</t>
+        </is>
+      </c>
+      <c r="Y85" s="3" t="inlineStr">
+        <is>
+          <t>Combined MD+CFO role since March 2024 (reappointed Aug 2026). No direct/personal email found publicly (only shared IR inbox); masked company-domain email not guessed.</t>
+        </is>
+      </c>
+      <c r="Z85" s="4" t="inlineStr">
+        <is>
+          <t>K. Anand Kumar | President - Finance (Senior Management), effective 14 Feb 2026; previously Group CFO at PVP Ventures | investorinfo@thirumalaichemicals.com; +91 44 6605 7700  (HIGH)
+Aditya Sharma | Company Secretary &amp; Compliance Officer (appointed effective 18 Aug 2025, Membership No. A39666) | investorinfo@thirumalaichemicals.com | +91 44 6605 7736  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA85" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -9808,16 +10101,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R86" s="4" t="n"/>
-      <c r="S86" s="4" t="n"/>
-      <c r="T86" s="4" t="n"/>
-      <c r="U86" s="4" t="n"/>
-      <c r="V86" s="4" t="n"/>
-      <c r="W86" s="4" t="n"/>
-      <c r="X86" s="4" t="n"/>
-      <c r="Y86" s="4" t="n"/>
-      <c r="Z86" s="4" t="n"/>
-      <c r="AA86" s="4" t="n"/>
+      <c r="R86" s="3" t="inlineStr">
+        <is>
+          <t>Geena Thomas</t>
+        </is>
+      </c>
+      <c r="S86" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T86" s="3" t="n"/>
+      <c r="U86" s="3" t="n"/>
+      <c r="V86" s="3" t="inlineStr">
+        <is>
+          <t>mvfl@muthootgroup.com / +91-484-3222002 (registered corporate office, Kochi)</t>
+        </is>
+      </c>
+      <c r="W86" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X86" s="3" t="inlineStr">
+        <is>
+          <t>Muthoot Vehicle &amp; Asset Finance Limited 33rd Annual Report 2024-25 (mvafl.com) - identified via search-engine indexing; two independent search queries returned the same designation from the same official annual report</t>
+        </is>
+      </c>
+      <c r="Y86" s="3" t="inlineStr">
+        <is>
+          <t>No direct mobile or personal email found for Geena Thomas; use registered landline/general email as fallback until direct line confirmed.</t>
+        </is>
+      </c>
+      <c r="Z86" s="4" t="inlineStr">
+        <is>
+          <t>Geena Ajith | Chief Finance Manager (possibly a name variant of CFO Geena Thomas; unverified whether same individual) | 7593864403 | geenaajith@muthootgroup.com  (LOW)
+Manoj Jacob | Whole Time Director (chartered accountant, oversees governance/finance strategy)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA86" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9873,16 +10199,53 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R87" s="4" t="n"/>
-      <c r="S87" s="4" t="n"/>
-      <c r="T87" s="4" t="n"/>
-      <c r="U87" s="4" t="n"/>
-      <c r="V87" s="4" t="n"/>
-      <c r="W87" s="4" t="n"/>
-      <c r="X87" s="4" t="n"/>
-      <c r="Y87" s="4" t="n"/>
-      <c r="Z87" s="4" t="n"/>
-      <c r="AA87" s="4" t="n"/>
+      <c r="R87" s="5" t="inlineStr">
+        <is>
+          <t>Hemant Agarwal</t>
+        </is>
+      </c>
+      <c r="S87" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T87" s="5" t="n"/>
+      <c r="U87" s="5" t="inlineStr">
+        <is>
+          <t>hemant.agarwal@hectorbeverages.com</t>
+        </is>
+      </c>
+      <c r="V87" s="5" t="inlineStr">
+        <is>
+          <t>hectorbeverages.com general/registered office; paperboat@hectorbeverages.com brand contact</t>
+        </is>
+      </c>
+      <c r="W87" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X87" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn (title: CFO at Hector Beverages); TheOrg.com org chart, in role since Jan 2024 - two independent sources agree on name+designation</t>
+        </is>
+      </c>
+      <c r="Y87" s="5" t="inlineStr">
+        <is>
+          <t>Email is INFERRED from company's dominant firstname.lastname@hectorbeverages.com pattern (~57% of listed staff per LeadIQ/RocketReach), not directly confirmed. Do not treat as verified without direct confirmation. No phone number found.</t>
+        </is>
+      </c>
+      <c r="Z87" s="4" t="inlineStr">
+        <is>
+          <t>Neeraj Kakkar | Co-Founder &amp; CEO | neeraj@hectorbeverages.com  (HIGH)
+General/registered office contact | +91 18604254425 (general company phone line)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA87" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -9933,16 +10296,41 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R88" s="4" t="n"/>
-      <c r="S88" s="4" t="n"/>
-      <c r="T88" s="4" t="n"/>
-      <c r="U88" s="4" t="n"/>
-      <c r="V88" s="4" t="n"/>
-      <c r="W88" s="4" t="n"/>
-      <c r="X88" s="4" t="n"/>
-      <c r="Y88" s="4" t="n"/>
-      <c r="Z88" s="4" t="n"/>
-      <c r="AA88" s="4" t="n"/>
+      <c r="R88" s="6" t="n"/>
+      <c r="S88" s="6" t="n"/>
+      <c r="T88" s="6" t="n"/>
+      <c r="U88" s="6" t="n"/>
+      <c r="V88" s="6" t="inlineStr">
+        <is>
+          <t>rohanpn@rohanbuilders.com / +91-20-7101-7101 (registered office: 1 Modibaug, Ganeshkhind Road, Shivaji Nagar, Pune - 411016)</t>
+        </is>
+      </c>
+      <c r="W88" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X88" s="6" t="inlineStr">
+        <is>
+          <t>Zaubacorp / IndiaFilings / Corporatedir company-registry listings for CIN U45203PN2007PLC130755; Rohan Builders official contact page confirmed matching registered address/phone</t>
+        </is>
+      </c>
+      <c r="Y88" s="6" t="inlineStr">
+        <is>
+          <t>No named CFO/Treasury head/finance controller identified for this SPV despite searching MCA/registry, CARE Ratings rationale for related entity, Rajdeep Group and Rohan Builders sites. Existing hint email confirmed real but appears general/BD mailbox rather than finance-specific.</t>
+        </is>
+      </c>
+      <c r="Z88" s="4" t="inlineStr">
+        <is>
+          <t>Rohan Suhas Lunkad | Managing Director  (MEDIUM)
+Dilip Popatlal Dhadiwal | Director (also director at Rajdeep Buildcon Pvt Ltd, co-promoter group)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA88" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">

</xml_diff>

<commit_message>
enrich batch (1AM pass): rows 87-101
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -10401,16 +10401,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R89" s="4" t="n"/>
-      <c r="S89" s="4" t="n"/>
-      <c r="T89" s="4" t="n"/>
-      <c r="U89" s="4" t="n"/>
-      <c r="V89" s="4" t="n"/>
-      <c r="W89" s="4" t="n"/>
-      <c r="X89" s="4" t="n"/>
-      <c r="Y89" s="4" t="n"/>
-      <c r="Z89" s="4" t="n"/>
-      <c r="AA89" s="4" t="n"/>
+      <c r="R89" s="5" t="inlineStr">
+        <is>
+          <t>Sivaram D V</t>
+        </is>
+      </c>
+      <c r="S89" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, My Home Group (CFO of group entities incl. My Home Industries Pvt Ltd / My Home Holdings Pvt Ltd)</t>
+        </is>
+      </c>
+      <c r="T89" s="5" t="n"/>
+      <c r="U89" s="5" t="n"/>
+      <c r="V89" s="5" t="inlineStr">
+        <is>
+          <t>info@myhomeinfrastructures.com; My Home Group HQ landline +91-40-6700 0000 (My Home Hub, Hi-Tech City, Madhapur, Hyderabad)</t>
+        </is>
+      </c>
+      <c r="W89" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X89" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn profile (CFO, My Home Holdings/My Home Industries Pvt Ltd), corroborated by ZoomInfo and RocketReach; company registered email from ZaubaCorp/IndiaFilings/D&amp;B listings</t>
+        </is>
+      </c>
+      <c r="Y89" s="5" t="inlineStr">
+        <is>
+          <t>My Home Group runs centralized finance across real estate/cement/infra arms from same Hyderabad HQ. Sivaram D V confirmed as CFO of Group/Industries &amp; Holdings entities, but no source explicitly names him CFO of 'My Home Infrastructures Pvt Ltd' specifically - likely-but-unconfirmed for this exact entity. No NCD/debenture trustee filing found for this entity.</t>
+        </is>
+      </c>
+      <c r="Z89" s="4" t="inlineStr">
+        <is>
+          <t>Registered company email (generic) | info@myhomeinfrastructures.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA89" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -10476,16 +10508,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R90" s="4" t="n"/>
-      <c r="S90" s="4" t="n"/>
-      <c r="T90" s="4" t="n"/>
-      <c r="U90" s="4" t="n"/>
-      <c r="V90" s="4" t="n"/>
-      <c r="W90" s="4" t="n"/>
-      <c r="X90" s="4" t="n"/>
-      <c r="Y90" s="4" t="n"/>
-      <c r="Z90" s="4" t="n"/>
-      <c r="AA90" s="4" t="n"/>
+      <c r="R90" s="3" t="inlineStr">
+        <is>
+          <t>Arvind Kumar Talan</t>
+        </is>
+      </c>
+      <c r="S90" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO), EESL</t>
+        </is>
+      </c>
+      <c r="T90" s="3" t="n"/>
+      <c r="U90" s="3" t="n"/>
+      <c r="V90" s="3" t="inlineStr">
+        <is>
+          <t>helpline@eesl.co.in; EESL Noida office phone 0120-6541600; toll-free 09240268676</t>
+        </is>
+      </c>
+      <c r="W90" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X90" s="3" t="inlineStr">
+        <is>
+          <t>PSUWatch, APAC News Network (2 articles), LinkedIn, ZoomInfo listing confirming @eesl.co.in domain and CFO title</t>
+        </is>
+      </c>
+      <c r="Y90" s="3" t="inlineStr">
+        <is>
+          <t>Appointed CFO of EESL 20 June 2024; CA with ~25 years experience. Multiple sources agree on identity, but no verified direct email/mobile found - masked on ZoomInfo/RocketReach, not reproduced. General helpline/RTI contact offered as fallback only.</t>
+        </is>
+      </c>
+      <c r="Z90" s="4" t="inlineStr">
+        <is>
+          <t>Sanjiv Garg | Director (part-time, nominee), EESL / Executive Director (Finance), REC Limited  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA90" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -10546,16 +10610,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R91" s="4" t="n"/>
-      <c r="S91" s="4" t="n"/>
-      <c r="T91" s="4" t="n"/>
-      <c r="U91" s="4" t="n"/>
-      <c r="V91" s="4" t="n"/>
-      <c r="W91" s="4" t="n"/>
-      <c r="X91" s="4" t="n"/>
-      <c r="Y91" s="4" t="n"/>
-      <c r="Z91" s="4" t="n"/>
-      <c r="AA91" s="4" t="n"/>
+      <c r="R91" s="3" t="inlineStr">
+        <is>
+          <t>Rakesh Tiwary</t>
+        </is>
+      </c>
+      <c r="S91" s="3" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer, Raymond Limited (parent/promoter group of the former Ring Plus Aqua Ltd.)</t>
+        </is>
+      </c>
+      <c r="T91" s="3" t="n"/>
+      <c r="U91" s="3" t="n"/>
+      <c r="V91" s="3" t="inlineStr">
+        <is>
+          <t>corp.secretarial@raymond.in; Raymond Limited registered office (Thane) phone +91-22-6152 7000</t>
+        </is>
+      </c>
+      <c r="W91" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X91" s="3" t="inlineStr">
+        <is>
+          <t>Multiple corroborating news reports (exchange4media, storyboard18, mediabrief, rprealtyplus, themachinemaker) confirming Rakesh Tiwary's appointment as Raymond's Group CFO effective 3 Dec 2025; CARE Ratings rationale PDF confirming Ring Plus Aqua as a Raymond step-down subsidiary</t>
+        </is>
+      </c>
+      <c r="Y91" s="3" t="inlineStr">
+        <is>
+          <t>IMPORTANT: Ring Plus Aqua Limited was legally amalgamated per NCLT (Mumbai) order dated 4 July 2025, merged into JK Maini Precision Technology Limited, and ceased to exist as a separate legal entity. Not a live NCD issuer to contact directly. Could not verify direct personal email/phone for Rakesh Tiwary. Existing hint contact amit.jangid@raymond.in could not be corroborated to a specific named person.</t>
+        </is>
+      </c>
+      <c r="Z91" s="4" t="inlineStr">
+        <is>
+          <t>Sridhar Venkatachari (V. Sridhar / Sridhar V) | Chief Financial Officer, Maini Precision Products Ltd (Raymond-Maini JV entity now housing the former Ring Plus Aqua auto-components business)  (MEDIUM)
+Company Secretary / Investor Relations desk, Raymond Limited group | corp.secretarial@raymond.in | +91-22-6152 7000 (Raymond Ltd registered office, Thane West)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA91" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -10606,16 +10703,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R92" s="4" t="n"/>
-      <c r="S92" s="4" t="n"/>
-      <c r="T92" s="4" t="n"/>
-      <c r="U92" s="4" t="n"/>
-      <c r="V92" s="4" t="n"/>
-      <c r="W92" s="4" t="n"/>
-      <c r="X92" s="4" t="n"/>
-      <c r="Y92" s="4" t="n"/>
-      <c r="Z92" s="4" t="n"/>
-      <c r="AA92" s="4" t="n"/>
+      <c r="R92" s="3" t="inlineStr">
+        <is>
+          <t>Milind Gandhi</t>
+        </is>
+      </c>
+      <c r="S92" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, IL&amp;FS Transportation Networks Ltd. (ITNL) / Roadstar Investment Managers Ltd. (Investment Manager of Roadstar Infra Investment Trust, sponsor of this SPV); also a Director on the board of Moradabad Bareilly Expressway Ltd. itself</t>
+        </is>
+      </c>
+      <c r="T92" s="3" t="n"/>
+      <c r="U92" s="3" t="n"/>
+      <c r="V92" s="3" t="inlineStr">
+        <is>
+          <t>itnl.secretarial@ilfsindia.com (ITNL group secretarial contact); Roadstar Investment Managers Ltd. general line: 022-2653 3333 / riml@roadstarinfra.com</t>
+        </is>
+      </c>
+      <c r="W92" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X92" s="3" t="inlineStr">
+        <is>
+          <t>Business Standard (ITNL CFO appointment, Milind Gandhi effective Oct 2022); Roadstar Infra Investment Trust team/bio page describing him as CFO of the Investment Manager since Feb 2020; ZaubaCorp/Tofler director listing naming Milind Ramesh Gandhi as director</t>
+        </is>
+      </c>
+      <c r="Y92" s="3" t="inlineStr">
+        <is>
+          <t>This is an IL&amp;FS Group toll-road SPV; day-to-day finance is run centrally by ITNL/Roadstar Investment Managers rather than a dedicated on-site CFO. No direct personal email/mobile found in public sources - only group secretarial/IR desk contacts.</t>
+        </is>
+      </c>
+      <c r="Z92" s="4" t="inlineStr">
+        <is>
+          <t>Krishna Ghag | Vice President &amp; Company Secretary, IL&amp;FS Transportation Networks Ltd. | krishna.ghag@ilfsindia.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA92" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -10666,16 +10795,48 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R93" s="4" t="n"/>
-      <c r="S93" s="4" t="n"/>
-      <c r="T93" s="4" t="n"/>
-      <c r="U93" s="4" t="n"/>
-      <c r="V93" s="4" t="n"/>
-      <c r="W93" s="4" t="n"/>
-      <c r="X93" s="4" t="n"/>
-      <c r="Y93" s="4" t="n"/>
-      <c r="Z93" s="4" t="n"/>
-      <c r="AA93" s="4" t="n"/>
+      <c r="R93" s="3" t="inlineStr">
+        <is>
+          <t>Aditya Arora</t>
+        </is>
+      </c>
+      <c r="S93" s="3" t="inlineStr">
+        <is>
+          <t>Senior Vice President - Finance &amp; Strategy, Conscient Group (parent/flagship of Heritage Max Realtech Pvt. Ltd.)</t>
+        </is>
+      </c>
+      <c r="T93" s="3" t="n"/>
+      <c r="U93" s="3" t="inlineStr">
+        <is>
+          <t>aditya.arora@conscient.in</t>
+        </is>
+      </c>
+      <c r="V93" s="3" t="n"/>
+      <c r="W93" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X93" s="3" t="inlineStr">
+        <is>
+          <t>RocketReach, Apollo.io, and LinkedIn all independently list Aditya Arora as Conscient Group Senior VP - Finance and Strategy</t>
+        </is>
+      </c>
+      <c r="Y93" s="3" t="inlineStr">
+        <is>
+          <t>Confirms existing hint contact is a genuine, current senior finance leader (CA, ex-EY) at group level covering Heritage Max Realtech. No dedicated standalone CFO found for this SPV itself.</t>
+        </is>
+      </c>
+      <c r="Z93" s="4" t="inlineStr">
+        <is>
+          <t>Ankur Gupta | Company Secretary (KMP) and Director, Heritage Max Realtech Pvt. Ltd.  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA93" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10756,16 +10917,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R94" s="4" t="n"/>
-      <c r="S94" s="4" t="n"/>
-      <c r="T94" s="4" t="n"/>
-      <c r="U94" s="4" t="n"/>
-      <c r="V94" s="4" t="n"/>
-      <c r="W94" s="4" t="n"/>
-      <c r="X94" s="4" t="n"/>
-      <c r="Y94" s="4" t="n"/>
-      <c r="Z94" s="4" t="n"/>
-      <c r="AA94" s="4" t="n"/>
+      <c r="R94" s="3" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="S94" s="3" t="inlineStr">
+        <is>
+          <t>Director (Finance) &amp; Chief Financial Officer, BSNL</t>
+        </is>
+      </c>
+      <c r="T94" s="3" t="n"/>
+      <c r="U94" s="3" t="inlineStr">
+        <is>
+          <t>dirfin@bsnl.co.in</t>
+        </is>
+      </c>
+      <c r="V94" s="3" t="inlineStr">
+        <is>
+          <t>BSNL Corporate Office landline: 011-23714141 (Director Finance office); general: +91-11-23713333</t>
+        </is>
+      </c>
+      <c r="W94" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X94" s="3" t="inlineStr">
+        <is>
+          <t>Official BSNL website board_of_directors page profiling Rajiv Kumar as Director-(Finance); ACC approval news extending additional charge as MTNL Director Finance from 1 Dec 2025; multiple LinkedIn profiles and ZoomInfo listing 'Director Finance &amp; CFO at BSNL'</t>
+        </is>
+      </c>
+      <c r="Y94" s="3" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar assumed charge as Director (Finance) &amp; CFO, BSNL on 01.12.2022, current as of most recent 2025-dated appointment news. dirfin@bsnl.co.in is a role-based official email per standard BSNL convention, tied specifically to this office.</t>
+        </is>
+      </c>
+      <c r="Z94" s="4" t="inlineStr">
+        <is>
+          <t>H. C. Pant (existing hint contact) | Unverified - appears in 2020-era BSNL/MTNL merger coordination correspondence; current role could not be confirmed | 91-11-23717844 | hcpant@bsnl.co.in  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA94" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -10826,16 +11023,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R95" s="4" t="n"/>
-      <c r="S95" s="4" t="n"/>
-      <c r="T95" s="4" t="n"/>
-      <c r="U95" s="4" t="n"/>
-      <c r="V95" s="4" t="n"/>
-      <c r="W95" s="4" t="n"/>
-      <c r="X95" s="4" t="n"/>
-      <c r="Y95" s="4" t="n"/>
-      <c r="Z95" s="4" t="n"/>
-      <c r="AA95" s="4" t="n"/>
+      <c r="R95" s="5" t="inlineStr">
+        <is>
+          <t>Namrata Aasi</t>
+        </is>
+      </c>
+      <c r="S95" s="5" t="inlineStr">
+        <is>
+          <t>Company Secretary &amp; Compliance Officer</t>
+        </is>
+      </c>
+      <c r="T95" s="5" t="n"/>
+      <c r="U95" s="5" t="inlineStr">
+        <is>
+          <t>compsec@greenstar.net.in</t>
+        </is>
+      </c>
+      <c r="V95" s="5" t="inlineStr">
+        <is>
+          <t>feedback@greenstar.net.in; Registered office: SPIC House, No. 88, Mount Road, Guindy, Chennai 600032</t>
+        </is>
+      </c>
+      <c r="W95" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X95" s="5" t="inlineStr">
+        <is>
+          <t>Aggregated from company AGM notice via search-engine indexing, corroborated by ZaubaCorp/company director listings and RocketReach</t>
+        </is>
+      </c>
+      <c r="Y95" s="5" t="inlineStr">
+        <is>
+          <t>No named CFO identified for this unlisted company despite multiple searches. Namrata Aasi's LinkedIn/RocketReach shows current affiliation as SPIC (related group company), raising doubt whether still active CS at Greenstar specifically - hence medium not high confidence.</t>
+        </is>
+      </c>
+      <c r="Z95" s="4" t="inlineStr">
+        <is>
+          <t>Manish Nagpal | Director (Non-Executive) - CA, structured trade/corporate finance background  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA95" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -10896,16 +11129,53 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R96" s="4" t="n"/>
-      <c r="S96" s="4" t="n"/>
-      <c r="T96" s="4" t="n"/>
-      <c r="U96" s="4" t="n"/>
-      <c r="V96" s="4" t="n"/>
-      <c r="W96" s="4" t="n"/>
-      <c r="X96" s="4" t="n"/>
-      <c r="Y96" s="4" t="n"/>
-      <c r="Z96" s="4" t="n"/>
-      <c r="AA96" s="4" t="n"/>
+      <c r="R96" s="5" t="inlineStr">
+        <is>
+          <t>Sameer Satish Negandhi</t>
+        </is>
+      </c>
+      <c r="S96" s="5" t="inlineStr">
+        <is>
+          <t>Company Secretary &amp; Director</t>
+        </is>
+      </c>
+      <c r="T96" s="5" t="n"/>
+      <c r="U96" s="5" t="inlineStr">
+        <is>
+          <t>sameer@gspbl.com</t>
+        </is>
+      </c>
+      <c r="V96" s="5" t="inlineStr">
+        <is>
+          <t>gayatrishakti@vsnl.net (old domain, unverified as active); registered office Andheri West, Mumbai</t>
+        </is>
+      </c>
+      <c r="W96" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X96" s="5" t="inlineStr">
+        <is>
+          <t>ZoomInfo, RocketReach, LinkedIn (in.linkedin.com/in/sameer-negandhi-a7410314), company contact-page indexing</t>
+        </is>
+      </c>
+      <c r="Y96" s="5" t="inlineStr">
+        <is>
+          <t>Email follows firstname@domain pattern matching search-indexed contact but not independently verified on live page. No separate named CFO found for this company.</t>
+        </is>
+      </c>
+      <c r="Z96" s="4" t="inlineStr">
+        <is>
+          <t>Kishan Varun | Assistant Manager, Accounts &amp; Finance  (LOW)
+Shailendrakumar Singh | Assistant Vice President (CA by qualification, department not confirmed)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA96" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -10976,16 +11246,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R97" s="4" t="n"/>
-      <c r="S97" s="4" t="n"/>
-      <c r="T97" s="4" t="n"/>
-      <c r="U97" s="4" t="n"/>
-      <c r="V97" s="4" t="n"/>
-      <c r="W97" s="4" t="n"/>
-      <c r="X97" s="4" t="n"/>
-      <c r="Y97" s="4" t="n"/>
-      <c r="Z97" s="4" t="n"/>
-      <c r="AA97" s="4" t="n"/>
+      <c r="R97" s="3" t="inlineStr">
+        <is>
+          <t>K. Prasad (Kolluru Prasad)</t>
+        </is>
+      </c>
+      <c r="S97" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T97" s="3" t="n"/>
+      <c r="U97" s="3" t="inlineStr">
+        <is>
+          <t>prasadk@sagarcements.in</t>
+        </is>
+      </c>
+      <c r="V97" s="3" t="inlineStr">
+        <is>
+          <t>investors@sagarcements.in; Tel: 040-23351571</t>
+        </is>
+      </c>
+      <c r="W97" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X97" s="3" t="inlineStr">
+        <is>
+          <t>sagarcements.in/investors/contact page (via search-engine indexing), LinkedIn (self-identifies as CFO), ZoomInfo, RocketReach, Bloomberg Markets profile - 4+ independent sources agree</t>
+        </is>
+      </c>
+      <c r="Y97" s="3" t="inlineStr">
+        <is>
+          <t>Qualified CA. Email/phone match company official domain/format, corroborated across 4+ sources. No personal mobile found.</t>
+        </is>
+      </c>
+      <c r="Z97" s="4" t="inlineStr">
+        <is>
+          <t>Dr. S. Anand Reddy | Managing Director | anand@sagarcements.in | Tel: 040-23351571  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA97" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -11036,16 +11342,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R98" s="4" t="n"/>
-      <c r="S98" s="4" t="n"/>
-      <c r="T98" s="4" t="n"/>
-      <c r="U98" s="4" t="n"/>
-      <c r="V98" s="4" t="n"/>
-      <c r="W98" s="4" t="n"/>
-      <c r="X98" s="4" t="n"/>
-      <c r="Y98" s="4" t="n"/>
-      <c r="Z98" s="4" t="n"/>
-      <c r="AA98" s="4" t="n"/>
+      <c r="R98" s="3" t="inlineStr">
+        <is>
+          <t>Kuppusamy Ezhil Arasan</t>
+        </is>
+      </c>
+      <c r="S98" s="3" t="inlineStr">
+        <is>
+          <t>Director &amp; CFO, SPI Technologies India Pvt Ltd (Straive group entity)</t>
+        </is>
+      </c>
+      <c r="T98" s="3" t="n"/>
+      <c r="U98" s="3" t="inlineStr">
+        <is>
+          <t>ezhil.arasan@straive.com</t>
+        </is>
+      </c>
+      <c r="V98" s="3" t="n"/>
+      <c r="W98" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X98" s="3" t="inlineStr">
+        <is>
+          <t>Company's own leadership page (spitechindia.com/about-us/leadership) lists him as Director &amp; CFO; corroborated by MCA-based director records (mycorporateinfo.com, appointed 04-09-2012) and ZaubaCorp/Tofler director listings</t>
+        </is>
+      </c>
+      <c r="Y98" s="3" t="inlineStr">
+        <is>
+          <t>Same email already on file, now corroborated as belonging to the company's Director/CFO. No direct mobile number found publicly.</t>
+        </is>
+      </c>
+      <c r="Z98" s="4" t="inlineStr">
+        <is>
+          <t>Kumar Subramaniam | Director; Group CFO (now styled Chief Risk Officer &amp; Head of Corporate Development) at Straive, parent group  (LOW)
+Stuti Mathur | Company Secretary &amp; Compliance Officer (appointed 3 Sep 2020)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA98" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -11106,16 +11445,48 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R99" s="4" t="n"/>
-      <c r="S99" s="4" t="n"/>
-      <c r="T99" s="4" t="n"/>
-      <c r="U99" s="4" t="n"/>
-      <c r="V99" s="4" t="n"/>
-      <c r="W99" s="4" t="n"/>
-      <c r="X99" s="4" t="n"/>
-      <c r="Y99" s="4" t="n"/>
-      <c r="Z99" s="4" t="n"/>
-      <c r="AA99" s="4" t="n"/>
+      <c r="R99" s="5" t="inlineStr">
+        <is>
+          <t>Vaibhav Goyal</t>
+        </is>
+      </c>
+      <c r="S99" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Indium (rebranded from Indium Software in 2026)</t>
+        </is>
+      </c>
+      <c r="T99" s="5" t="n"/>
+      <c r="U99" s="5" t="n"/>
+      <c r="V99" s="5" t="inlineStr">
+        <is>
+          <t>isil@indiumsoft.com; accounts.helpdesk@indiumsoft.com</t>
+        </is>
+      </c>
+      <c r="W99" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X99" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn, ZoomInfo, RocketReach and EasyLeadz profiles listing him as CFO at Indium, appointed circa May 2025</t>
+        </is>
+      </c>
+      <c r="Y99" s="5" t="inlineStr">
+        <is>
+          <t>Name and CFO title corroborated across LinkedIn plus multiple aggregators. Personal email appears only masked with inconsistent domains across sources - left null rather than guessed.</t>
+        </is>
+      </c>
+      <c r="Z99" s="4" t="inlineStr">
+        <is>
+          <t>Generic company/registrar mailbox (ISIL = Indium Software India Ltd) | isil@indiumsoft.com | accounts.helpdesk@indiumsoft.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA99" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -11176,16 +11547,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R100" s="4" t="n"/>
-      <c r="S100" s="4" t="n"/>
-      <c r="T100" s="4" t="n"/>
-      <c r="U100" s="4" t="n"/>
-      <c r="V100" s="4" t="n"/>
-      <c r="W100" s="4" t="n"/>
-      <c r="X100" s="4" t="n"/>
-      <c r="Y100" s="4" t="n"/>
-      <c r="Z100" s="4" t="n"/>
-      <c r="AA100" s="4" t="n"/>
+      <c r="R100" s="3" t="inlineStr">
+        <is>
+          <t>Sarbani Mitra</t>
+        </is>
+      </c>
+      <c r="S100" s="3" t="inlineStr">
+        <is>
+          <t>Company Secretary &amp; Compliance Officer; Senior General Manager, Head - Legal &amp; Corporate Communications</t>
+        </is>
+      </c>
+      <c r="T100" s="3" t="n"/>
+      <c r="U100" s="3" t="n"/>
+      <c r="V100" s="3" t="inlineStr">
+        <is>
+          <t>investors@hpl.co.in; landline +91 (033) 2367 3484/3485/3383 (Kolkata); plant line +91 (03224) 274007/384/400/876 (Haldia)</t>
+        </is>
+      </c>
+      <c r="W100" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X100" s="3" t="inlineStr">
+        <is>
+          <t>Signatory on official BSE regulatory filings (NCD-related), corroborated by TheOrg and ZoomInfo listing same name/title</t>
+        </is>
+      </c>
+      <c r="Y100" s="3" t="inlineStr">
+        <is>
+          <t>As Company Secretary, named signatory on the company's actual NCD/debenture-related BSE filings. Direct email/mobile not publicly found, verified IR mailbox given as fallback.</t>
+        </is>
+      </c>
+      <c r="Z100" s="4" t="inlineStr">
+        <is>
+          <t>Neela Madhab Patnaik | EVP &amp; CFO, Haldia Petrochemicals Limited (per current org-chart listing)  (LOW)
+Durga Sankar Chakrabarti | Head - Finance &amp; Accounts, Senior Vice President and CFO  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA100" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -11246,16 +11650,52 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R101" s="4" t="n"/>
-      <c r="S101" s="4" t="n"/>
-      <c r="T101" s="4" t="n"/>
-      <c r="U101" s="4" t="n"/>
-      <c r="V101" s="4" t="n"/>
-      <c r="W101" s="4" t="n"/>
-      <c r="X101" s="4" t="n"/>
-      <c r="Y101" s="4" t="n"/>
-      <c r="Z101" s="4" t="n"/>
-      <c r="AA101" s="4" t="n"/>
+      <c r="R101" s="3" t="inlineStr">
+        <is>
+          <t>Vineet Sukumar</t>
+        </is>
+      </c>
+      <c r="S101" s="3" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO/Managing Director, Vivriti Asset Management</t>
+        </is>
+      </c>
+      <c r="T101" s="3" t="n"/>
+      <c r="U101" s="3" t="inlineStr">
+        <is>
+          <t>vineet@vivritiamc.com</t>
+        </is>
+      </c>
+      <c r="V101" s="3" t="inlineStr">
+        <is>
+          <t>+91-44-4007-4800 (Vivriti AMC Chennai office, Prestige Zackria Metropolitan, Anna Salai, Chennai 600002)</t>
+        </is>
+      </c>
+      <c r="W101" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X101" s="3" t="inlineStr">
+        <is>
+          <t>YourStory company profile, PMS Bazaar AMC profile, company About-us page - existing on-file email matches confirmed role as Founder/CEO</t>
+        </is>
+      </c>
+      <c r="Y101" s="3" t="inlineStr">
+        <is>
+          <t>Vineet Sukumar leads the AMC entity (CIN U65929TN2019PTC127644) itself, distinct from sister NBFC Vivriti Capital Ltd. No separately-named dedicated CFO for the AMC entity could be verified.</t>
+        </is>
+      </c>
+      <c r="Z101" s="4" t="inlineStr">
+        <is>
+          <t>Srinivasaraghavan Badrinathan | Chief Financial Officer, Vivriti Capital Limited (Group/parent NBFC sister entity)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA101" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -11336,16 +11776,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R102" s="4" t="n"/>
-      <c r="S102" s="4" t="n"/>
-      <c r="T102" s="4" t="n"/>
-      <c r="U102" s="4" t="n"/>
-      <c r="V102" s="4" t="n"/>
-      <c r="W102" s="4" t="n"/>
-      <c r="X102" s="4" t="n"/>
-      <c r="Y102" s="4" t="n"/>
-      <c r="Z102" s="4" t="n"/>
-      <c r="AA102" s="4" t="n"/>
+      <c r="R102" s="3" t="inlineStr">
+        <is>
+          <t>Jairam Paravastu Sampath</t>
+        </is>
+      </c>
+      <c r="S102" s="3" t="inlineStr">
+        <is>
+          <t>Whole-Time Director &amp; Chief Financial Officer (DIN 08064368)</t>
+        </is>
+      </c>
+      <c r="T102" s="3" t="n"/>
+      <c r="U102" s="3" t="n"/>
+      <c r="V102" s="3" t="inlineStr">
+        <is>
+          <t>kaynestechcs@kaynestechnology.net; phone 91-821-4002805</t>
+        </is>
+      </c>
+      <c r="W102" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X102" s="3" t="inlineStr">
+        <is>
+          <t>Kaynes Technology's own Our Team page, TheOrg org chart, ZoomInfo, Inc42 news, LinkedIn - multiple independent sources agree</t>
+        </is>
+      </c>
+      <c r="Y102" s="3" t="inlineStr">
+        <is>
+          <t>With company since 2011, leads finance &amp; strategy. Direct corporate email masked on people-data sites, left null. Verified company/CS email is safest channel.</t>
+        </is>
+      </c>
+      <c r="Z102" s="4" t="inlineStr">
+        <is>
+          <t>Sumit Kumar Verma | Investor Relations &amp; Business Analyst | sumit.verma@kaynestechnology.net | ir@kaynestechnology.net  (MEDIUM)
+Sudhasri Addepalli | Company Secretary &amp; Compliance Officer | kaynestechcs@kaynestechnology.net  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA102" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -11406,16 +11879,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R103" s="4" t="n"/>
-      <c r="S103" s="4" t="n"/>
-      <c r="T103" s="4" t="n"/>
-      <c r="U103" s="4" t="n"/>
-      <c r="V103" s="4" t="n"/>
-      <c r="W103" s="4" t="n"/>
-      <c r="X103" s="4" t="n"/>
-      <c r="Y103" s="4" t="n"/>
-      <c r="Z103" s="4" t="n"/>
-      <c r="AA103" s="4" t="n"/>
+      <c r="R103" s="5" t="inlineStr">
+        <is>
+          <t>Chitrakala Rajkumar</t>
+        </is>
+      </c>
+      <c r="S103" s="5" t="inlineStr">
+        <is>
+          <t>Director &amp; Co-Founder (promoter-director; no dedicated CFO/finance officer identified)</t>
+        </is>
+      </c>
+      <c r="T103" s="5" t="n"/>
+      <c r="U103" s="5" t="inlineStr">
+        <is>
+          <t>chitrakala_8@hotmail.com</t>
+        </is>
+      </c>
+      <c r="V103" s="5" t="n"/>
+      <c r="W103" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X103" s="5" t="inlineStr">
+        <is>
+          <t>Tofler director record, Zauba Corp company/director listing, corroborated by hospital's own history (co-founded Lifeline Hospital in 1997 with Dr. J.S. Rajkumar)</t>
+        </is>
+      </c>
+      <c r="Y103" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed director/promoter, not a titled finance executive. No separate CFO/Head of Finance/Treasury contact found despite being a rated debt issuer (CRISIL BB-/Stable); rating documents did not surface named finance contacts.</t>
+        </is>
+      </c>
+      <c r="Z103" s="4" t="inlineStr">
+        <is>
+          <t>Anirudh Rajkumar | Joint Managing Director (surgeon by profession; DIN 02060595)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA103" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">

</xml_diff>

<commit_message>
enrich batch (1AM pass): rows 102-116
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -12001,16 +12001,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R104" s="4" t="n"/>
-      <c r="S104" s="4" t="n"/>
-      <c r="T104" s="4" t="n"/>
-      <c r="U104" s="4" t="n"/>
-      <c r="V104" s="4" t="n"/>
-      <c r="W104" s="4" t="n"/>
-      <c r="X104" s="4" t="n"/>
-      <c r="Y104" s="4" t="n"/>
-      <c r="Z104" s="4" t="n"/>
-      <c r="AA104" s="4" t="n"/>
+      <c r="R104" s="3" t="inlineStr">
+        <is>
+          <t>Ankit Jain</t>
+        </is>
+      </c>
+      <c r="S104" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T104" s="3" t="n"/>
+      <c r="U104" s="3" t="n"/>
+      <c r="V104" s="3" t="inlineStr">
+        <is>
+          <t>deepika_sharma@mas.co.in / +91-79-41106500</t>
+        </is>
+      </c>
+      <c r="W104" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X104" s="3" t="inlineStr">
+        <is>
+          <t>Corroborated across ZoomInfo, Bloomberg Markets profile, MarketScreener insider profile, LinkedIn, and BSE corporate filing reference - CFO since ~2021</t>
+        </is>
+      </c>
+      <c r="Y104" s="3" t="inlineStr">
+        <is>
+          <t>Direct email/mobile could not be found; masked on aggregators. Not populated per hard rule against guessing.</t>
+        </is>
+      </c>
+      <c r="Z104" s="4" t="inlineStr">
+        <is>
+          <t>Deepika Sharma | Contact on record (role unverified - possibly Company Secretary/Compliance or IR desk staff) | +91-79-41106500 | deepika_sharma@mas.co.in  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA104" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -12091,16 +12123,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R105" s="4" t="n"/>
-      <c r="S105" s="4" t="n"/>
-      <c r="T105" s="4" t="n"/>
-      <c r="U105" s="4" t="n"/>
-      <c r="V105" s="4" t="n"/>
-      <c r="W105" s="4" t="n"/>
-      <c r="X105" s="4" t="n"/>
-      <c r="Y105" s="4" t="n"/>
-      <c r="Z105" s="4" t="n"/>
-      <c r="AA105" s="4" t="n"/>
+      <c r="R105" s="3" t="inlineStr">
+        <is>
+          <t>Vineet Singhal</t>
+        </is>
+      </c>
+      <c r="S105" s="3" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer (Group CFO)</t>
+        </is>
+      </c>
+      <c r="T105" s="3" t="n"/>
+      <c r="U105" s="3" t="n"/>
+      <c r="V105" s="3" t="inlineStr">
+        <is>
+          <t>gaursons@gaursonsindia.com / +91-120-4343333; customercare@gaursonsindia.com</t>
+        </is>
+      </c>
+      <c r="W105" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X105" s="3" t="inlineStr">
+        <is>
+          <t>Corroborated across RocketReach, Salesgear.io, Crunchbase, ZoomInfo, and LinkedIn as Group CFO/Director of Finance</t>
+        </is>
+      </c>
+      <c r="Y105" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant, previously Finance Controller at Aircom. Direct verified email/mobile not found; masked address on unrelated project-entity domain, not populated per hard rule.</t>
+        </is>
+      </c>
+      <c r="Z105" s="4" t="inlineStr">
+        <is>
+          <t>Anjali Verma | DGM &amp; Company Secretary / Compliance Officer, Gaursons Group (Membership No. F7362) | customercare@gaursonsindia.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA105" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -12181,16 +12245,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R106" s="4" t="n"/>
-      <c r="S106" s="4" t="n"/>
-      <c r="T106" s="4" t="n"/>
-      <c r="U106" s="4" t="n"/>
-      <c r="V106" s="4" t="n"/>
-      <c r="W106" s="4" t="n"/>
-      <c r="X106" s="4" t="n"/>
-      <c r="Y106" s="4" t="n"/>
-      <c r="Z106" s="4" t="n"/>
-      <c r="AA106" s="4" t="n"/>
+      <c r="R106" s="3" t="inlineStr">
+        <is>
+          <t>Jasmeet Singh</t>
+        </is>
+      </c>
+      <c r="S106" s="3" t="inlineStr">
+        <is>
+          <t>Vice President - Finance (company does not appear to publicly designate a separate CFO title)</t>
+        </is>
+      </c>
+      <c r="T106" s="3" t="n"/>
+      <c r="U106" s="3" t="n"/>
+      <c r="V106" s="3" t="inlineStr">
+        <is>
+          <t>njain@geecl.com / +91-124-2580470; info@geecl.com</t>
+        </is>
+      </c>
+      <c r="W106" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X106" s="3" t="inlineStr">
+        <is>
+          <t>Corroborated across TheOrg.com org chart, RocketReach, and LinkedIn - VP Finance since June 2012</t>
+        </is>
+      </c>
+      <c r="Y106" s="3" t="inlineStr">
+        <is>
+          <t>No GEECL-specific CFO appointment/resignation filing found, so VP Finance is put forward as primary contact. Direct email/mobile not found, not populated per hard rule.</t>
+        </is>
+      </c>
+      <c r="Z106" s="4" t="inlineStr">
+        <is>
+          <t>Pawan Kumar | AGM Finance, Great Eastern Energy Corporation  (LOW)
+Ajeet Kumar | Senior Manager Finance, Great Eastern Energy Corporation  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA106" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -12251,16 +12348,44 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R107" s="4" t="n"/>
-      <c r="S107" s="4" t="n"/>
-      <c r="T107" s="4" t="n"/>
-      <c r="U107" s="4" t="n"/>
-      <c r="V107" s="4" t="n"/>
-      <c r="W107" s="4" t="n"/>
-      <c r="X107" s="4" t="n"/>
-      <c r="Y107" s="4" t="n"/>
+      <c r="R107" s="3" t="inlineStr">
+        <is>
+          <t>Murali Krishna Yarla</t>
+        </is>
+      </c>
+      <c r="S107" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T107" s="3" t="n"/>
+      <c r="U107" s="3" t="n"/>
+      <c r="V107" s="3" t="inlineStr">
+        <is>
+          <t>connect@greengold.tv; phone +91 40 4436 1900/1990 (Hyderabad HQ)</t>
+        </is>
+      </c>
+      <c r="W107" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X107" s="3" t="inlineStr">
+        <is>
+          <t>TheOrg profile, ZoomInfo listing, and LinkedIn profile - consistent across 3 independent sources, CFO since Oct 2022</t>
+        </is>
+      </c>
+      <c r="Y107" s="3" t="inlineStr">
+        <is>
+          <t>Masked email on ZoomInfo, no reliable domain pattern to infer from, left null. Appears to be part-time/fractional CFO, concurrently VP-Finance at ANA Oils and Fats India. Existing hint email looks like external CA consultant's personal address, could not confirm validity.</t>
+        </is>
+      </c>
       <c r="Z107" s="4" t="n"/>
-      <c r="AA107" s="4" t="n"/>
+      <c r="AA107" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -12321,16 +12446,52 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R108" s="4" t="n"/>
-      <c r="S108" s="4" t="n"/>
-      <c r="T108" s="4" t="n"/>
-      <c r="U108" s="4" t="n"/>
-      <c r="V108" s="4" t="n"/>
-      <c r="W108" s="4" t="n"/>
-      <c r="X108" s="4" t="n"/>
-      <c r="Y108" s="4" t="n"/>
-      <c r="Z108" s="4" t="n"/>
-      <c r="AA108" s="4" t="n"/>
+      <c r="R108" s="5" t="inlineStr">
+        <is>
+          <t>Shubhabrata Banerjee</t>
+        </is>
+      </c>
+      <c r="S108" s="5" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer &amp; EVP</t>
+        </is>
+      </c>
+      <c r="T108" s="5" t="n"/>
+      <c r="U108" s="5" t="inlineStr">
+        <is>
+          <t>shubhabrata.banerjee@nihilent.com</t>
+        </is>
+      </c>
+      <c r="V108" s="5" t="inlineStr">
+        <is>
+          <t>Rahul Bhandari, Company Secretary - rahul.bhandari@nihilent.com</t>
+        </is>
+      </c>
+      <c r="W108" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X108" s="5" t="inlineStr">
+        <is>
+          <t>Corroborated by 6 independent sources (Crunchbase, TheOrg, Bloomberg, RocketReach, ZoomInfo, LinkedIn). Email inferred from observed firstname.lastname@nihilent.com pattern confirmed real for existing hint contact</t>
+        </is>
+      </c>
+      <c r="Y108" s="5" t="inlineStr">
+        <is>
+          <t>Exact CFO email is INFERRED from company naming convention, not directly confirmed - medium confidence per rule. Two other CFO name variants surfaced in search were discarded as apparent mix-ups with unrelated people.</t>
+        </is>
+      </c>
+      <c r="Z108" s="4" t="inlineStr">
+        <is>
+          <t>Rahul Bhandari | Company Secretary (handles secretarial/compliance, including debt instruments) | rahul.bhandari@nihilent.com  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA108" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -12411,16 +12572,41 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R109" s="4" t="n"/>
-      <c r="S109" s="4" t="n"/>
-      <c r="T109" s="4" t="n"/>
-      <c r="U109" s="4" t="n"/>
-      <c r="V109" s="4" t="n"/>
-      <c r="W109" s="4" t="n"/>
-      <c r="X109" s="4" t="n"/>
-      <c r="Y109" s="4" t="n"/>
-      <c r="Z109" s="4" t="n"/>
-      <c r="AA109" s="4" t="n"/>
+      <c r="R109" s="6" t="n"/>
+      <c r="S109" s="6" t="n"/>
+      <c r="T109" s="6" t="n"/>
+      <c r="U109" s="6" t="n"/>
+      <c r="V109" s="6" t="inlineStr">
+        <is>
+          <t>compliance@ncml.com; existing landline 91-124-4338200 (existing sanjay.khare@ncmsl.com unverified as still active)</t>
+        </is>
+      </c>
+      <c r="W109" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X109" s="6" t="inlineStr">
+        <is>
+          <t>ZaubaCorp/Tracxn MCA aggregator listing for CIN U74140MH2004PLC148859 (registered email compliance@ncml.com)</t>
+        </is>
+      </c>
+      <c r="Y109" s="6" t="inlineStr">
+        <is>
+          <t>Could not confirm current named CFO. Most recent named Group CFO (Anuj Kumar Vasdev) left this role for Singer India Limited (CFO-Designate effective 18 Sep 2025). Existing hint contact Sanjay Khare now shows as Managing Partner at an unrelated advisory firm - downgraded to unverified fallback.</t>
+        </is>
+      </c>
+      <c r="Z109" s="4" t="inlineStr">
+        <is>
+          <t>Ashima Aneja | Company Secretary &amp; Compliance Officer  (LOW)
+Sanjay Kumar Gupta | Managing Director &amp; CEO  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA109" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -12471,16 +12657,52 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R110" s="4" t="n"/>
-      <c r="S110" s="4" t="n"/>
-      <c r="T110" s="4" t="n"/>
-      <c r="U110" s="4" t="n"/>
-      <c r="V110" s="4" t="n"/>
-      <c r="W110" s="4" t="n"/>
-      <c r="X110" s="4" t="n"/>
-      <c r="Y110" s="4" t="n"/>
-      <c r="Z110" s="4" t="n"/>
-      <c r="AA110" s="4" t="n"/>
+      <c r="R110" s="5" t="inlineStr">
+        <is>
+          <t>Sumant Sinha</t>
+        </is>
+      </c>
+      <c r="S110" s="5" t="inlineStr">
+        <is>
+          <t>Promoter/Director (Founder-Chairman &amp; CEO, ReNew Power/ReNew Energy Global; beneficial owner of Wisemore Advisory)</t>
+        </is>
+      </c>
+      <c r="T110" s="5" t="n"/>
+      <c r="U110" s="5" t="inlineStr">
+        <is>
+          <t>sumant@renewpower.in</t>
+        </is>
+      </c>
+      <c r="V110" s="5" t="inlineStr">
+        <is>
+          <t>wisemoreadvisory@gmail.com</t>
+        </is>
+      </c>
+      <c r="W110" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X110" s="5" t="inlineStr">
+        <is>
+          <t>Zauba Corp MCA-derived company/director record; CARE Ratings press release on Wisemore Advisory NCDs (16-Aug-2022) confirming SPV structure</t>
+        </is>
+      </c>
+      <c r="Y110" s="5" t="inlineStr">
+        <is>
+          <t>Wisemore Advisory is a promoter-held investment/holding SPV to hold pledged ReNew Power shares as security for listed zero-coupon NCDs. No independently identifiable CFO/treasury head/finance dept of its own. Email tied to director per aggregator, not independently confirmed - medium confidence. Registered gmail is safer first contact point.</t>
+        </is>
+      </c>
+      <c r="Z110" s="4" t="inlineStr">
+        <is>
+          <t>Vaishali Nigam Sinha | Director / Managing Director, Wisemore Advisory (also Chief Sustainability, CSR &amp; Communications Officer, ReNew Energy Global)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA110" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -12531,16 +12753,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R111" s="4" t="n"/>
-      <c r="S111" s="4" t="n"/>
-      <c r="T111" s="4" t="n"/>
-      <c r="U111" s="4" t="n"/>
-      <c r="V111" s="4" t="n"/>
-      <c r="W111" s="4" t="n"/>
-      <c r="X111" s="4" t="n"/>
-      <c r="Y111" s="4" t="n"/>
-      <c r="Z111" s="4" t="n"/>
-      <c r="AA111" s="4" t="n"/>
+      <c r="R111" s="5" t="inlineStr">
+        <is>
+          <t>Mariyappan M</t>
+        </is>
+      </c>
+      <c r="S111" s="5" t="inlineStr">
+        <is>
+          <t>Treasury Manager, ABT Industries Limited</t>
+        </is>
+      </c>
+      <c r="T111" s="5" t="n"/>
+      <c r="U111" s="5" t="n"/>
+      <c r="V111" s="5" t="inlineStr">
+        <is>
+          <t>mnatarajan@abtindustries.net</t>
+        </is>
+      </c>
+      <c r="W111" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X111" s="5" t="inlineStr">
+        <is>
+          <t>RocketReach company finance-department listing - single source, direct email/phone withheld by aggregator paywall</t>
+        </is>
+      </c>
+      <c r="Y111" s="5" t="inlineStr">
+        <is>
+          <t>Part of Coimbatore-based ABT/Sakthi Group. A CFO reportedly appointed 14-Feb-2022 but name could not be located. Treasury Manager title is best-verified finance-specific role found.</t>
+        </is>
+      </c>
+      <c r="Z111" s="4" t="inlineStr">
+        <is>
+          <t>Kanna Venkatachalam | Company Secretary, ABT Industries Limited | mnatarajan@abtindustries.net  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA111" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -12601,16 +12855,48 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R112" s="4" t="n"/>
-      <c r="S112" s="4" t="n"/>
-      <c r="T112" s="4" t="n"/>
-      <c r="U112" s="4" t="n"/>
-      <c r="V112" s="4" t="n"/>
-      <c r="W112" s="4" t="n"/>
-      <c r="X112" s="4" t="n"/>
-      <c r="Y112" s="4" t="n"/>
-      <c r="Z112" s="4" t="n"/>
-      <c r="AA112" s="4" t="n"/>
+      <c r="R112" s="5" t="inlineStr">
+        <is>
+          <t>Sankha Bhattacharya</t>
+        </is>
+      </c>
+      <c r="S112" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director, Casablanca Industries Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="T112" s="5" t="n"/>
+      <c r="U112" s="5" t="n"/>
+      <c r="V112" s="5" t="inlineStr">
+        <is>
+          <t>cs1@casablancaindustries.in</t>
+        </is>
+      </c>
+      <c r="W112" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X112" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn profile, corroborated by ZoomInfo/RocketReach and MCA director records (indiafilings.com CIN U28113DL2011PTC223576)</t>
+        </is>
+      </c>
+      <c r="Y112" s="5" t="inlineStr">
+        <is>
+          <t>As MD, senior-most executive and de facto finance decision-maker; no dedicated CFO identified. Company was acquired by Trivium Packaging (effective 27-Feb-2025) - finance reporting lines may have changed, verify before outreach. A stale opwglobal.com email surfaced but was deliberately not used (prior employer). Registered cs1@ address is safer fallback.</t>
+        </is>
+      </c>
+      <c r="Z112" s="4" t="inlineStr">
+        <is>
+          <t>Rishheb Wassan | Director, Casablanca Industries (DIN 02477346; primary role as Director/Owner, Stella Indusstries Ltd.)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA112" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -12681,16 +12967,40 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R113" s="4" t="n"/>
-      <c r="S113" s="4" t="n"/>
-      <c r="T113" s="4" t="n"/>
-      <c r="U113" s="4" t="n"/>
-      <c r="V113" s="4" t="n"/>
-      <c r="W113" s="4" t="n"/>
-      <c r="X113" s="4" t="n"/>
-      <c r="Y113" s="4" t="n"/>
-      <c r="Z113" s="4" t="n"/>
-      <c r="AA113" s="4" t="n"/>
+      <c r="R113" s="6" t="n"/>
+      <c r="S113" s="6" t="n"/>
+      <c r="T113" s="6" t="n"/>
+      <c r="U113" s="6" t="n"/>
+      <c r="V113" s="6" t="inlineStr">
+        <is>
+          <t>essel.roads@gmail.com / 91-22-71084444</t>
+        </is>
+      </c>
+      <c r="W113" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X113" s="6" t="inlineStr">
+        <is>
+          <t>User-supplied MCA registered contact; email pattern corroborated as shared correspondence address across other Essel-group toll-road SPVs per IndiaFilings</t>
+        </is>
+      </c>
+      <c r="Y113" s="6" t="inlineStr">
+        <is>
+          <t>No named CFO/Treasury head/finance officer found for this SPV. Directors recur across multiple sister Essel toll-road SPVs, suggesting nominee/professional directors rather than dedicated finance executives. Wider Essel Infraprojects/Essel Highways group is under severe financial distress (CIRP proceedings on related entities), though this entity itself was still publishing quarterly results as of Dec 2024.</t>
+        </is>
+      </c>
+      <c r="Z113" s="4" t="inlineStr">
+        <is>
+          <t>Anjul Choudhary | Director (role/function unconfirmed - possibly nominee director)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA113" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -12751,16 +13061,48 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R114" s="4" t="n"/>
-      <c r="S114" s="4" t="n"/>
-      <c r="T114" s="4" t="n"/>
-      <c r="U114" s="4" t="n"/>
-      <c r="V114" s="4" t="n"/>
-      <c r="W114" s="4" t="n"/>
-      <c r="X114" s="4" t="n"/>
-      <c r="Y114" s="4" t="n"/>
-      <c r="Z114" s="4" t="n"/>
-      <c r="AA114" s="4" t="n"/>
+      <c r="R114" s="5" t="inlineStr">
+        <is>
+          <t>Chandrasekaran Vijayagopal</t>
+        </is>
+      </c>
+      <c r="S114" s="5" t="inlineStr">
+        <is>
+          <t>Finance Head / CFO (appointed CFO effective 11 Dec 2025)</t>
+        </is>
+      </c>
+      <c r="T114" s="5" t="n"/>
+      <c r="U114" s="5" t="n"/>
+      <c r="V114" s="5" t="inlineStr">
+        <is>
+          <t>nrfsi@nrfsi.com</t>
+        </is>
+      </c>
+      <c r="W114" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X114" s="5" t="inlineStr">
+        <is>
+          <t>ZoomInfo profile listing title Finance Head at NRFSI, CFO appointment dated 11 Dec 2025; corroborated by Highperformr aggregator</t>
+        </is>
+      </c>
+      <c r="Y114" s="5" t="inlineStr">
+        <is>
+          <t>Not independently confirmed via NRFSI's own website (blocked by egress) or MCA/DIN filing. Email masked on ZoomInfo, left null rather than guessed. Prior role: Director, Accounts at Northern Arc.</t>
+        </is>
+      </c>
+      <c r="Z114" s="4" t="inlineStr">
+        <is>
+          <t>Harmandeep Singh Walia | Managing Director | nrfsi@nrfsi.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA114" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -12821,16 +13163,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R115" s="4" t="n"/>
-      <c r="S115" s="4" t="n"/>
-      <c r="T115" s="4" t="n"/>
-      <c r="U115" s="4" t="n"/>
-      <c r="V115" s="4" t="n"/>
-      <c r="W115" s="4" t="n"/>
-      <c r="X115" s="4" t="n"/>
-      <c r="Y115" s="4" t="n"/>
-      <c r="Z115" s="4" t="n"/>
-      <c r="AA115" s="4" t="n"/>
+      <c r="R115" s="5" t="inlineStr">
+        <is>
+          <t>Rahul Jain</t>
+        </is>
+      </c>
+      <c r="S115" s="5" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer, Suzlon Energy Ltd (parent) - KMP effective 15 Dec 2025</t>
+        </is>
+      </c>
+      <c r="T115" s="5" t="n"/>
+      <c r="U115" s="5" t="n"/>
+      <c r="V115" s="5" t="inlineStr">
+        <is>
+          <t>mca@suzlon.com</t>
+        </is>
+      </c>
+      <c r="W115" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X115" s="5" t="inlineStr">
+        <is>
+          <t>Suzlon Energy official press release, corroborated by Business Standard/BusinessToday/People Matters coverage of the Oct 29, 2025 board announcement</t>
+        </is>
+      </c>
+      <c r="Y115" s="5" t="inlineStr">
+        <is>
+          <t>Appointment as Group CFO of listed parent is high confidence but applicability to this specific subsidiary is inferred (centralized group treasury, shared mca@suzlon.com mailbox), so downgraded to medium. Replaced Himanshu Mody (resigned 31 Aug 2025). No direct email found, not asserted.</t>
+        </is>
+      </c>
+      <c r="Z115" s="4" t="inlineStr">
+        <is>
+          <t>Om Prakash Talwar | CFO, Suzlon Global Services Ltd (per one LinkedIn profile; a second profile for same name says 'Ex CFO')  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA115" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -12881,16 +13255,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R116" s="4" t="n"/>
-      <c r="S116" s="4" t="n"/>
-      <c r="T116" s="4" t="n"/>
-      <c r="U116" s="4" t="n"/>
-      <c r="V116" s="4" t="n"/>
-      <c r="W116" s="4" t="n"/>
-      <c r="X116" s="4" t="n"/>
-      <c r="Y116" s="4" t="n"/>
-      <c r="Z116" s="4" t="n"/>
-      <c r="AA116" s="4" t="n"/>
+      <c r="R116" s="3" t="inlineStr">
+        <is>
+          <t>Nitesh Jain</t>
+        </is>
+      </c>
+      <c r="S116" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T116" s="3" t="n"/>
+      <c r="U116" s="3" t="n"/>
+      <c r="V116" s="3" t="inlineStr">
+        <is>
+          <t>rainbowfoundations@gmail.com; Landline 044-24344647/24354647; Registrar (Cameo Corporate Services) investor@cameoindia.com, +91-44-28462700</t>
+        </is>
+      </c>
+      <c r="W116" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X116" s="3" t="inlineStr">
+        <is>
+          <t>Corroborated across LinkedIn, ZoomInfo, and Bloomberg Markets profile as CFO; also appears in a BSE corporate filing dated 08-Sep-2025</t>
+        </is>
+      </c>
+      <c r="Y116" s="3" t="inlineStr">
+        <is>
+          <t>Identity and CFO title confirmed by 3+ sources. Masked personal email on rainbowfoundations.in domain, not verified, left null. No direct mobile found.</t>
+        </is>
+      </c>
+      <c r="Z116" s="4" t="inlineStr">
+        <is>
+          <t>Ikkapadath Bilal Mohammadali (also Bilal Muhammad) | Company Secretary &amp; Compliance Officer | rainbowfoundations@gmail.com; 044-24344647/24354647  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA116" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -12961,16 +13367,44 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R117" s="4" t="n"/>
-      <c r="S117" s="4" t="n"/>
-      <c r="T117" s="4" t="n"/>
-      <c r="U117" s="4" t="n"/>
-      <c r="V117" s="4" t="n"/>
-      <c r="W117" s="4" t="n"/>
-      <c r="X117" s="4" t="n"/>
-      <c r="Y117" s="4" t="n"/>
+      <c r="R117" s="3" t="inlineStr">
+        <is>
+          <t>Rajesh Katoch</t>
+        </is>
+      </c>
+      <c r="S117" s="3" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer (CEO) &amp; Director</t>
+        </is>
+      </c>
+      <c r="T117" s="3" t="n"/>
+      <c r="U117" s="3" t="n"/>
+      <c r="V117" s="3" t="inlineStr">
+        <is>
+          <t>info@ezcapital.in; phone 78370 78390</t>
+        </is>
+      </c>
+      <c r="W117" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X117" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed via ZoomInfo, LinkedIn, lead411.com, rocketreach.co, and company's own Board and Management Team page (ezcapital.in)</t>
+        </is>
+      </c>
+      <c r="Y117" s="3" t="inlineStr">
+        <is>
+          <t>Company operates under brand 'EZ Capital'. As of Aug 2026, company is actively recruiting for a dedicated CFO - indicating no confirmed named CFO currently; CEO is senior-most person overseeing financial strategy in the interim. Masked email not populated.</t>
+        </is>
+      </c>
       <c r="Z117" s="4" t="n"/>
-      <c r="AA117" s="4" t="n"/>
+      <c r="AA117" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -13036,16 +13470,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R118" s="4" t="n"/>
-      <c r="S118" s="4" t="n"/>
-      <c r="T118" s="4" t="n"/>
-      <c r="U118" s="4" t="n"/>
-      <c r="V118" s="4" t="n"/>
-      <c r="W118" s="4" t="n"/>
-      <c r="X118" s="4" t="n"/>
-      <c r="Y118" s="4" t="n"/>
-      <c r="Z118" s="4" t="n"/>
-      <c r="AA118" s="4" t="n"/>
+      <c r="R118" s="5" t="inlineStr">
+        <is>
+          <t>Pradeep Kumar Dhandhania</t>
+        </is>
+      </c>
+      <c r="S118" s="5" t="inlineStr">
+        <is>
+          <t>Director / VP - Finance, Sattva (Salarpuria Sattva) Group</t>
+        </is>
+      </c>
+      <c r="T118" s="5" t="n"/>
+      <c r="U118" s="5" t="n"/>
+      <c r="V118" s="5" t="inlineStr">
+        <is>
+          <t>Registered office landline +91-80-42699000 (Salarpuria Sattva Group HQ, Bengaluru)</t>
+        </is>
+      </c>
+      <c r="W118" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X118" s="5" t="inlineStr">
+        <is>
+          <t>Director status confirmed via thecompanycheck.com, tofler.in, indiafilings.com (DIN 00387006); VP-Finance role at Sattva Group described on sattvagroup.com leadership content, corroborated by rocketreach.co/ZoomInfo</t>
+        </is>
+      </c>
+      <c r="Y118" s="5" t="inlineStr">
+        <is>
+          <t>SPV of Salarpuria Sattva Group; Dhandhania is both director of this entity and group's long-standing finance chief - most relevant contact though no single source combines both facts, hence medium confidence. Existing on-file contact 'girish@...' could not be independently corroborated, retained as unverified fallback only.</t>
+        </is>
+      </c>
+      <c r="Z118" s="4" t="inlineStr">
+        <is>
+          <t>Mahesh Kumar Khaitan | Director, Sattva Group / Director, Darshita Southern India Happy Homes Pvt. Ltd.  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA118" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">

</xml_diff>

<commit_message>
enrich batch (1AM pass): rows 117-131
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -13572,16 +13572,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R119" s="4" t="n"/>
-      <c r="S119" s="4" t="n"/>
-      <c r="T119" s="4" t="n"/>
-      <c r="U119" s="4" t="n"/>
-      <c r="V119" s="4" t="n"/>
-      <c r="W119" s="4" t="n"/>
-      <c r="X119" s="4" t="n"/>
-      <c r="Y119" s="4" t="n"/>
-      <c r="Z119" s="4" t="n"/>
-      <c r="AA119" s="4" t="n"/>
+      <c r="R119" s="3" t="inlineStr">
+        <is>
+          <t>Niraj Kumar Gautam</t>
+        </is>
+      </c>
+      <c r="S119" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Puravankara Limited (parent group CFO; SPV has no separate dedicated CFO)</t>
+        </is>
+      </c>
+      <c r="T119" s="3" t="n"/>
+      <c r="U119" s="3" t="n"/>
+      <c r="V119" s="3" t="inlineStr">
+        <is>
+          <t>investors@puravankara.com / +91 80 25599000 (43439999), Puravankara Ltd registered office, Bengaluru</t>
+        </is>
+      </c>
+      <c r="W119" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X119" s="3" t="inlineStr">
+        <is>
+          <t>MarketScreener, rprealtyplus.com, boardstewardship.com, stockinsights.ai management-changes filing - appointment effective 24-Sep-2025</t>
+        </is>
+      </c>
+      <c r="Y119" s="3" t="inlineStr">
+        <is>
+          <t>This SPV's own directors are only promoter family (Jasbir Ashish Puravankara, Ashish Ravi Puravankara). Finance leadership operates at Puravankara group level. No direct email/mobile for Gautam found publicly.</t>
+        </is>
+      </c>
+      <c r="Z119" s="4" t="inlineStr">
+        <is>
+          <t>Sudip Chatterjee | Group Head - Company Secretary &amp; Compliance Officer, Puravankara Limited | sudip.chatterjee@puravankara.com | 080-43439999, No. 130/2, Ulsoor Road, Bangalore-560042  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA119" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -13642,16 +13674,44 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R120" s="4" t="n"/>
-      <c r="S120" s="4" t="n"/>
-      <c r="T120" s="4" t="n"/>
-      <c r="U120" s="4" t="n"/>
-      <c r="V120" s="4" t="n"/>
-      <c r="W120" s="4" t="n"/>
-      <c r="X120" s="4" t="n"/>
-      <c r="Y120" s="4" t="n"/>
+      <c r="R120" s="3" t="inlineStr">
+        <is>
+          <t>Vishu Mahajan, IAS</t>
+        </is>
+      </c>
+      <c r="S120" s="3" t="inlineStr">
+        <is>
+          <t>Joint Managing Director (Finance), TANGEDCO</t>
+        </is>
+      </c>
+      <c r="T120" s="3" t="n"/>
+      <c r="U120" s="3" t="n"/>
+      <c r="V120" s="3" t="inlineStr">
+        <is>
+          <t>cpro@tnebnet.org, +91 44 2852 0131 (TANGEDCO HQ, Chennai)</t>
+        </is>
+      </c>
+      <c r="W120" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X120" s="3" t="inlineStr">
+        <is>
+          <t>IndianBureaucracy.com, ZoomInfo listing as JMD at TANGEDCO, X/PPPF-2026 event post confirming current role, thesecretariat.in IAS bio page</t>
+        </is>
+      </c>
+      <c r="Y120" s="3" t="inlineStr">
+        <is>
+          <t>TANGEDCO was administratively restructured in 2024-25 into separate generation/distribution/renewable entities. JMD(Finance) role currently held by IAS officer Vishu Mahajan. No direct personal email/mobile found. Existing hint email chairman@tnebnet.org is Chairman/CMD's generic address, not finance-specific.</t>
+        </is>
+      </c>
       <c r="Z120" s="4" t="n"/>
-      <c r="AA120" s="4" t="n"/>
+      <c r="AA120" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -13717,16 +13777,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R121" s="4" t="n"/>
-      <c r="S121" s="4" t="n"/>
-      <c r="T121" s="4" t="n"/>
-      <c r="U121" s="4" t="n"/>
-      <c r="V121" s="4" t="n"/>
-      <c r="W121" s="4" t="n"/>
-      <c r="X121" s="4" t="n"/>
-      <c r="Y121" s="4" t="n"/>
-      <c r="Z121" s="4" t="n"/>
-      <c r="AA121" s="4" t="n"/>
+      <c r="R121" s="5" t="inlineStr">
+        <is>
+          <t>Biju Sreeramachandran</t>
+        </is>
+      </c>
+      <c r="S121" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Inditrade Capital Limited (listed group parent)</t>
+        </is>
+      </c>
+      <c r="T121" s="5" t="n"/>
+      <c r="U121" s="5" t="n"/>
+      <c r="V121" s="5" t="inlineStr">
+        <is>
+          <t>imfl@inditrade.com, +91-22-61424750</t>
+        </is>
+      </c>
+      <c r="W121" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X121" s="5" t="inlineStr">
+        <is>
+          <t>BSE corporate filing dated 17-Jul-2024 stating appointment as CFO &amp; Manager effective 30-May-2024; corroborated by QuickCompany director record</t>
+        </is>
+      </c>
+      <c r="Y121" s="5" t="inlineStr">
+        <is>
+          <t>Subsidiary board comprises non-finance-executive directors; group CFO is most relevant finance contact found. No direct personal email/mobile located.</t>
+        </is>
+      </c>
+      <c r="Z121" s="4" t="inlineStr">
+        <is>
+          <t>Sudip Bandyopadhyay | Chairman/Promoter, Inditrade Capital Limited; Director, Inditrade Microfinance Ltd | imfl@inditrade.com, +91-22-61424750  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA121" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -13777,16 +13869,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R122" s="4" t="n"/>
-      <c r="S122" s="4" t="n"/>
-      <c r="T122" s="4" t="n"/>
-      <c r="U122" s="4" t="n"/>
-      <c r="V122" s="4" t="n"/>
-      <c r="W122" s="4" t="n"/>
-      <c r="X122" s="4" t="n"/>
-      <c r="Y122" s="4" t="n"/>
-      <c r="Z122" s="4" t="n"/>
-      <c r="AA122" s="4" t="n"/>
+      <c r="R122" s="5" t="inlineStr">
+        <is>
+          <t>Nirbhay Fancy Vassa</t>
+        </is>
+      </c>
+      <c r="S122" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (KMP, Abans Finance Pvt Ltd)</t>
+        </is>
+      </c>
+      <c r="T122" s="5" t="n"/>
+      <c r="U122" s="5" t="n"/>
+      <c r="V122" s="5" t="inlineStr">
+        <is>
+          <t>abansrealty@abans.co.in (generic Abans Group mailbox, not confirmed specific to Abans Finance Pvt Ltd)</t>
+        </is>
+      </c>
+      <c r="W122" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X122" s="5" t="inlineStr">
+        <is>
+          <t>MCA-derived KMP listing aggregated by ZaubaCorp/TheCompanyCheck, corroborated by Bloomberg and MarketScreener insider profiles listing him as CFO &amp; Director, Abans Holdings/Abans Finserv group</t>
+        </is>
+      </c>
+      <c r="Y122" s="5" t="inlineStr">
+        <is>
+          <t>Named as CFO KMP specifically for this CIN per aggregator sites. Separate 2026 news indicates he may be leaving related entity Abans Financial Services Ltd effective 15-May-2026 - unclear if applies to this specific entity. No verified direct email/mobile found.</t>
+        </is>
+      </c>
+      <c r="Z122" s="4" t="inlineStr">
+        <is>
+          <t>Dharav Ashok Sheth | Company Secretary (KMP)  (MEDIUM)
+Raghunathan Mudaliar | CFO, Abans Financial Services Ltd (related group entity - possibly not this specific entity)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA122" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -13852,16 +13977,36 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R123" s="4" t="n"/>
-      <c r="S123" s="4" t="n"/>
-      <c r="T123" s="4" t="n"/>
-      <c r="U123" s="4" t="n"/>
-      <c r="V123" s="4" t="n"/>
-      <c r="W123" s="4" t="n"/>
-      <c r="X123" s="4" t="n"/>
-      <c r="Y123" s="4" t="n"/>
+      <c r="R123" s="6" t="n"/>
+      <c r="S123" s="6" t="n"/>
+      <c r="T123" s="6" t="n"/>
+      <c r="U123" s="6" t="n"/>
+      <c r="V123" s="6" t="inlineStr">
+        <is>
+          <t>powersec@essar.com; 91-22-66601100</t>
+        </is>
+      </c>
+      <c r="W123" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X123" s="6" t="inlineStr">
+        <is>
+          <t>Existing registered contact, corroborated as genuine Essar Power-vertical mailbox pattern via search results</t>
+        </is>
+      </c>
+      <c r="Y123" s="6" t="inlineStr">
+        <is>
+          <t>No named CFO/finance head confirmed for this specific SPV. MCA directors show mostly nominee directors tied to project lenders. Group-level CFO (Rajat Gupta) left for Azure Power Sept 2025; no successor found for this entity as of Aug 2026.</t>
+        </is>
+      </c>
       <c r="Z123" s="4" t="n"/>
-      <c r="AA123" s="4" t="n"/>
+      <c r="AA123" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -13912,16 +14057,44 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R124" s="4" t="n"/>
-      <c r="S124" s="4" t="n"/>
-      <c r="T124" s="4" t="n"/>
-      <c r="U124" s="4" t="n"/>
-      <c r="V124" s="4" t="n"/>
-      <c r="W124" s="4" t="n"/>
-      <c r="X124" s="4" t="n"/>
-      <c r="Y124" s="4" t="n"/>
+      <c r="R124" s="6" t="inlineStr">
+        <is>
+          <t>Manohar Lal Aggarwal</t>
+        </is>
+      </c>
+      <c r="S124" s="6" t="inlineStr">
+        <is>
+          <t>Whole-time Director (likely handles finance function given small family-run NBFC structure - inferred, not a confirmed formal finance title)</t>
+        </is>
+      </c>
+      <c r="T124" s="6" t="n"/>
+      <c r="U124" s="6" t="n"/>
+      <c r="V124" s="6" t="inlineStr">
+        <is>
+          <t>bansalcredits@gmail.com; 011-23242127-30</t>
+        </is>
+      </c>
+      <c r="W124" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X124" s="6" t="inlineStr">
+        <is>
+          <t>MCA-derived director/designation data via search snippets (ZaubaCorp, IndiaFilings); registered address/phone via JustDial listing</t>
+        </is>
+      </c>
+      <c r="Y124" s="6" t="inlineStr">
+        <is>
+          <t>Small closely-held Delhi NBFC (promoter family). No distinct CFO or CS-for-debt role found. Inference based on typical small-NBFC structure, not verified finance title.</t>
+        </is>
+      </c>
       <c r="Z124" s="4" t="n"/>
-      <c r="AA124" s="4" t="n"/>
+      <c r="AA124" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -14002,16 +14175,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R125" s="4" t="n"/>
-      <c r="S125" s="4" t="n"/>
-      <c r="T125" s="4" t="n"/>
-      <c r="U125" s="4" t="n"/>
-      <c r="V125" s="4" t="n"/>
-      <c r="W125" s="4" t="n"/>
-      <c r="X125" s="4" t="n"/>
-      <c r="Y125" s="4" t="n"/>
-      <c r="Z125" s="4" t="n"/>
-      <c r="AA125" s="4" t="n"/>
+      <c r="R125" s="5" t="inlineStr">
+        <is>
+          <t>Ravi Porwal</t>
+        </is>
+      </c>
+      <c r="S125" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO) &amp; Senior Management Personnel</t>
+        </is>
+      </c>
+      <c r="T125" s="5" t="n"/>
+      <c r="U125" s="5" t="n"/>
+      <c r="V125" s="5" t="inlineStr">
+        <is>
+          <t>investorrelation@koltepatil.com / 91-20-66226500</t>
+        </is>
+      </c>
+      <c r="W125" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X125" s="5" t="inlineStr">
+        <is>
+          <t>MarketScreener news (CFO appointment effective 8 Oct 2024), Bloomberg Markets profile, Zeebiz (predecessor's exit corroborating transition)</t>
+        </is>
+      </c>
+      <c r="Y125" s="5" t="inlineStr">
+        <is>
+          <t>Identity/designation corroborated by 2+ sources but no verified direct email/mobile found. CA/CS with prior stints at Birla Estates and Shapoorji Pallonji.</t>
+        </is>
+      </c>
+      <c r="Z125" s="4" t="inlineStr">
+        <is>
+          <t>Dipti Rajput, CFA | Vice President - Investor Relations | +91 74004 81432 | dipti.rajput@koltepatil.com | investorrelation@koltepatil.com / 91-20-66226500  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA125" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -14072,16 +14277,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R126" s="4" t="n"/>
-      <c r="S126" s="4" t="n"/>
-      <c r="T126" s="4" t="n"/>
-      <c r="U126" s="4" t="n"/>
-      <c r="V126" s="4" t="n"/>
-      <c r="W126" s="4" t="n"/>
-      <c r="X126" s="4" t="n"/>
-      <c r="Y126" s="4" t="n"/>
-      <c r="Z126" s="4" t="n"/>
-      <c r="AA126" s="4" t="n"/>
+      <c r="R126" s="3" t="inlineStr">
+        <is>
+          <t>Keyur Sanat Shah</t>
+        </is>
+      </c>
+      <c r="S126" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Birla Estates Pvt Ltd (parent); incoming CFO, Aditya Birla Real Estate Ltd effective 1 Mar 2026; also a Director on this SPV's board</t>
+        </is>
+      </c>
+      <c r="T126" s="3" t="n"/>
+      <c r="U126" s="3" t="n"/>
+      <c r="V126" s="3" t="inlineStr">
+        <is>
+          <t>Ankit.R.Agarwal@adityabirla.com (existing registered contact, co-director)</t>
+        </is>
+      </c>
+      <c r="W126" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X126" s="3" t="inlineStr">
+        <is>
+          <t>MCA director listing cross-referenced with TipRanks corporate announcement, TheCompanyCheck director profile, TheOrg org-chart entry</t>
+        </is>
+      </c>
+      <c r="Y126" s="3" t="inlineStr">
+        <is>
+          <t>2+ sources agree he is both group CFO and a named director of this SPV specifically. No direct email/mobile found publicly, not guessed. SPV bought Hindalco's Kalwa land parcel, [ICRA]AA (Stable) NCD rating (~Rs 500 cr) per Aug 2025 rationale.</t>
+        </is>
+      </c>
+      <c r="Z126" s="4" t="inlineStr">
+        <is>
+          <t>Ankit R. Agarwal | Director, Ekamaya Properties Pvt Ltd; Aditya Birla Real Estate/Birla Estates business leadership (finance-specific title not confirmed) | Ankit.R.Agarwal@adityabirla.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA126" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -14132,16 +14369,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R127" s="4" t="n"/>
-      <c r="S127" s="4" t="n"/>
-      <c r="T127" s="4" t="n"/>
-      <c r="U127" s="4" t="n"/>
-      <c r="V127" s="4" t="n"/>
-      <c r="W127" s="4" t="n"/>
-      <c r="X127" s="4" t="n"/>
-      <c r="Y127" s="4" t="n"/>
-      <c r="Z127" s="4" t="n"/>
-      <c r="AA127" s="4" t="n"/>
+      <c r="R127" s="5" t="inlineStr">
+        <is>
+          <t>CH. SRC Murthy</t>
+        </is>
+      </c>
+      <c r="S127" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, BSCPL Infrastructure Ltd (parent; this SPV has no separate finance team)</t>
+        </is>
+      </c>
+      <c r="T127" s="5" t="n"/>
+      <c r="U127" s="5" t="n"/>
+      <c r="V127" s="5" t="inlineStr">
+        <is>
+          <t>info@bscpl.net / 040-23307704 (BSCPL registered office, Hyderabad)</t>
+        </is>
+      </c>
+      <c r="W127" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X127" s="5" t="inlineStr">
+        <is>
+          <t>BSCPL Infrastructure Ltd Senior Management page as reflected in search-engine indexing (direct fetch egress-blocked)</t>
+        </is>
+      </c>
+      <c r="Y127" s="5" t="inlineStr">
+        <is>
+          <t>Name abbreviated/initials-only as listed by company, full expansion not found, only single-source - medium confidence. No direct email/mobile found.</t>
+        </is>
+      </c>
+      <c r="Z127" s="4" t="inlineStr">
+        <is>
+          <t>B. S. Bhaskar | Company Secretary &amp; Compliance Officer, BSCPL Infrastructure Ltd (may be former CS) | bhaskar@bscpl.net | info@bscpl.net / 040-23307704  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA127" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -14192,16 +14461,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R128" s="4" t="n"/>
-      <c r="S128" s="4" t="n"/>
-      <c r="T128" s="4" t="n"/>
-      <c r="U128" s="4" t="n"/>
-      <c r="V128" s="4" t="n"/>
-      <c r="W128" s="4" t="n"/>
-      <c r="X128" s="4" t="n"/>
-      <c r="Y128" s="4" t="n"/>
-      <c r="Z128" s="4" t="n"/>
-      <c r="AA128" s="4" t="n"/>
+      <c r="R128" s="5" t="inlineStr">
+        <is>
+          <t>Bhushan Prasad</t>
+        </is>
+      </c>
+      <c r="S128" s="5" t="inlineStr">
+        <is>
+          <t>Director, JTPM Atsali Ltd. (JSW-nominee); Senior VP - Finance &amp; Commercial, JSW Steel Ltd. / CFO, JSW Projects Ltd.</t>
+        </is>
+      </c>
+      <c r="T128" s="5" t="n"/>
+      <c r="U128" s="5" t="inlineStr">
+        <is>
+          <t>bhushan.prasad@jsw.in</t>
+        </is>
+      </c>
+      <c r="V128" s="5" t="inlineStr">
+        <is>
+          <t>csjtpmatsali@jsw.in</t>
+        </is>
+      </c>
+      <c r="W128" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X128" s="5" t="inlineStr">
+        <is>
+          <t>ZaubaCorp director listing; ZoomInfo/RocketReach profile; web search snippet surfacing email associated with JTPM Atsali records</t>
+        </is>
+      </c>
+      <c r="Y128" s="5" t="inlineStr">
+        <is>
+          <t>SPV/holding entity with no dedicated in-house CFO. Email inferred from standard JSW Group pattern and search snippet, not from official filing - medium confidence. Board composition appears to have changed over time - re-verify before outreach. Debentures reportedly suspended from trading on BSE at one point.</t>
+        </is>
+      </c>
+      <c r="Z128" s="4" t="inlineStr">
+        <is>
+          <t>Manoj Kumar Mohta | Non-Executive Director, JTPM Atsali Ltd.; Director, CEO &amp; CFO, JSW Holdings Ltd. | csjtpmatsali@jsw.in  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA128" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -14262,16 +14567,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R129" s="4" t="n"/>
-      <c r="S129" s="4" t="n"/>
-      <c r="T129" s="4" t="n"/>
-      <c r="U129" s="4" t="n"/>
-      <c r="V129" s="4" t="n"/>
-      <c r="W129" s="4" t="n"/>
-      <c r="X129" s="4" t="n"/>
-      <c r="Y129" s="4" t="n"/>
-      <c r="Z129" s="4" t="n"/>
-      <c r="AA129" s="4" t="n"/>
+      <c r="R129" s="3" t="inlineStr">
+        <is>
+          <t>Ramesh Kumar Jha</t>
+        </is>
+      </c>
+      <c r="S129" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Afcons Infrastructure Ltd.</t>
+        </is>
+      </c>
+      <c r="T129" s="3" t="n"/>
+      <c r="U129" s="3" t="n"/>
+      <c r="V129" s="3" t="inlineStr">
+        <is>
+          <t>secretarial@afcons.com; Tel: +91-22-6719 1000</t>
+        </is>
+      </c>
+      <c r="W129" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X129" s="3" t="inlineStr">
+        <is>
+          <t>Afcons Q1 FY27 earnings call transcript naming him as CFO, corroborated by RocketReach/ZoomInfo CFO listings and FileSure director record; Afcons press release 'Best CFO title'</t>
+        </is>
+      </c>
+      <c r="Y129" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed by 2+ independent sources including live earnings call. Direct email/mobile not publicly available, redacted on ZoomInfo, not reported.</t>
+        </is>
+      </c>
+      <c r="Z129" s="4" t="inlineStr">
+        <is>
+          <t>Gaurang Maheshchandra Parekh | Company Secretary &amp; Compliance Officer, Afcons Infrastructure Ltd. | gaurang@afcons.com | Tel: 022-6719 1214  (HIGH)
+P.R. Rajendran | Former Company Secretary (2009-10 Annual Report); now retired | rajendran@afcons.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA129" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -14332,16 +14670,44 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R130" s="4" t="n"/>
-      <c r="S130" s="4" t="n"/>
-      <c r="T130" s="4" t="n"/>
-      <c r="U130" s="4" t="n"/>
-      <c r="V130" s="4" t="n"/>
-      <c r="W130" s="4" t="n"/>
-      <c r="X130" s="4" t="n"/>
-      <c r="Y130" s="4" t="n"/>
+      <c r="R130" s="6" t="inlineStr">
+        <is>
+          <t>Thanga Raja</t>
+        </is>
+      </c>
+      <c r="S130" s="6" t="inlineStr">
+        <is>
+          <t>Manager, Finance &amp; Accounts, KALS Distilleries Pvt Ltd (~17 years experience)</t>
+        </is>
+      </c>
+      <c r="T130" s="6" t="n"/>
+      <c r="U130" s="6" t="n"/>
+      <c r="V130" s="6" t="inlineStr">
+        <is>
+          <t>rsampath@kals.co.in; customercare@kals.co.in; Tel: +91 44 2434 5254/5264</t>
+        </is>
+      </c>
+      <c r="W130" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X130" s="6" t="inlineStr">
+        <is>
+          <t>ZoomInfo profile; SignalHire employee-directory listing</t>
+        </is>
+      </c>
+      <c r="Y130" s="6" t="inlineStr">
+        <is>
+          <t>Closely-held family-run company, no dedicated CFO/named finance head verified via site, MCA, or press coverage. Single third-party data broker source only, no working email confirmed.</t>
+        </is>
+      </c>
       <c r="Z130" s="4" t="n"/>
-      <c r="AA130" s="4" t="n"/>
+      <c r="AA130" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -14392,16 +14758,48 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R131" s="4" t="n"/>
-      <c r="S131" s="4" t="n"/>
-      <c r="T131" s="4" t="n"/>
-      <c r="U131" s="4" t="n"/>
-      <c r="V131" s="4" t="n"/>
-      <c r="W131" s="4" t="n"/>
-      <c r="X131" s="4" t="n"/>
-      <c r="Y131" s="4" t="n"/>
-      <c r="Z131" s="4" t="n"/>
-      <c r="AA131" s="4" t="n"/>
+      <c r="R131" s="3" t="inlineStr">
+        <is>
+          <t>Rajesh Deo</t>
+        </is>
+      </c>
+      <c r="S131" s="3" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer, Nexus Select Trust (formerly CFO &amp; Director of Westerly Retail Pvt Ltd, 2017-2022)</t>
+        </is>
+      </c>
+      <c r="T131" s="3" t="n"/>
+      <c r="U131" s="3" t="n"/>
+      <c r="V131" s="3" t="inlineStr">
+        <is>
+          <t>IR@nexusselecttrust.com</t>
+        </is>
+      </c>
+      <c r="W131" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X131" s="3" t="inlineStr">
+        <is>
+          <t>Corroborated by ZoomInfo, Crunchbase, MarketScreener bios; ZaubaCorp/Tofler confirm Westerly Retail's current MCA status as Amalgamated</t>
+        </is>
+      </c>
+      <c r="Y131" s="3" t="inlineStr">
+        <is>
+          <t>Westerly Retail was Blackstone-backed SPV owning Seawoods Grand Central mall (Navi Mumbai), folded into Nexus Select Trust REIT. Historical CFO now Group CFO of Nexus Select Trust - most credible current finance contact. No direct email/mobile found. Original hint email is a Blackstone deal-side/legal contact, not finance.</t>
+        </is>
+      </c>
+      <c r="Z131" s="4" t="inlineStr">
+        <is>
+          <t>Siddharth Nawal | Blackstone (real estate deal team) - contact on Westerly Retail's MCA/registry record | siddharth.nawal@blackstone.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA131" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -14482,16 +14880,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R132" s="4" t="n"/>
-      <c r="S132" s="4" t="n"/>
-      <c r="T132" s="4" t="n"/>
-      <c r="U132" s="4" t="n"/>
-      <c r="V132" s="4" t="n"/>
-      <c r="W132" s="4" t="n"/>
-      <c r="X132" s="4" t="n"/>
-      <c r="Y132" s="4" t="n"/>
-      <c r="Z132" s="4" t="n"/>
-      <c r="AA132" s="4" t="n"/>
+      <c r="R132" s="3" t="inlineStr">
+        <is>
+          <t>Rachit Nagpal</t>
+        </is>
+      </c>
+      <c r="S132" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T132" s="3" t="n"/>
+      <c r="U132" s="3" t="n"/>
+      <c r="V132" s="3" t="inlineStr">
+        <is>
+          <t>satiapaper@satiagroup.com; investor line 01633-262215 / registered office 91-1633-262001</t>
+        </is>
+      </c>
+      <c r="W132" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X132" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn, ZoomInfo, and MarketScreener/Goodreturns management-team pages independently confirm as CFO</t>
+        </is>
+      </c>
+      <c r="Y132" s="3" t="inlineStr">
+        <is>
+          <t>2+ sources agree on name/designation - high confidence. Direct email not confirmed, masked on ZoomInfo, left null rather than guessed.</t>
+        </is>
+      </c>
+      <c r="Z132" s="4" t="inlineStr">
+        <is>
+          <t>Rakesh Kumar Dhuria | Company Secretary &amp; Compliance Officer (GM - Secretarial) | satiapaper@satiagroup.com; registered office Village Rupana, Sri Muktsar Sahib-152032, Punjab  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA132" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -14557,16 +14987,41 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R133" s="4" t="n"/>
-      <c r="S133" s="4" t="n"/>
-      <c r="T133" s="4" t="n"/>
-      <c r="U133" s="4" t="n"/>
-      <c r="V133" s="4" t="n"/>
-      <c r="W133" s="4" t="n"/>
-      <c r="X133" s="4" t="n"/>
-      <c r="Y133" s="4" t="n"/>
-      <c r="Z133" s="4" t="n"/>
-      <c r="AA133" s="4" t="n"/>
+      <c r="R133" s="6" t="n"/>
+      <c r="S133" s="6" t="n"/>
+      <c r="T133" s="6" t="n"/>
+      <c r="U133" s="6" t="n"/>
+      <c r="V133" s="6" t="inlineStr">
+        <is>
+          <t>91-40-66285000 (existing registered/property landline - ownership has since changed, not re-verified as current)</t>
+        </is>
+      </c>
+      <c r="W133" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X133" s="6" t="inlineStr">
+        <is>
+          <t>MCA/registry aggregators; CapitaLand/CLINT press releases confirming divestment; theedgemalaysia.com confirming buyer identity</t>
+        </is>
+      </c>
+      <c r="Y133" s="6" t="inlineStr">
+        <is>
+          <t>OWNERSHIP CHANGE: Until 29 Sept 2025 part of CapitaLand India Trust portfolio (CFO Cheah Ying Soon), then divested to Viko Ventures (family office of Yerram Vikranth Reddy) for ~INR 11,031 million. Rs 240 crore charge registered in favour of Axis Trustee Services on 24 Oct 2025 - consistent with fresh NCD issuance under new ownership, live current target. No named CFO/finance officer found for new ownership structure.</t>
+        </is>
+      </c>
+      <c r="Z133" s="4" t="inlineStr">
+        <is>
+          <t>Yerram Vikranthreddy (DIN 01220652) | Additional Director (promoter/founder of Viko Group, new owner)  (MEDIUM)
+Apoorva Reddy Yerram | Additional Director (Designated Partner, Viko Ventures LLP)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA133" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">

</xml_diff>

<commit_message>
enrich batch (1AM pass): rows 132-146
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -15082,16 +15082,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R134" s="4" t="n"/>
-      <c r="S134" s="4" t="n"/>
-      <c r="T134" s="4" t="n"/>
-      <c r="U134" s="4" t="n"/>
-      <c r="V134" s="4" t="n"/>
-      <c r="W134" s="4" t="n"/>
-      <c r="X134" s="4" t="n"/>
-      <c r="Y134" s="4" t="n"/>
-      <c r="Z134" s="4" t="n"/>
-      <c r="AA134" s="4" t="n"/>
+      <c r="R134" s="3" t="inlineStr">
+        <is>
+          <t>Sameer Agarwal</t>
+        </is>
+      </c>
+      <c r="S134" s="3" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer, Manipal Hospitals / Manipal Health Enterprises Ltd (parent group)</t>
+        </is>
+      </c>
+      <c r="T134" s="3" t="n"/>
+      <c r="U134" s="3" t="n"/>
+      <c r="V134" s="3" t="inlineStr">
+        <is>
+          <t>legalcs@manipalhospitals.com / +91 80 4936 0300</t>
+        </is>
+      </c>
+      <c r="W134" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X134" s="3" t="inlineStr">
+        <is>
+          <t>ZaubaCorp director listing, LinkedIn, TheOrg org chart, official Manipal Hospitals Facebook posts, Manipal Health Enterprises Ltd DRHP/RHP (2026 IPO filings)</t>
+        </is>
+      </c>
+      <c r="Y134" s="3" t="inlineStr">
+        <is>
+          <t>Manipal Hospitals (East) India (formerly AMRI Hospitals) is subsidiary of Manipal Health Enterprises Ltd (India's largest healthcare IPO, Aug 2026). Sameer Agarwal is group-level CFO since May 2016, not entity-specific. Direct email/mobile not verified, masked address not usable.</t>
+        </is>
+      </c>
+      <c r="Z134" s="4" t="inlineStr">
+        <is>
+          <t>Sathish Kolar Ramamoorthy | Company Secretary and Compliance Officer, Manipal Health Enterprises Ltd (group parent) | legalcs@manipalhospitals.com | +91 80 4936 0300, Bengaluru 560017  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA134" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -15142,16 +15174,44 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R135" s="4" t="n"/>
-      <c r="S135" s="4" t="n"/>
-      <c r="T135" s="4" t="n"/>
-      <c r="U135" s="4" t="n"/>
-      <c r="V135" s="4" t="n"/>
-      <c r="W135" s="4" t="n"/>
-      <c r="X135" s="4" t="n"/>
-      <c r="Y135" s="4" t="n"/>
+      <c r="R135" s="5" t="inlineStr">
+        <is>
+          <t>Girish Dharampal Jain</t>
+        </is>
+      </c>
+      <c r="S135" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director (oversees Corporate Finance, Project Finance, Investor Relations per company's own management page)</t>
+        </is>
+      </c>
+      <c r="T135" s="5" t="n"/>
+      <c r="U135" s="5" t="n"/>
+      <c r="V135" s="5" t="inlineStr">
+        <is>
+          <t>dpjain.company@dpjaingroup.com; Nagpur, Maharashtra registered office</t>
+        </is>
+      </c>
+      <c r="W135" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X135" s="5" t="inlineStr">
+        <is>
+          <t>dpjaingroup.com/management (via search cache); ZaubaCorp/Tofler director records; Brickwork/ICRA rating rationale references</t>
+        </is>
+      </c>
+      <c r="Y135" s="5" t="inlineStr">
+        <is>
+          <t>No separately titled CFO in public sources; MD is repeatedly described as finance-responsible leader - inferred functional match, not formal CFO title. No verified direct email/mobile found.</t>
+        </is>
+      </c>
       <c r="Z135" s="4" t="n"/>
-      <c r="AA135" s="4" t="n"/>
+      <c r="AA135" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -15222,16 +15282,52 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R136" s="4" t="n"/>
-      <c r="S136" s="4" t="n"/>
-      <c r="T136" s="4" t="n"/>
-      <c r="U136" s="4" t="n"/>
-      <c r="V136" s="4" t="n"/>
-      <c r="W136" s="4" t="n"/>
-      <c r="X136" s="4" t="n"/>
-      <c r="Y136" s="4" t="n"/>
-      <c r="Z136" s="4" t="n"/>
-      <c r="AA136" s="4" t="n"/>
+      <c r="R136" s="5" t="inlineStr">
+        <is>
+          <t>Ananthakumar T (Anantha Kumar Thangavel)</t>
+        </is>
+      </c>
+      <c r="S136" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, IIFL Samasta Finance Ltd</t>
+        </is>
+      </c>
+      <c r="T136" s="5" t="n"/>
+      <c r="U136" s="5" t="inlineStr">
+        <is>
+          <t>ananthakumart@iiflsamasta.com</t>
+        </is>
+      </c>
+      <c r="V136" s="5" t="inlineStr">
+        <is>
+          <t>+91 80 4291 3509; registered office Bangalore 560027</t>
+        </is>
+      </c>
+      <c r="W136" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X136" s="5" t="inlineStr">
+        <is>
+          <t>iiflsamasta.com About Us page (via search cache), LinkedIn, ZoomInfo/aggregator listings</t>
+        </is>
+      </c>
+      <c r="Y136" s="5" t="inlineStr">
+        <is>
+          <t>Name/title corroborated by 2+ sources, but email/phone surfaced only via third-party aggregator, not directly verified on primary page - kept at medium per confidence rules.</t>
+        </is>
+      </c>
+      <c r="Z136" s="4" t="inlineStr">
+        <is>
+          <t>Venkatesh N | Founder &amp; Managing Director, IIFL Samasta Finance Ltd | venkateshn@samasta.co.in (legacy domain, from existing hint)  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA136" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -15292,16 +15388,52 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R137" s="4" t="n"/>
-      <c r="S137" s="4" t="n"/>
-      <c r="T137" s="4" t="n"/>
-      <c r="U137" s="4" t="n"/>
-      <c r="V137" s="4" t="n"/>
-      <c r="W137" s="4" t="n"/>
-      <c r="X137" s="4" t="n"/>
-      <c r="Y137" s="4" t="n"/>
-      <c r="Z137" s="4" t="n"/>
-      <c r="AA137" s="4" t="n"/>
+      <c r="R137" s="5" t="inlineStr">
+        <is>
+          <t>Mukesh Gupta</t>
+        </is>
+      </c>
+      <c r="S137" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director (functions as de facto chief finance decision-maker; ~25 years in private/merchant banking finance before founding the company)</t>
+        </is>
+      </c>
+      <c r="T137" s="5" t="n"/>
+      <c r="U137" s="5" t="inlineStr">
+        <is>
+          <t>mukesh@smileelectronics.com</t>
+        </is>
+      </c>
+      <c r="V137" s="5" t="inlineStr">
+        <is>
+          <t>Registered office landline 080-4038 2727; general contact jameel@smileelectronics.com (Admin/HR, not finance)</t>
+        </is>
+      </c>
+      <c r="W137" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X137" s="5" t="inlineStr">
+        <is>
+          <t>ZoomInfo profile, YourStory profile of Mukesh Gupta/Smile Electronics, smileelectronics.com Management Team page (via search snippets), ZaubaCorp/Tracxn/TheCompanyCheck director listings</t>
+        </is>
+      </c>
+      <c r="Y137" s="5" t="inlineStr">
+        <is>
+          <t>CORRECTION: Smile Electronics Ltd. is NOT a hospital/healthcare group - it's a Bengaluru-based Electronics Manufacturing Services (EMS) company, PCB assembly, aerospace/defence electronics, supplied components for ISRO's Mangalyaan mission. Founded 2000, ~Rs.477 Cr revenue (FY23), unlisted. No distinct named CFO/Treasury Head/CS found - Mukesh Gupta (MD) publicly described as personally running finance. Email is INFERRED from confirmed firstname@smileelectronics.com convention, not independently verified - treat as a guess.</t>
+        </is>
+      </c>
+      <c r="Z137" s="4" t="inlineStr">
+        <is>
+          <t>Jameel Bakshi | Manager, Admin &amp; HR (not a finance role) | jameel@smileelectronics.com | 080 4038 2727 (company registered office)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA137" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -15362,16 +15494,53 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R138" s="4" t="n"/>
-      <c r="S138" s="4" t="n"/>
-      <c r="T138" s="4" t="n"/>
-      <c r="U138" s="4" t="n"/>
-      <c r="V138" s="4" t="n"/>
-      <c r="W138" s="4" t="n"/>
-      <c r="X138" s="4" t="n"/>
-      <c r="Y138" s="4" t="n"/>
-      <c r="Z138" s="4" t="n"/>
-      <c r="AA138" s="4" t="n"/>
+      <c r="R138" s="5" t="inlineStr">
+        <is>
+          <t>Premnath Ravindranath</t>
+        </is>
+      </c>
+      <c r="S138" s="5" t="inlineStr">
+        <is>
+          <t>Executive Director, Kerala Financial Corporation (previously GM - Finance &amp; Marketing per a 2017 legal record)</t>
+        </is>
+      </c>
+      <c r="T138" s="5" t="n"/>
+      <c r="U138" s="5" t="inlineStr">
+        <is>
+          <t>premnathravindranath@kfc.org</t>
+        </is>
+      </c>
+      <c r="V138" s="5" t="inlineStr">
+        <is>
+          <t>Main KFC switchboard +91-471-2737500/2737777; general email kfc@kfc.org</t>
+        </is>
+      </c>
+      <c r="W138" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X138" s="5" t="inlineStr">
+        <is>
+          <t>RocketReach org-chart aggregator, ZoomInfo profile, LinkedIn profile, Indian Kanoon case record (2017) referencing him as GM (Finance &amp; Marketing)</t>
+        </is>
+      </c>
+      <c r="Y138" s="5" t="inlineStr">
+        <is>
+          <t>Sourced mainly from data aggregators, not KFC's own site (blocked). As Executive Director appears senior-most full-time finance-linked executive under government-appointed Chairman/CMD - reasonable primary contact but verify against kfc.org before use.</t>
+        </is>
+      </c>
+      <c r="Z138" s="4" t="inlineStr">
+        <is>
+          <t>Chairman &amp; Managing Director (CMD), Kerala Financial Corporation | md@kfc.org; main switchboard +91-471-2737500  (LOW)
+General corporate contact desk | kfc@kfc.org | +91-471-2737500/2737503/2737576; toll-free 1800-425-8590  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA138" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -15442,16 +15611,53 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R139" s="4" t="n"/>
-      <c r="S139" s="4" t="n"/>
-      <c r="T139" s="4" t="n"/>
-      <c r="U139" s="4" t="n"/>
-      <c r="V139" s="4" t="n"/>
-      <c r="W139" s="4" t="n"/>
-      <c r="X139" s="4" t="n"/>
-      <c r="Y139" s="4" t="n"/>
-      <c r="Z139" s="4" t="n"/>
-      <c r="AA139" s="4" t="n"/>
+      <c r="R139" s="3" t="inlineStr">
+        <is>
+          <t>Niraj Kumar Gautam</t>
+        </is>
+      </c>
+      <c r="S139" s="3" t="inlineStr">
+        <is>
+          <t>Group Chief Financial Officer (CFO), Puravankara Limited - listed parent of Provident Housing Ltd. Elevated from Deputy Group CFO effective 24 Sept 2025</t>
+        </is>
+      </c>
+      <c r="T139" s="3" t="n"/>
+      <c r="U139" s="3" t="inlineStr">
+        <is>
+          <t>neeraj.gautam@puravankara.com</t>
+        </is>
+      </c>
+      <c r="V139" s="3" t="inlineStr">
+        <is>
+          <t>Puravankara registered office 080-4343 9999 / 080-2559 9000; Group Investor Relations desk investors@puravankara.com</t>
+        </is>
+      </c>
+      <c r="W139" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X139" s="3" t="inlineStr">
+        <is>
+          <t>MarketScreener official CFO-appointment announcement, RPRealtyPlus, HR Today, boardstewardship.com, StockInsights.ai management-change filing (Nov 2025), corroborated independently by ZoomInfo and RocketReach</t>
+        </is>
+      </c>
+      <c r="Y139" s="3" t="inlineStr">
+        <is>
+          <t>Provident Housing is 100%-owned subsidiary/affordable-housing brand of Puravankara Limited (BSE:532891/NSE:PURVA); parent's Group CFO is correct top finance contact. Predecessor Deepak Rastogi held role only Jan-Sept 2025. Original hint contact ravikumar.reddy@puravankara.com could NOT be matched to any named individual - closest match is HR Chief, not finance - treat as likely stale.</t>
+        </is>
+      </c>
+      <c r="Z139" s="4" t="inlineStr">
+        <is>
+          <t>Bindu D | Company Secretary &amp; Compliance Officer, Puravankara Limited | bindu.d@puravankara.com  (MEDIUM)
+Group Investor Relations desk | investors@puravankara.com | Mumbai IR office +91-22-4080 7000  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA139" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -15517,16 +15723,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R140" s="4" t="n"/>
-      <c r="S140" s="4" t="n"/>
-      <c r="T140" s="4" t="n"/>
-      <c r="U140" s="4" t="n"/>
-      <c r="V140" s="4" t="n"/>
-      <c r="W140" s="4" t="n"/>
-      <c r="X140" s="4" t="n"/>
-      <c r="Y140" s="4" t="n"/>
-      <c r="Z140" s="4" t="n"/>
-      <c r="AA140" s="4" t="n"/>
+      <c r="R140" s="3" t="inlineStr">
+        <is>
+          <t>Amit Jaiswal</t>
+        </is>
+      </c>
+      <c r="S140" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T140" s="3" t="n"/>
+      <c r="U140" s="3" t="inlineStr">
+        <is>
+          <t>cfo@royalorchidhotels.com</t>
+        </is>
+      </c>
+      <c r="V140" s="3" t="inlineStr">
+        <is>
+          <t>Landline: 080-41783000</t>
+        </is>
+      </c>
+      <c r="W140" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X140" s="3" t="inlineStr">
+        <is>
+          <t>Official Contact Details of KMP document on royalorchidhotels.com, corroborated by Bloomberg Markets profile, Zee Business interview, and LinkedIn</t>
+        </is>
+      </c>
+      <c r="Y140" s="3" t="inlineStr">
+        <is>
+          <t>No mobile number found publicly; email/designation confirmed directly from company's own KMP contact sheet.</t>
+        </is>
+      </c>
+      <c r="Z140" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Ranabir Sanyal | Group Company Secretary &amp; Chief Compliance Officer | cosec@royalorchidhotels.com | Landline: 080-41783000  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA140" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -15587,16 +15829,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R141" s="4" t="n"/>
-      <c r="S141" s="4" t="n"/>
-      <c r="T141" s="4" t="n"/>
-      <c r="U141" s="4" t="n"/>
-      <c r="V141" s="4" t="n"/>
-      <c r="W141" s="4" t="n"/>
-      <c r="X141" s="4" t="n"/>
-      <c r="Y141" s="4" t="n"/>
-      <c r="Z141" s="4" t="n"/>
-      <c r="AA141" s="4" t="n"/>
+      <c r="R141" s="5" t="inlineStr">
+        <is>
+          <t>Nitin Singh</t>
+        </is>
+      </c>
+      <c r="S141" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="T141" s="5" t="n"/>
+      <c r="U141" s="5" t="n"/>
+      <c r="V141" s="5" t="inlineStr">
+        <is>
+          <t>eogepl@essarenp.co.in; care@eogepl.com; service@eogepl.com; phone +91 9376841414</t>
+        </is>
+      </c>
+      <c r="W141" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X141" s="5" t="inlineStr">
+        <is>
+          <t>Company's own executive management page (eogepl.com/executive-management/) and ZoomInfo profile both list Nitin Singh as CFO</t>
+        </is>
+      </c>
+      <c r="Y141" s="5" t="inlineStr">
+        <is>
+          <t>Direct email masked/paywalled on ZoomInfo/RocketReach, left null. Existing hint email independently reconfirmed as company's general contact email.</t>
+        </is>
+      </c>
+      <c r="Z141" s="4" t="inlineStr">
+        <is>
+          <t>Pankaj Kalra | Director (India board) / CEO, Essar Exploration &amp; Production Ltd, Mauritius | eogepl@essarenp.co.in  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA141" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -15677,16 +15951,44 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R142" s="4" t="n"/>
-      <c r="S142" s="4" t="n"/>
-      <c r="T142" s="4" t="n"/>
-      <c r="U142" s="4" t="n"/>
-      <c r="V142" s="4" t="n"/>
-      <c r="W142" s="4" t="n"/>
-      <c r="X142" s="4" t="n"/>
-      <c r="Y142" s="4" t="n"/>
+      <c r="R142" s="5" t="inlineStr">
+        <is>
+          <t>Muneesh Chawla</t>
+        </is>
+      </c>
+      <c r="S142" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer / Whole-time Director (also referred to as Executive Director / Group Financial Controller in some sources)</t>
+        </is>
+      </c>
+      <c r="T142" s="5" t="n"/>
+      <c r="U142" s="5" t="n"/>
+      <c r="V142" s="5" t="inlineStr">
+        <is>
+          <t>info@reventengineering.com; phone +91-7058955570</t>
+        </is>
+      </c>
+      <c r="W142" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X142" s="5" t="inlineStr">
+        <is>
+          <t>Tofler and TheCompanyCheck MCA records showing appointment as CFO/whole-time director on 06 May 2024; LinkedIn lists as Executive Director - Revent Group</t>
+        </is>
+      </c>
+      <c r="Y142" s="5" t="inlineStr">
+        <is>
+          <t>Designation varies across sources - medium confidence. Existing hint contact (aal@amtek.com) belongs to old Amtek Auto Ltd entity, acquired out of insolvency by Deccan Value Investors Dec 2021 and renamed Revent Precision Engineering - old contact likely stale, use reventengineering.com contacts instead.</t>
+        </is>
+      </c>
       <c r="Z142" s="4" t="n"/>
-      <c r="AA142" s="4" t="n"/>
+      <c r="AA142" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -15737,16 +16039,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R143" s="4" t="n"/>
-      <c r="S143" s="4" t="n"/>
-      <c r="T143" s="4" t="n"/>
-      <c r="U143" s="4" t="n"/>
-      <c r="V143" s="4" t="n"/>
-      <c r="W143" s="4" t="n"/>
-      <c r="X143" s="4" t="n"/>
-      <c r="Y143" s="4" t="n"/>
-      <c r="Z143" s="4" t="n"/>
-      <c r="AA143" s="4" t="n"/>
+      <c r="R143" s="5" t="inlineStr">
+        <is>
+          <t>Kartik Deuskar</t>
+        </is>
+      </c>
+      <c r="S143" s="5" t="inlineStr">
+        <is>
+          <t>Director - Finance (Shapoorji Pallonji Family Office / SP Ports); listed director of S P Imperial Star Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="T143" s="5" t="n"/>
+      <c r="U143" s="5" t="inlineStr">
+        <is>
+          <t>kartik.deuskar@shapoorji.com</t>
+        </is>
+      </c>
+      <c r="V143" s="5" t="inlineStr">
+        <is>
+          <t>sanket.shah@shapoorji.com / +91-22-6749-0000</t>
+        </is>
+      </c>
+      <c r="W143" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X143" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch aggregation of ZoomInfo/RocketReach/SignalHire/LinkedIn snippets; ZaubaCorp confirms he and Amit Saboo are directors</t>
+        </is>
+      </c>
+      <c r="Y143" s="5" t="inlineStr">
+        <is>
+          <t>Email surfaced via third-party aggregator snippets, not independently double-verified. His day-to-day title is Director Finance at SP Ports/Family Office, not exclusive to this SPV, but named director here.</t>
+        </is>
+      </c>
+      <c r="Z143" s="4" t="inlineStr">
+        <is>
+          <t>Amit Saboo | Director - Family Office, Shapoorji Pallonji Group (also CEO, SP Ports); director of this SPV  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA143" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -15817,16 +16155,40 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R144" s="4" t="n"/>
-      <c r="S144" s="4" t="n"/>
-      <c r="T144" s="4" t="n"/>
-      <c r="U144" s="4" t="n"/>
-      <c r="V144" s="4" t="n"/>
-      <c r="W144" s="4" t="n"/>
-      <c r="X144" s="4" t="n"/>
-      <c r="Y144" s="4" t="n"/>
-      <c r="Z144" s="4" t="n"/>
-      <c r="AA144" s="4" t="n"/>
+      <c r="R144" s="5" t="n"/>
+      <c r="S144" s="5" t="n"/>
+      <c r="T144" s="5" t="n"/>
+      <c r="U144" s="5" t="n"/>
+      <c r="V144" s="5" t="inlineStr">
+        <is>
+          <t>dhanisecetarial@dhani.com / +91-124-6681199</t>
+        </is>
+      </c>
+      <c r="W144" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X144" s="5" t="inlineStr">
+        <is>
+          <t>Existing registered contact cross-checked against Dhani Services Ltd's published HQ details confirming domain/area code genuine and in use</t>
+        </is>
+      </c>
+      <c r="Y144" s="5" t="inlineStr">
+        <is>
+          <t>No named CFO/treasury head/CS found for this smaller non-listed group NBFC entity. No NCD/debt listing found for this specific CIN. Company's group structure ambiguous post Oct-2025 NCLT merger of 17 Dhani/Indiabulls entities.</t>
+        </is>
+      </c>
+      <c r="Z144" s="4" t="inlineStr">
+        <is>
+          <t>Rajiv Agarwal | Chief Financial Officer, Indiabulls Limited (group entity from Oct-2025 merger) | support@indiabulls.com  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA144" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -15892,16 +16254,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R145" s="4" t="n"/>
-      <c r="S145" s="4" t="n"/>
-      <c r="T145" s="4" t="n"/>
-      <c r="U145" s="4" t="n"/>
-      <c r="V145" s="4" t="n"/>
-      <c r="W145" s="4" t="n"/>
-      <c r="X145" s="4" t="n"/>
-      <c r="Y145" s="4" t="n"/>
-      <c r="Z145" s="4" t="n"/>
-      <c r="AA145" s="4" t="n"/>
+      <c r="R145" s="3" t="inlineStr">
+        <is>
+          <t>Amit Kr. Agarwal</t>
+        </is>
+      </c>
+      <c r="S145" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer - Bhilangana Hydro Power Ltd. / Polyplex Hydro Group</t>
+        </is>
+      </c>
+      <c r="T145" s="3" t="n"/>
+      <c r="U145" s="3" t="n"/>
+      <c r="V145" s="3" t="inlineStr">
+        <is>
+          <t>rjindal@polyplex.com / +91-120-4621300</t>
+        </is>
+      </c>
+      <c r="W145" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X145" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn, RocketReach, ZoomInfo, EasyLeadz, TheOrg all identify him as CFO since 2005 - 4+ independent sources agree</t>
+        </is>
+      </c>
+      <c r="Y145" s="3" t="inlineStr">
+        <is>
+          <t>Direct email/phone masked everywhere, not verified, left null. Polyplex.com domain confirmed correct via existing verified contact.</t>
+        </is>
+      </c>
+      <c r="Z145" s="4" t="inlineStr">
+        <is>
+          <t>Rajesh Kumar Jindal | Director, Bhilangana Hydro Power Ltd. (Polyplex/Jindal group) | rjindal@polyplex.com | +91-120-4621300  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA145" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -15967,16 +16361,44 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R146" s="4" t="n"/>
-      <c r="S146" s="4" t="n"/>
-      <c r="T146" s="4" t="n"/>
-      <c r="U146" s="4" t="n"/>
-      <c r="V146" s="4" t="n"/>
-      <c r="W146" s="4" t="n"/>
-      <c r="X146" s="4" t="n"/>
-      <c r="Y146" s="4" t="n"/>
+      <c r="R146" s="5" t="inlineStr">
+        <is>
+          <t>Pankaj Singh</t>
+        </is>
+      </c>
+      <c r="S146" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Gulshan Group (parent group)</t>
+        </is>
+      </c>
+      <c r="T146" s="5" t="n"/>
+      <c r="U146" s="5" t="n"/>
+      <c r="V146" s="5" t="inlineStr">
+        <is>
+          <t>info@gulshanhomz.com / +91 95 8050 8050</t>
+        </is>
+      </c>
+      <c r="W146" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X146" s="5" t="inlineStr">
+        <is>
+          <t>News coverage of appointment mid-July 2026: indiaretailing.com, medianews4u.com, newspatrolling.com, constrofacilitator.com, todaystraveller.net - 5 independent outlets corroborate</t>
+        </is>
+      </c>
+      <c r="Y146" s="5" t="inlineStr">
+        <is>
+          <t>Appointment confirmed by multiple outlets, but no direct email/mobile found - capped at medium. He is CFO of Gulshan Group (parent conglomerate), not confirmed exclusive to Gulshan Homz legal entity.</t>
+        </is>
+      </c>
       <c r="Z146" s="4" t="n"/>
-      <c r="AA146" s="4" t="n"/>
+      <c r="AA146" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -16042,16 +16464,56 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R147" s="4" t="n"/>
-      <c r="S147" s="4" t="n"/>
-      <c r="T147" s="4" t="n"/>
-      <c r="U147" s="4" t="n"/>
-      <c r="V147" s="4" t="n"/>
-      <c r="W147" s="4" t="n"/>
-      <c r="X147" s="4" t="n"/>
-      <c r="Y147" s="4" t="n"/>
-      <c r="Z147" s="4" t="n"/>
-      <c r="AA147" s="4" t="n"/>
+      <c r="R147" s="3" t="inlineStr">
+        <is>
+          <t>Sathish Kolar Ramamoorthy</t>
+        </is>
+      </c>
+      <c r="S147" s="3" t="inlineStr">
+        <is>
+          <t>Company Secretary &amp; Compliance Officer, Manipal Health Enterprises Limited (MHEL) - group's listed operating entity</t>
+        </is>
+      </c>
+      <c r="T147" s="3" t="inlineStr">
+        <is>
+          <t>+91 80 4936 0300</t>
+        </is>
+      </c>
+      <c r="U147" s="3" t="inlineStr">
+        <is>
+          <t>legalcs@manipalhospitals.com</t>
+        </is>
+      </c>
+      <c r="V147" s="3" t="inlineStr">
+        <is>
+          <t>jyotika.kamath@manipalgroup.com / +91-80-30789100</t>
+        </is>
+      </c>
+      <c r="W147" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X147" s="3" t="inlineStr">
+        <is>
+          <t>Manipal Health Enterprises Limited RHP/DRHP via Kotak Investment Banking and SEBI/BSE/NSE filings; corroborated by ZaubaCorp listings for this CIN showing status 'Amalgamated'</t>
+        </is>
+      </c>
+      <c r="Y147" s="3" t="inlineStr">
+        <is>
+          <t>This entity's CIN shows status Amalgamated - merged into wider Manipal Group hospital structure. Listed/operating entity that issues debt is MHEL (IPO'd July-Aug 2026). Directors on record: Ranjan Ramdas Pai and Shruti Ranjan Pai (promoter family).</t>
+        </is>
+      </c>
+      <c r="Z147" s="4" t="inlineStr">
+        <is>
+          <t>Sameer Agarwal | Group CFO, Manipal Health Enterprises / Manipal Hospitals  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA147" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -16122,16 +16584,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R148" s="4" t="n"/>
-      <c r="S148" s="4" t="n"/>
-      <c r="T148" s="4" t="n"/>
-      <c r="U148" s="4" t="n"/>
-      <c r="V148" s="4" t="n"/>
-      <c r="W148" s="4" t="n"/>
-      <c r="X148" s="4" t="n"/>
-      <c r="Y148" s="4" t="n"/>
-      <c r="Z148" s="4" t="n"/>
-      <c r="AA148" s="4" t="n"/>
+      <c r="R148" s="3" t="inlineStr">
+        <is>
+          <t>Meghana Lale</t>
+        </is>
+      </c>
+      <c r="S148" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Purple Finance Limited (appointed effective 3 Feb 2025)</t>
+        </is>
+      </c>
+      <c r="T148" s="3" t="n"/>
+      <c r="U148" s="3" t="n"/>
+      <c r="V148" s="3" t="inlineStr">
+        <is>
+          <t>customersupport@purplefinance.in / +91-22 6916 5100</t>
+        </is>
+      </c>
+      <c r="W148" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X148" s="3" t="inlineStr">
+        <is>
+          <t>Official BSE corporate announcement (board meeting 19 Jan 2025) as reported by marketscreener.com; registered office contact confirmed via multiple business-listing sources</t>
+        </is>
+      </c>
+      <c r="Y148" s="3" t="inlineStr">
+        <is>
+          <t>CFO appointment is a regulatory BSE disclosure - strong official source. No verified direct email/mobile found. A conflicting stale web snippet naming a different person as CFO was disregarded as unreliable.</t>
+        </is>
+      </c>
+      <c r="Z148" s="4" t="inlineStr">
+        <is>
+          <t>Ruchi Jitendra Nishar | Company Secretary &amp; Compliance Officer (also a promoter) | customersupport@purplefinance.in / +91-22 6916 5100  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA148" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">

</xml_diff>

<commit_message>
enrich batch (1AM pass): rows 147-163 - all pending complete
</commit_message>
<xml_diff>
--- a/NCD Mobile - Enriched.xlsx
+++ b/NCD Mobile - Enriched.xlsx
@@ -16701,16 +16701,48 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R149" s="4" t="n"/>
-      <c r="S149" s="4" t="n"/>
-      <c r="T149" s="4" t="n"/>
-      <c r="U149" s="4" t="n"/>
-      <c r="V149" s="4" t="n"/>
-      <c r="W149" s="4" t="n"/>
-      <c r="X149" s="4" t="n"/>
-      <c r="Y149" s="4" t="n"/>
+      <c r="R149" s="5" t="inlineStr">
+        <is>
+          <t>Bhupendra Chhapwale</t>
+        </is>
+      </c>
+      <c r="S149" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T149" s="5" t="n"/>
+      <c r="U149" s="5" t="inlineStr">
+        <is>
+          <t>bhupendra.chhapwale@inbrew.com</t>
+        </is>
+      </c>
+      <c r="V149" s="5" t="inlineStr">
+        <is>
+          <t>intimation@inbrew.com; Bengaluru HQ: Tower B, RMZ Millenia, Halasuru, Bengaluru 560008</t>
+        </is>
+      </c>
+      <c r="W149" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X149" s="5" t="inlineStr">
+        <is>
+          <t>TheOrg, RocketReach, ZoomInfo, LinkedIn - 3+ independent sources corroborate identity/role</t>
+        </is>
+      </c>
+      <c r="Y149" s="5" t="inlineStr">
+        <is>
+          <t>High confidence on identity/role, but email is INFERRED from RocketReach's firstname.lastname@inbrew.com pattern data, not confirmed verbatim - medium confidence. No mobile found. Prior CFO experience: Molson Coors, SABMiller, Mondelez, AB InBev.</t>
+        </is>
+      </c>
       <c r="Z149" s="4" t="n"/>
-      <c r="AA149" s="4" t="n"/>
+      <c r="AA149" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -16791,16 +16823,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R150" s="4" t="n"/>
-      <c r="S150" s="4" t="n"/>
-      <c r="T150" s="4" t="n"/>
-      <c r="U150" s="4" t="n"/>
-      <c r="V150" s="4" t="n"/>
-      <c r="W150" s="4" t="n"/>
-      <c r="X150" s="4" t="n"/>
-      <c r="Y150" s="4" t="n"/>
-      <c r="Z150" s="4" t="n"/>
-      <c r="AA150" s="4" t="n"/>
+      <c r="R150" s="3" t="inlineStr">
+        <is>
+          <t>Natarajan R (CA)</t>
+        </is>
+      </c>
+      <c r="S150" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO) &amp; Key Managerial Personnel</t>
+        </is>
+      </c>
+      <c r="T150" s="3" t="n"/>
+      <c r="U150" s="3" t="n"/>
+      <c r="V150" s="3" t="inlineStr">
+        <is>
+          <t>cs@salemerode.com; salemerodeinvestmentsltd@gmail.com; landline +91 33 24752834 and +91 487 2828071</t>
+        </is>
+      </c>
+      <c r="W150" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X150" s="3" t="inlineStr">
+        <is>
+          <t>Company's own regulatory appointment filing (salemerode.com), corroborated by corporate-information page</t>
+        </is>
+      </c>
+      <c r="Y150" s="3" t="inlineStr">
+        <is>
+          <t>Appointed CFO/KMP effective 30 June 2021 per official company disclosure - primary source, high confidence. No personal email/mobile found. CIN appears inconsistently across sources, worth reconciling before outreach.</t>
+        </is>
+      </c>
+      <c r="Z150" s="4" t="inlineStr">
+        <is>
+          <t>Manisha N. Menon | Company Secretary &amp; Compliance Officer | cs@salemerode.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA150" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -16851,16 +16915,44 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R151" s="4" t="n"/>
-      <c r="S151" s="4" t="n"/>
-      <c r="T151" s="4" t="n"/>
-      <c r="U151" s="4" t="n"/>
-      <c r="V151" s="4" t="n"/>
-      <c r="W151" s="4" t="n"/>
-      <c r="X151" s="4" t="n"/>
-      <c r="Y151" s="4" t="n"/>
+      <c r="R151" s="5" t="inlineStr">
+        <is>
+          <t>Amit Kumar Verma</t>
+        </is>
+      </c>
+      <c r="S151" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (Group CFO, Dish TV India Ltd - also listed as CFO/KMP of this subsidiary)</t>
+        </is>
+      </c>
+      <c r="T151" s="5" t="n"/>
+      <c r="U151" s="5" t="n"/>
+      <c r="V151" s="5" t="inlineStr">
+        <is>
+          <t>investor@dishd2h.com; ranjit@xingdth.in (existing registered email, appears generic/admin)</t>
+        </is>
+      </c>
+      <c r="W151" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X151" s="5" t="inlineStr">
+        <is>
+          <t>thecompanycheck.com lists him as CFO of this specific entity appointed 26 Dec 2024, corroborated for parent-company role by exchange4media.com and boardstewardship.com</t>
+        </is>
+      </c>
+      <c r="Y151" s="5" t="inlineStr">
+        <is>
+          <t>Parent-level appointment (effective 1 Oct 2024) well corroborated by 2+ sources; subsidiary-specific appointment reported by only one aggregator, not independently cross-verified - medium confidence overall. 20+ years with Dish/Zee group.</t>
+        </is>
+      </c>
       <c r="Z151" s="4" t="n"/>
-      <c r="AA151" s="4" t="n"/>
+      <c r="AA151" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -16931,16 +17023,52 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R152" s="4" t="n"/>
-      <c r="S152" s="4" t="n"/>
-      <c r="T152" s="4" t="n"/>
-      <c r="U152" s="4" t="n"/>
-      <c r="V152" s="4" t="n"/>
-      <c r="W152" s="4" t="n"/>
-      <c r="X152" s="4" t="n"/>
-      <c r="Y152" s="4" t="n"/>
-      <c r="Z152" s="4" t="n"/>
-      <c r="AA152" s="4" t="n"/>
+      <c r="R152" s="3" t="inlineStr">
+        <is>
+          <t>Mangala Sachin Savla</t>
+        </is>
+      </c>
+      <c r="S152" s="3" t="inlineStr">
+        <is>
+          <t>Company Secretary &amp; Compliance Officer</t>
+        </is>
+      </c>
+      <c r="T152" s="3" t="n"/>
+      <c r="U152" s="3" t="inlineStr">
+        <is>
+          <t>info@titanintech.in</t>
+        </is>
+      </c>
+      <c r="V152" s="3" t="inlineStr">
+        <is>
+          <t>+91 87908 14671</t>
+        </is>
+      </c>
+      <c r="W152" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X152" s="3" t="inlineStr">
+        <is>
+          <t>Company's official BSE-mandated disclosure 'Contact information of designated officials of listed entity', corroborated by other BSE corporate filings</t>
+        </is>
+      </c>
+      <c r="Y152" s="3" t="inlineStr">
+        <is>
+          <t>Officially designated compliance/nodal contact under SEBI LODR, not a named CFO. Email/phone are official listed contact, not personal.</t>
+        </is>
+      </c>
+      <c r="Z152" s="4" t="inlineStr">
+        <is>
+          <t>Kumarraju Rudraraju | Managing Director  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA152" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -16991,16 +17119,40 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R153" s="4" t="n"/>
-      <c r="S153" s="4" t="n"/>
-      <c r="T153" s="4" t="n"/>
-      <c r="U153" s="4" t="n"/>
-      <c r="V153" s="4" t="n"/>
-      <c r="W153" s="4" t="n"/>
-      <c r="X153" s="4" t="n"/>
-      <c r="Y153" s="4" t="n"/>
-      <c r="Z153" s="4" t="n"/>
-      <c r="AA153" s="4" t="n"/>
+      <c r="R153" s="6" t="n"/>
+      <c r="S153" s="6" t="n"/>
+      <c r="T153" s="6" t="n"/>
+      <c r="U153" s="6" t="n"/>
+      <c r="V153" s="6" t="inlineStr">
+        <is>
+          <t>kedar.natu@sumashilp.com (Suma Shilp group office, Erandawane, Pune)</t>
+        </is>
+      </c>
+      <c r="W153" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X153" s="6" t="inlineStr">
+        <is>
+          <t>MCA registration record contact matching Suma Shilp Group registered office; could not verify Kedar Natu's designation via any public source</t>
+        </is>
+      </c>
+      <c r="Y153" s="6" t="inlineStr">
+        <is>
+          <t>No named CFO/Finance Controller/Treasury head found. Company operates Westend Mall, Aundh, Pune (Nexus Malls/Blackstone 50%, Suma Shilp Group 50%). Finance likely sits with one of the JV partners' finance teams, neither identified by name for this entity.</t>
+        </is>
+      </c>
+      <c r="Z153" s="4" t="inlineStr">
+        <is>
+          <t>Virendrasingh Shivkumar Thakur | Whole-Time Director, Chitrali Properties Pvt. Ltd. (also Sr. Center Director, Nexus Malls, Pune)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA153" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -17051,16 +17203,44 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R154" s="4" t="n"/>
-      <c r="S154" s="4" t="n"/>
-      <c r="T154" s="4" t="n"/>
-      <c r="U154" s="4" t="n"/>
-      <c r="V154" s="4" t="n"/>
-      <c r="W154" s="4" t="n"/>
-      <c r="X154" s="4" t="n"/>
-      <c r="Y154" s="4" t="n"/>
-      <c r="Z154" s="4" t="n"/>
-      <c r="AA154" s="4" t="n"/>
+      <c r="R154" s="5" t="inlineStr">
+        <is>
+          <t>Jay Viresh Dayani</t>
+        </is>
+      </c>
+      <c r="S154" s="5" t="inlineStr">
+        <is>
+          <t>Senior Vice President, Finance - Virtuous Retail / Xander Group (also a director on this SPV's board)</t>
+        </is>
+      </c>
+      <c r="T154" s="5" t="n"/>
+      <c r="U154" s="5" t="n"/>
+      <c r="V154" s="5" t="n"/>
+      <c r="W154" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X154" s="5" t="inlineStr">
+        <is>
+          <t>Director listing for VR Konkan Private Limited cross-referenced with LinkedIn, TheOrg Virtuous Retail Finance team page, and ZoomInfo profile</t>
+        </is>
+      </c>
+      <c r="Y154" s="5" t="inlineStr">
+        <is>
+          <t>This SPV is a Virtuous Retail (Xander Group + APG JV) project developing ~7 million sq ft mixed-use project in Thane West. Jay Dayani is both board director and group's Senior VP Finance - most credible finance contact. Email masked on ZoomInfo, not guessed.</t>
+        </is>
+      </c>
+      <c r="Z154" s="4" t="inlineStr">
+        <is>
+          <t>Ramachanderan Ramamurthy | Managing Partner, Vachanaa Corporate Services LLP (CPA, ACS) | ram@vachanaa.com | ram@vachanaa.com  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA154" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -17121,16 +17301,40 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R155" s="4" t="n"/>
-      <c r="S155" s="4" t="n"/>
-      <c r="T155" s="4" t="n"/>
-      <c r="U155" s="4" t="n"/>
-      <c r="V155" s="4" t="n"/>
-      <c r="W155" s="4" t="n"/>
-      <c r="X155" s="4" t="n"/>
-      <c r="Y155" s="4" t="n"/>
-      <c r="Z155" s="4" t="n"/>
-      <c r="AA155" s="4" t="n"/>
+      <c r="R155" s="6" t="n"/>
+      <c r="S155" s="6" t="n"/>
+      <c r="T155" s="6" t="n"/>
+      <c r="U155" s="6" t="n"/>
+      <c r="V155" s="6" t="inlineStr">
+        <is>
+          <t>csavvnl@gmail.com; AVVNL corporate helpline 1800-180-6127/6565</t>
+        </is>
+      </c>
+      <c r="W155" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X155" s="6" t="inlineStr">
+        <is>
+          <t>Web search across zaubacorp.com, energy.rajasthan.gov.in, AVVNL tender documents, and news - no authoritative page fetchable, findings from search snippets only</t>
+        </is>
+      </c>
+      <c r="Y155" s="6" t="inlineStr">
+        <is>
+          <t>Could not identify currently serving named Director (Finance)/CFO. MD is K.P. Verma (technocrat/engineer, not finance-specific). Prior Chief Accounts Officer B.L. Sharma has since retired. Board list does not clearly flag a Director Finance title.</t>
+        </is>
+      </c>
+      <c r="Z155" s="4" t="inlineStr">
+        <is>
+          <t>K.P. Verma (Kamal Prakash Verma) | Managing Director, AVVNL (technocrat/engineer background, not finance-specific)  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA155" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -17211,16 +17415,49 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R156" s="4" t="n"/>
-      <c r="S156" s="4" t="n"/>
-      <c r="T156" s="4" t="n"/>
-      <c r="U156" s="4" t="n"/>
-      <c r="V156" s="4" t="n"/>
-      <c r="W156" s="4" t="n"/>
-      <c r="X156" s="4" t="n"/>
-      <c r="Y156" s="4" t="n"/>
-      <c r="Z156" s="4" t="n"/>
-      <c r="AA156" s="4" t="n"/>
+      <c r="R156" s="3" t="inlineStr">
+        <is>
+          <t>Rajesh K R N Namboodiripad</t>
+        </is>
+      </c>
+      <c r="S156" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, Asirvad Micro Finance Limited</t>
+        </is>
+      </c>
+      <c r="T156" s="3" t="n"/>
+      <c r="U156" s="3" t="n"/>
+      <c r="V156" s="3" t="inlineStr">
+        <is>
+          <t>sec@asirvad.in / 91-44-42124493</t>
+        </is>
+      </c>
+      <c r="W156" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X156" s="3" t="inlineStr">
+        <is>
+          <t>Asirvad official website Management Team page corroborated independently by MarketScreener India insider profile</t>
+        </is>
+      </c>
+      <c r="Y156" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant, 22+ years experience, joined as CFO Dec 2021 per both sources. No direct personal mobile/email found, none guessed. A conflicting LinkedIn listing for a different person as CFO is uncorroborated and likely inaccurate.</t>
+        </is>
+      </c>
+      <c r="Z156" s="4" t="inlineStr">
+        <is>
+          <t>Aparna Menon | Company Secretary &amp; Compliance Officer, Asirvad Micro Finance Limited | sec@asirvad.in  (MEDIUM)
+Buvanesh Tharashankar | Group Chief Financial Officer, Manappuram Finance Ltd (parent company)  (HIGH)</t>
+        </is>
+      </c>
+      <c r="AA156" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -17291,16 +17528,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R157" s="4" t="n"/>
-      <c r="S157" s="4" t="n"/>
-      <c r="T157" s="4" t="n"/>
-      <c r="U157" s="4" t="n"/>
-      <c r="V157" s="4" t="n"/>
-      <c r="W157" s="4" t="n"/>
-      <c r="X157" s="4" t="n"/>
-      <c r="Y157" s="4" t="n"/>
-      <c r="Z157" s="4" t="n"/>
-      <c r="AA157" s="4" t="n"/>
+      <c r="R157" s="5" t="n"/>
+      <c r="S157" s="5" t="inlineStr">
+        <is>
+          <t>Director (Finance), Meghalaya Energy Corporation Limited (MeECL)</t>
+        </is>
+      </c>
+      <c r="T157" s="5" t="n"/>
+      <c r="U157" s="5" t="inlineStr">
+        <is>
+          <t>dirfinance.meecl@meghalaya.gov.in</t>
+        </is>
+      </c>
+      <c r="V157" s="5" t="inlineStr">
+        <is>
+          <t>meseb-shil-meg@nic.in / 91-364-2590610</t>
+        </is>
+      </c>
+      <c r="W157" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X157" s="5" t="inlineStr">
+        <is>
+          <t>MeECL official Official Email IDs circular, referenced via web search snippet dated August 2024</t>
+        </is>
+      </c>
+      <c r="Y157" s="5" t="inlineStr">
+        <is>
+          <t>Official position-specific government email, but current named individual could not be identified - role is rotating IAS/state-cadre appointment. Email is role-based, not verified to reach a specific named person.</t>
+        </is>
+      </c>
+      <c r="Z157" s="4" t="inlineStr">
+        <is>
+          <t>Ramakrishna Chitturi, IAS | Formerly Director (Finance) &amp; Member, MeECL (per Annual Report FY2022-23)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA157" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -17376,16 +17645,44 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R158" s="4" t="n"/>
-      <c r="S158" s="4" t="n"/>
-      <c r="T158" s="4" t="n"/>
-      <c r="U158" s="4" t="n"/>
-      <c r="V158" s="4" t="n"/>
-      <c r="W158" s="4" t="n"/>
-      <c r="X158" s="4" t="n"/>
-      <c r="Y158" s="4" t="n"/>
+      <c r="R158" s="5" t="inlineStr">
+        <is>
+          <t>Manoj V. Mathew</t>
+        </is>
+      </c>
+      <c r="S158" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T158" s="5" t="n"/>
+      <c r="U158" s="5" t="n"/>
+      <c r="V158" s="5" t="inlineStr">
+        <is>
+          <t>mca@unimoniindia.com; Toll-free 1800 102 0555</t>
+        </is>
+      </c>
+      <c r="W158" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X158" s="5" t="inlineStr">
+        <is>
+          <t>Cross-verified across LinkedIn, company Facebook post naming him CFO, and Tracxn/RocketReach profile for Wizzmoni Financial Services Ltd (renamed from Unimoni Financial Services)</t>
+        </is>
+      </c>
+      <c r="Y158" s="5" t="inlineStr">
+        <is>
+          <t>Company renamed 'Wizzmoni Financial Services Ltd'. Identity corroborated by 2+ sources but no verified corporate email/mobile found. CEO is CA Krishnan R; registered office Manipal Centre, Bangalore.</t>
+        </is>
+      </c>
       <c r="Z158" s="4" t="n"/>
-      <c r="AA158" s="4" t="n"/>
+      <c r="AA158" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -17456,16 +17753,52 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R159" s="4" t="n"/>
-      <c r="S159" s="4" t="n"/>
-      <c r="T159" s="4" t="n"/>
-      <c r="U159" s="4" t="n"/>
-      <c r="V159" s="4" t="n"/>
-      <c r="W159" s="4" t="n"/>
-      <c r="X159" s="4" t="n"/>
-      <c r="Y159" s="4" t="n"/>
-      <c r="Z159" s="4" t="n"/>
-      <c r="AA159" s="4" t="n"/>
+      <c r="R159" s="5" t="inlineStr">
+        <is>
+          <t>Kundan Sangwar</t>
+        </is>
+      </c>
+      <c r="S159" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer (appointed as KMP effective 12 August 2026)</t>
+        </is>
+      </c>
+      <c r="T159" s="5" t="n"/>
+      <c r="U159" s="5" t="inlineStr">
+        <is>
+          <t>kundan.sangwar@shalimarpaints.com</t>
+        </is>
+      </c>
+      <c r="V159" s="5" t="inlineStr">
+        <is>
+          <t>askus@shalimarpaints.com</t>
+        </is>
+      </c>
+      <c r="W159" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X159" s="5" t="inlineStr">
+        <is>
+          <t>Board resolution/SEBI Regulation 30 disclosure reported via scanx.trade; previously AGM at JSW Paints per Apollo.io</t>
+        </is>
+      </c>
+      <c r="Y159" s="5" t="inlineStr">
+        <is>
+          <t>Very recent appointment from single stock-exchange-disclosure source - medium confidence pending second confirmation. Email is inferred pattern based on confirmed CS email, treat as unverified. Predecessors: Sachin Naik (resigned 30-May-2026), Manoj Kumar Pasari (appointed Feb 2024).</t>
+        </is>
+      </c>
+      <c r="Z159" s="4" t="inlineStr">
+        <is>
+          <t>Snehal (Mahendra) Saboo | Company Secretary &amp; Compliance Officer | snehal.saboo@shalimarpaints.com | askus@shalimarpaints.com; Registrar (Beetal Financial) 011-29961281-83  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA159" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -17526,16 +17859,44 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R160" s="4" t="n"/>
-      <c r="S160" s="4" t="n"/>
-      <c r="T160" s="4" t="n"/>
-      <c r="U160" s="4" t="n"/>
-      <c r="V160" s="4" t="n"/>
-      <c r="W160" s="4" t="n"/>
-      <c r="X160" s="4" t="n"/>
-      <c r="Y160" s="4" t="n"/>
+      <c r="R160" s="3" t="inlineStr">
+        <is>
+          <t>CMA Kshirod Chandra Nanda</t>
+        </is>
+      </c>
+      <c r="S160" s="3" t="inlineStr">
+        <is>
+          <t>Director (Finance) / CFO, GRIDCO Ltd (Board-level Whole-Time Director)</t>
+        </is>
+      </c>
+      <c r="T160" s="3" t="n"/>
+      <c r="U160" s="3" t="n"/>
+      <c r="V160" s="3" t="inlineStr">
+        <is>
+          <t>gridcofca@gridco.co.in; cs@gridco.co.in; phone 0674-2540098/2540877</t>
+        </is>
+      </c>
+      <c r="W160" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X160" s="3" t="inlineStr">
+        <is>
+          <t>ICMAI Bhubaneswar Chapter felicitation coverage on appointment (~7 July 2025), corroborated by FalconEbiz/TheCompanyCheck director-record aggregators via his DIN</t>
+        </is>
+      </c>
+      <c r="Y160" s="3" t="inlineStr">
+        <is>
+          <t>Identity corroborated by 2+ independent sources. gridcofca@ address treated as Finance &amp; Corporate Affairs desk fallback, not personal inbox. MD is Satya Priya Rath, IAS (appointed July 2025) as alternate.</t>
+        </is>
+      </c>
       <c r="Z160" s="4" t="n"/>
-      <c r="AA160" s="4" t="n"/>
+      <c r="AA160" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -17586,16 +17947,36 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R161" s="4" t="n"/>
-      <c r="S161" s="4" t="n"/>
-      <c r="T161" s="4" t="n"/>
-      <c r="U161" s="4" t="n"/>
-      <c r="V161" s="4" t="n"/>
-      <c r="W161" s="4" t="n"/>
-      <c r="X161" s="4" t="n"/>
-      <c r="Y161" s="4" t="n"/>
+      <c r="R161" s="5" t="n"/>
+      <c r="S161" s="5" t="n"/>
+      <c r="T161" s="5" t="n"/>
+      <c r="U161" s="5" t="n"/>
+      <c r="V161" s="5" t="inlineStr">
+        <is>
+          <t>fin@designarch.in (Designarch Group Finance desk)</t>
+        </is>
+      </c>
+      <c r="W161" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X161" s="5" t="inlineStr">
+        <is>
+          <t>EasyLeadz company profile and Dun &amp; Bradstreet business directory listing both confirm fin@designarch.in as finance contact</t>
+        </is>
+      </c>
+      <c r="Y161" s="5" t="inlineStr">
+        <is>
+          <t>No named CFO/Finance Head identified specifically for this entity. Directors on record are Shivang Bhardwaj and Rajeev Arora (Technical Director, not finance). Could not find Designarch-group CFO/Finance Controller via LinkedIn/ZoomInfo/site searches.</t>
+        </is>
+      </c>
       <c r="Z161" s="4" t="n"/>
-      <c r="AA161" s="4" t="n"/>
+      <c r="AA161" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -17651,16 +18032,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R162" s="4" t="n"/>
-      <c r="S162" s="4" t="n"/>
-      <c r="T162" s="4" t="n"/>
-      <c r="U162" s="4" t="n"/>
-      <c r="V162" s="4" t="n"/>
-      <c r="W162" s="4" t="n"/>
-      <c r="X162" s="4" t="n"/>
-      <c r="Y162" s="4" t="n"/>
-      <c r="Z162" s="4" t="n"/>
-      <c r="AA162" s="4" t="n"/>
+      <c r="R162" s="5" t="inlineStr">
+        <is>
+          <t>Sanket Jain</t>
+        </is>
+      </c>
+      <c r="S162" s="5" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer, The Wadhwa Group</t>
+        </is>
+      </c>
+      <c r="T162" s="5" t="n"/>
+      <c r="U162" s="5" t="n"/>
+      <c r="V162" s="5" t="inlineStr">
+        <is>
+          <t>Head Office landline 022-6144 6603 / toll-free 1800 209 6669</t>
+        </is>
+      </c>
+      <c r="W162" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X162" s="5" t="inlineStr">
+        <is>
+          <t>ZoomInfo and RocketReach both list him as CA/CFO of The Wadhwa Group; LinkedIn confirms, prior background at DLF/Godrej Properties/Nirmal Lifestyle</t>
+        </is>
+      </c>
+      <c r="Y162" s="5" t="inlineStr">
+        <is>
+          <t>Registered address matches The Wadhwa Group's head office. Email not found directly - was inferred from company pattern but not included per no-fabrication rule (left null). No direct phone found for him personally.</t>
+        </is>
+      </c>
+      <c r="Z162" s="4" t="inlineStr">
+        <is>
+          <t>N. Modani | Director, Finance, The Wadhwa Group  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA162" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -17736,16 +18149,56 @@
           <t>Direct email + No phone</t>
         </is>
       </c>
-      <c r="R163" s="4" t="n"/>
-      <c r="S163" s="4" t="n"/>
-      <c r="T163" s="4" t="n"/>
-      <c r="U163" s="4" t="n"/>
-      <c r="V163" s="4" t="n"/>
-      <c r="W163" s="4" t="n"/>
-      <c r="X163" s="4" t="n"/>
-      <c r="Y163" s="4" t="n"/>
-      <c r="Z163" s="4" t="n"/>
-      <c r="AA163" s="4" t="n"/>
+      <c r="R163" s="3" t="inlineStr">
+        <is>
+          <t>Shikha Kapoor</t>
+        </is>
+      </c>
+      <c r="S163" s="3" t="inlineStr">
+        <is>
+          <t>Company Secretary &amp; Compliance Officer</t>
+        </is>
+      </c>
+      <c r="T163" s="3" t="inlineStr">
+        <is>
+          <t>98786-38505</t>
+        </is>
+      </c>
+      <c r="U163" s="3" t="inlineStr">
+        <is>
+          <t>compliance@credif.in</t>
+        </is>
+      </c>
+      <c r="V163" s="3" t="inlineStr">
+        <is>
+          <t>Registered office phone 0181-4639903-06/08; corporate office (Skyline Financial Services, New Delhi) 011-26812682</t>
+        </is>
+      </c>
+      <c r="W163" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="X163" s="3" t="inlineStr">
+        <is>
+          <t>Official Credifin Limited Investor Contact page (credif.in/investor-contact), corroborated by regulatory filings citing her CS membership number A19146</t>
+        </is>
+      </c>
+      <c r="Y163" s="3" t="inlineStr">
+        <is>
+          <t>CS/Compliance role, not dedicated CFO, but most senior named finance-adjacent/debt-compliance contact found - typical CS-handles-debt-compliance setup at small NBFCs. 2 independent sources agree - high confidence.</t>
+        </is>
+      </c>
+      <c r="Z163" s="4" t="inlineStr">
+        <is>
+          <t>Vijay Kumar Sareen | Whole-Time Director | 0181-4639903-08  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA163" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -17826,16 +18279,48 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R164" s="4" t="n"/>
-      <c r="S164" s="4" t="n"/>
-      <c r="T164" s="4" t="n"/>
-      <c r="U164" s="4" t="n"/>
-      <c r="V164" s="4" t="n"/>
-      <c r="W164" s="4" t="n"/>
-      <c r="X164" s="4" t="n"/>
-      <c r="Y164" s="4" t="n"/>
-      <c r="Z164" s="4" t="n"/>
-      <c r="AA164" s="4" t="n"/>
+      <c r="R164" s="5" t="inlineStr">
+        <is>
+          <t>Vatsal M. Doshi</t>
+        </is>
+      </c>
+      <c r="S164" s="5" t="inlineStr">
+        <is>
+          <t>Whole-time Director &amp; Chief Financial Officer (CFO)</t>
+        </is>
+      </c>
+      <c r="T164" s="5" t="n"/>
+      <c r="U164" s="5" t="n"/>
+      <c r="V164" s="5" t="inlineStr">
+        <is>
+          <t>shalibhadra_mum@yahoo.co.in / +91-22-24322993, 24322994, 24224575</t>
+        </is>
+      </c>
+      <c r="W164" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="X164" s="5" t="inlineStr">
+        <is>
+          <t>MarketScreener insider profile, RocketReach org chart, Bloomberg profile page; registered office phone/email cross-checked against indiratrade.com board-members page</t>
+        </is>
+      </c>
+      <c r="Y164" s="5" t="inlineStr">
+        <is>
+          <t>Sources conflict on exact CFO attribution within this family-run NBFC board - another profile shows Minesh Mukund Doshi (MD) also as CFO since Aug 2023, a third mentions Dhruvil Doshi as prior Whole-Time Director cum CFO. No personal mobile/email found for any - verify by phone before outreach.</t>
+        </is>
+      </c>
+      <c r="Z164" s="4" t="inlineStr">
+        <is>
+          <t>Darshana Deepak Chauhan | Company Secretary &amp; Compliance Officer | shalibhadra_mum@yahoo.co.in / +91-22-24322993  (MEDIUM)</t>
+        </is>
+      </c>
+      <c r="AA164" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -17886,16 +18371,41 @@
           <t>Direct email + Landline</t>
         </is>
       </c>
-      <c r="R165" s="4" t="n"/>
-      <c r="S165" s="4" t="n"/>
-      <c r="T165" s="4" t="n"/>
-      <c r="U165" s="4" t="n"/>
-      <c r="V165" s="4" t="n"/>
-      <c r="W165" s="4" t="n"/>
-      <c r="X165" s="4" t="n"/>
-      <c r="Y165" s="4" t="n"/>
-      <c r="Z165" s="4" t="n"/>
-      <c r="AA165" s="4" t="n"/>
+      <c r="R165" s="6" t="n"/>
+      <c r="S165" s="6" t="n"/>
+      <c r="T165" s="6" t="n"/>
+      <c r="U165" s="6" t="n"/>
+      <c r="V165" s="6" t="inlineStr">
+        <is>
+          <t>cosecdbr@dbg.co.in; DB Group registered office +91-22-49742706 / info@dbg.co.in (Valor Estate Ltd/DB Realty, Mumbai)</t>
+        </is>
+      </c>
+      <c r="W165" s="6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="X165" s="6" t="inlineStr">
+        <is>
+          <t>Zauba Corp company record (via search snippet); group registered-office contact corroborated via BSE corporate filings for Valor Estate Limited (formerly D B Realty Ltd)</t>
+        </is>
+      </c>
+      <c r="Y165" s="6" t="inlineStr">
+        <is>
+          <t>Closely-held DB Group/Balwa-family SPV entity with no independent CFO/treasury head/IR desk found. Hint email strongly suggests correspondence routed through Valor Estate Ltd's company secretarial desk rather than a Pandora-specific contact.</t>
+        </is>
+      </c>
+      <c r="Z165" s="4" t="inlineStr">
+        <is>
+          <t>Atul Bhatnagar | Chief Financial Officer, Valor Estate Ltd. (formerly D B Realty Ltd) - listed DB Group flagship company | info@dbg.co.in / +91-22-49742706  (LOW)
+Abdul Hafeez Balwa | Director, Pandora Projects Pvt Ltd (Balwa family / DB Group)  (LOW)</t>
+        </is>
+      </c>
+      <c r="AA165" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14-0100</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>